<commit_message>
Introduction Eta / combinaison
</commit_message>
<xml_diff>
--- a/Manuel Validation/CAS C05/TEST C05.xlsx
+++ b/Manuel Validation/CAS C05/TEST C05.xlsx
@@ -101,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="178">
   <si>
     <t>Portee principale</t>
   </si>
@@ -623,6 +623,18 @@
   </si>
   <si>
     <t>Degré mini connexion</t>
+  </si>
+  <si>
+    <t>Eta Nc</t>
+  </si>
+  <si>
+    <t>ANP dans la semelle sup ?</t>
+  </si>
+  <si>
+    <t>MplRd(Eta)</t>
+  </si>
+  <si>
+    <t>Avec prise en compte degre connexion</t>
   </si>
 </sst>
 </file>
@@ -635,7 +647,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -675,6 +687,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -862,7 +881,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1014,6 +1033,18 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1718,17 +1749,17 @@
       <c r="W19" s="3"/>
       <c r="X19" s="17">
         <f>ABS(MIN(Q64:Q74))/MplRd_app</f>
-        <v>0.36935863136015534</v>
+        <v>0.80365439470760591</v>
       </c>
       <c r="Y19" s="3"/>
       <c r="Z19" s="17">
         <f>ABS(MIN(S64:S74))/MplRd_app</f>
-        <v>0.13029674327898993</v>
+        <v>0.16615602649116473</v>
       </c>
       <c r="AA19" s="3"/>
       <c r="AB19" s="17">
         <f>ABS(MIN(U64:U74))/MplRd_app</f>
-        <v>0.36935863136015534</v>
+        <v>0.80365439470760591</v>
       </c>
     </row>
     <row r="20" spans="3:28" x14ac:dyDescent="0.25">
@@ -1754,27 +1785,27 @@
       </c>
       <c r="W20" s="17">
         <f>MAX(Q75:Q95)/MplRd_1</f>
-        <v>0.11748547618378141</v>
+        <v>8.6080604793403168E-2</v>
       </c>
       <c r="X20" s="17">
         <f>ABS(MIN(Q75:Q95))/MplRd_app</f>
-        <v>0.3693586313601554</v>
+        <v>0.80365439470760591</v>
       </c>
       <c r="Y20" s="17">
         <f>MAX(S75:S95)/MplRd_1</f>
-        <v>0.56418659309650965</v>
+        <v>1.2620141945020804</v>
       </c>
       <c r="Z20" s="17">
         <f>ABS(MIN(S75:S95))/MplRd_app</f>
-        <v>0.13029674327898993</v>
+        <v>0.16615602649116476</v>
       </c>
       <c r="AA20" s="17">
         <f>MAX(U75:U95)/MplRd_1</f>
-        <v>0.49882043629895506</v>
+        <v>1.0853387514605828</v>
       </c>
       <c r="AB20" s="17">
         <f>ABS(MIN(U75:U95))/MplRd_app</f>
-        <v>0.3693586313601554</v>
+        <v>0.80365439470760591</v>
       </c>
     </row>
     <row r="21" spans="3:28" x14ac:dyDescent="0.25">
@@ -1818,7 +1849,7 @@
       <c r="W23" s="53"/>
       <c r="X23" s="54">
         <f>MAX(X19,Z19,AB19)</f>
-        <v>0.36935863136015534</v>
+        <v>0.80365439470760591</v>
       </c>
     </row>
     <row r="24" spans="3:28" x14ac:dyDescent="0.25">
@@ -1852,11 +1883,11 @@
       </c>
       <c r="W24" s="55">
         <f>MAX(W20,Y20,AA20)</f>
-        <v>0.56418659309650965</v>
+        <v>1.2620141945020804</v>
       </c>
       <c r="X24" s="56">
         <f>MAX(X20,Z20,AB20)</f>
-        <v>0.3693586313601554</v>
+        <v>0.80365439470760591</v>
       </c>
     </row>
     <row r="25" spans="3:28" x14ac:dyDescent="0.25">
@@ -1910,6 +1941,9 @@
       <c r="P26" t="s">
         <v>45</v>
       </c>
+      <c r="V26" s="15" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="27" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D27" s="2" t="s">
@@ -1937,6 +1971,21 @@
         <f>beff_a/e_s*1000</f>
         <v>8.3333333333333339</v>
       </c>
+      <c r="V27" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="W27" s="64">
+        <f>Connexion!D74</f>
+        <v>612.80229895647165</v>
+      </c>
+      <c r="X27" s="64">
+        <f>Connexion!E74</f>
+        <v>626.00933229871885</v>
+      </c>
+      <c r="Y27" s="64">
+        <f>Connexion!F74</f>
+        <v>640.27285237589899</v>
+      </c>
     </row>
     <row r="28" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D28" s="2" t="s">
@@ -1957,6 +2006,21 @@
       <c r="K28" t="s">
         <v>105</v>
       </c>
+      <c r="V28" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="W28" s="18">
+        <f>MAX(Q75:Q95)</f>
+        <v>62.090026722513699</v>
+      </c>
+      <c r="X28" s="18">
+        <f>MAX(S75:S95)</f>
+        <v>910.29210643778856</v>
+      </c>
+      <c r="Y28" s="18">
+        <f>MAX(U75:U95)</f>
+        <v>782.85593186644996</v>
+      </c>
     </row>
     <row r="29" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D29" s="2" t="s">
@@ -1978,6 +2042,18 @@
       </c>
       <c r="P29" t="s">
         <v>48</v>
+      </c>
+      <c r="W29" s="66">
+        <f>W28/W27</f>
+        <v>0.10132146506017604</v>
+      </c>
+      <c r="X29" s="66">
+        <f t="shared" ref="X29:Y29" si="0">X28/X27</f>
+        <v>1.4541190673550786</v>
+      </c>
+      <c r="Y29" s="66">
+        <f t="shared" si="0"/>
+        <v>1.2226911213890443</v>
       </c>
     </row>
     <row r="30" spans="3:28" x14ac:dyDescent="0.25">
@@ -2079,15 +2155,15 @@
       </c>
       <c r="W34" s="13">
         <f t="array" ref="W34">MAX(ABS(R64:R74))</f>
-        <v>104.28976285984055</v>
+        <v>226.91476285984055</v>
       </c>
       <c r="X34" s="13">
         <f t="array" ref="X34">MAX(ABS(T64:T74))</f>
-        <v>36.789762859840557</v>
+        <v>46.914762859840557</v>
       </c>
       <c r="Y34" s="13">
         <f t="array" ref="Y34">MAX(ABS(V64:V74))</f>
-        <v>104.28976285984055</v>
+        <v>226.91476285984055</v>
       </c>
     </row>
     <row r="35" spans="3:25" x14ac:dyDescent="0.25">
@@ -2118,15 +2194,15 @@
       </c>
       <c r="W35" s="18">
         <f t="array" ref="W35">MAX(ABS(R75:R95))</f>
-        <v>76.959735862043672</v>
+        <v>112.22848586204367</v>
       </c>
       <c r="X35" s="18">
         <f t="array" ref="X35">MAX(ABS(T75:T95))</f>
-        <v>179.33473586204366</v>
+        <v>385.22848586204367</v>
       </c>
       <c r="Y35" s="18">
         <f t="array" ref="Y35">MAX(ABS(V75:V95))</f>
-        <v>189.45973586204366</v>
+        <v>412.22848586204367</v>
       </c>
     </row>
     <row r="36" spans="3:25" x14ac:dyDescent="0.25">
@@ -2213,16 +2289,16 @@
         <v>108</v>
       </c>
       <c r="W38" s="17">
-        <f>W34/VplRd</f>
-        <v>0.14481258686445753</v>
+        <f t="shared" ref="W38:Y39" si="1">W34/VplRd</f>
+        <v>0.31508474951305188</v>
       </c>
       <c r="X38" s="17">
-        <f>X34/VplRd</f>
-        <v>5.1084790911102844E-2</v>
+        <f t="shared" si="1"/>
+        <v>6.5143960304106047E-2</v>
       </c>
       <c r="Y38" s="17">
-        <f>Y34/VplRd</f>
-        <v>0.14481258686445753</v>
+        <f t="shared" si="1"/>
+        <v>0.31508474951305188</v>
       </c>
     </row>
     <row r="39" spans="3:25" x14ac:dyDescent="0.25">
@@ -2245,16 +2321,16 @@
         <v>114</v>
       </c>
       <c r="W39" s="17">
-        <f>W35/VplRd</f>
-        <v>0.10686320621484002</v>
+        <f t="shared" si="1"/>
+        <v>0.15583597960046786</v>
       </c>
       <c r="X39" s="17">
-        <f>X35/VplRd</f>
-        <v>0.24901703007742795</v>
+        <f t="shared" si="1"/>
+        <v>0.53491284323403565</v>
       </c>
       <c r="Y39" s="17">
-        <f>Y35/VplRd</f>
-        <v>0.26307619947043115</v>
+        <f t="shared" si="1"/>
+        <v>0.57240396161537754</v>
       </c>
     </row>
     <row r="40" spans="3:25" x14ac:dyDescent="0.25">
@@ -2310,7 +2386,7 @@
       </c>
       <c r="W42" s="57">
         <f>MAX(W38:Y38)</f>
-        <v>0.14481258686445753</v>
+        <v>0.31508474951305188</v>
       </c>
     </row>
     <row r="43" spans="3:25" x14ac:dyDescent="0.25">
@@ -2319,7 +2395,7 @@
       </c>
       <c r="W43" s="57">
         <f>MAX(W39:Y39)</f>
-        <v>0.26307619947043115</v>
+        <v>0.57240396161537754</v>
       </c>
     </row>
     <row r="44" spans="3:25" x14ac:dyDescent="0.25">
@@ -2553,13 +2629,13 @@
       </c>
       <c r="E57" s="4">
         <f>H57*d</f>
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="F57" t="s">
         <v>99</v>
       </c>
       <c r="H57" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I57" t="s">
         <v>107</v>
@@ -2571,13 +2647,13 @@
       </c>
       <c r="E58" s="4">
         <f>H58*d</f>
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="F58" t="s">
         <v>99</v>
       </c>
       <c r="H58" s="4">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="I58" t="s">
         <v>107</v>
@@ -2693,31 +2769,31 @@
         <v>3</v>
       </c>
       <c r="E64" s="18">
-        <f>La-D64</f>
+        <f t="shared" ref="E64:E74" si="2">La-D64</f>
         <v>0</v>
       </c>
       <c r="F64" s="18">
-        <f>-qG_1/2*(La-D64)^2</f>
+        <f t="shared" ref="F64:F74" si="3">-qG_1/2*(La-D64)^2</f>
         <v>0</v>
       </c>
       <c r="G64" s="18">
-        <f>-qG_1*La*(1-D64/La)</f>
+        <f t="shared" ref="G64:G74" si="4">-qG_1*La*(1-D64/La)</f>
         <v>0</v>
       </c>
       <c r="H64" s="17">
-        <f>-qG_2/2*(La-D64)^2</f>
+        <f t="shared" ref="H64:H74" si="5">-qG_2/2*(La-D64)^2</f>
         <v>0</v>
       </c>
       <c r="I64" s="17">
-        <f>-qG_2*La*(1-D64/La)</f>
+        <f t="shared" ref="I64:I74" si="6">-qG_2*La*(1-D64/La)</f>
         <v>0</v>
       </c>
       <c r="J64" s="17">
-        <f>-qQ/2*(La-D64)^2</f>
+        <f t="shared" ref="J64:J74" si="7">-qQ/2*(La-D64)^2</f>
         <v>0</v>
       </c>
       <c r="K64" s="17">
-        <f>-qQ*La*(1-D64/La)</f>
+        <f t="shared" ref="K64:K74" si="8">-qQ*La*(1-D64/La)</f>
         <v>0</v>
       </c>
       <c r="L64" s="3">
@@ -2735,27 +2811,27 @@
         <v>0</v>
       </c>
       <c r="Q64" s="18">
-        <f>GammaG*(F64+H64)+GammaQ*J64</f>
+        <f t="shared" ref="Q64:Q95" si="9">GammaG*(F64+H64)+GammaQ*J64</f>
         <v>0</v>
       </c>
       <c r="R64" s="18">
-        <f>GammaG*(G64+I64)+GammaQ*K64</f>
+        <f t="shared" ref="R64:R95" si="10">GammaG*(G64+I64)+GammaQ*K64</f>
         <v>0</v>
       </c>
       <c r="S64" s="18">
-        <f>GammaG*(F64+H64)+GammaQ*L64</f>
+        <f t="shared" ref="S64:S95" si="11">GammaG*(F64+H64)+GammaQ*L64</f>
         <v>0</v>
       </c>
       <c r="T64" s="18">
-        <f>GammaG*(G64+I64)+GammaQ*M64</f>
+        <f t="shared" ref="T64:T95" si="12">GammaG*(G64+I64)+GammaQ*M64</f>
         <v>0</v>
       </c>
       <c r="U64" s="18">
-        <f>GammaG*(F64+H64)+GammaQ*N64</f>
+        <f t="shared" ref="U64:U95" si="13">GammaG*(F64+H64)+GammaQ*N64</f>
         <v>0</v>
       </c>
       <c r="V64" s="18">
-        <f>GammaG*(G64+I64)+GammaQ*O64</f>
+        <f t="shared" ref="V64:V95" si="14">GammaG*(G64+I64)+GammaQ*O64</f>
         <v>0</v>
       </c>
     </row>
@@ -2765,36 +2841,36 @@
         <v>2</v>
       </c>
       <c r="D65" s="28">
-        <f>D66+La/10</f>
+        <f t="shared" ref="D65:D73" si="15">D66+La/10</f>
         <v>2.6999999999999997</v>
       </c>
       <c r="E65" s="18">
-        <f>La-D65</f>
+        <f t="shared" si="2"/>
         <v>0.30000000000000027</v>
       </c>
       <c r="F65" s="18">
-        <f>-qG_1/2*(La-D65)^2</f>
+        <f t="shared" si="3"/>
         <v>-0.29627514288711776</v>
       </c>
       <c r="G65" s="18">
-        <f>-qG_1*La*(1-D65/La)</f>
+        <f t="shared" si="4"/>
         <v>-1.9751676192474501</v>
       </c>
       <c r="H65" s="17">
-        <f>-qG_2/2*(La-D65)^2</f>
-        <v>-0.11250000000000021</v>
+        <f t="shared" si="5"/>
+        <v>-0.22500000000000042</v>
       </c>
       <c r="I65" s="17">
-        <f>-qG_2*La*(1-D65/La)</f>
-        <v>-0.75000000000000067</v>
+        <f t="shared" si="6"/>
+        <v>-1.5000000000000013</v>
       </c>
       <c r="J65" s="17">
-        <f>-qQ/2*(La-D65)^2</f>
-        <v>-0.67500000000000127</v>
+        <f t="shared" si="7"/>
+        <v>-1.8000000000000034</v>
       </c>
       <c r="K65" s="17">
-        <f>-qQ*La*(1-D65/La)</f>
-        <v>-4.5000000000000036</v>
+        <f t="shared" si="8"/>
+        <v>-12.000000000000011</v>
       </c>
       <c r="L65" s="3">
         <v>0</v>
@@ -2803,36 +2879,36 @@
         <v>0</v>
       </c>
       <c r="N65" s="17">
-        <f t="shared" ref="N65:N74" si="0">J65+L65</f>
-        <v>-0.67500000000000127</v>
+        <f t="shared" ref="N65:N74" si="16">J65+L65</f>
+        <v>-1.8000000000000034</v>
       </c>
       <c r="O65" s="17">
-        <f t="shared" ref="O65:O74" si="1">K65+M65</f>
-        <v>-4.5000000000000036</v>
+        <f t="shared" ref="O65:O74" si="17">K65+M65</f>
+        <v>-12.000000000000011</v>
       </c>
       <c r="Q65" s="18">
-        <f>GammaG*(F65+H65)+GammaQ*J65</f>
-        <v>-1.5643464428976113</v>
+        <f t="shared" si="9"/>
+        <v>-3.4037214428976146</v>
       </c>
       <c r="R65" s="18">
-        <f>GammaG*(G65+I65)+GammaQ*K65</f>
-        <v>-10.428976285984064</v>
+        <f t="shared" si="10"/>
+        <v>-22.691476285984074</v>
       </c>
       <c r="S65" s="18">
-        <f>GammaG*(F65+H65)+GammaQ*L65</f>
-        <v>-0.55184644289760931</v>
+        <f t="shared" si="11"/>
+        <v>-0.70372144289760963</v>
       </c>
       <c r="T65" s="18">
-        <f>GammaG*(G65+I65)+GammaQ*M65</f>
-        <v>-3.6789762859840587</v>
+        <f t="shared" si="12"/>
+        <v>-4.6914762859840593</v>
       </c>
       <c r="U65" s="18">
-        <f>GammaG*(F65+H65)+GammaQ*N65</f>
-        <v>-1.5643464428976113</v>
+        <f t="shared" si="13"/>
+        <v>-3.4037214428976146</v>
       </c>
       <c r="V65" s="18">
-        <f>GammaG*(G65+I65)+GammaQ*O65</f>
-        <v>-10.428976285984064</v>
+        <f t="shared" si="14"/>
+        <v>-22.691476285984074</v>
       </c>
     </row>
     <row r="66" spans="2:23" x14ac:dyDescent="0.25">
@@ -2841,36 +2917,36 @@
         <v>3</v>
       </c>
       <c r="D66" s="28">
-        <f>D67+La/10</f>
+        <f t="shared" si="15"/>
         <v>2.4</v>
       </c>
       <c r="E66" s="18">
-        <f>La-D66</f>
+        <f t="shared" si="2"/>
         <v>0.60000000000000009</v>
       </c>
       <c r="F66" s="18">
-        <f>-qG_1/2*(La-D66)^2</f>
+        <f t="shared" si="3"/>
         <v>-1.1851005715484693</v>
       </c>
       <c r="G66" s="18">
-        <f>-qG_1*La*(1-D66/La)</f>
+        <f t="shared" si="4"/>
         <v>-3.950335238494898</v>
       </c>
       <c r="H66" s="17">
-        <f>-qG_2/2*(La-D66)^2</f>
-        <v>-0.45000000000000012</v>
+        <f t="shared" si="5"/>
+        <v>-0.90000000000000024</v>
       </c>
       <c r="I66" s="17">
-        <f>-qG_2*La*(1-D66/La)</f>
-        <v>-1.5000000000000004</v>
+        <f t="shared" si="6"/>
+        <v>-3.0000000000000009</v>
       </c>
       <c r="J66" s="17">
-        <f>-qQ/2*(La-D66)^2</f>
-        <v>-2.7000000000000006</v>
+        <f t="shared" si="7"/>
+        <v>-7.200000000000002</v>
       </c>
       <c r="K66" s="17">
-        <f>-qQ*La*(1-D66/La)</f>
-        <v>-9.0000000000000036</v>
+        <f t="shared" si="8"/>
+        <v>-24.000000000000007</v>
       </c>
       <c r="L66" s="3">
         <v>0</v>
@@ -2879,36 +2955,36 @@
         <v>0</v>
       </c>
       <c r="N66" s="17">
-        <f t="shared" si="0"/>
-        <v>-2.7000000000000006</v>
+        <f t="shared" si="16"/>
+        <v>-7.200000000000002</v>
       </c>
       <c r="O66" s="17">
-        <f t="shared" si="1"/>
-        <v>-9.0000000000000036</v>
+        <f t="shared" si="17"/>
+        <v>-24.000000000000007</v>
       </c>
       <c r="Q66" s="18">
-        <f>GammaG*(F66+H66)+GammaQ*J66</f>
-        <v>-6.2573857715904344</v>
+        <f t="shared" si="9"/>
+        <v>-13.614885771590437</v>
       </c>
       <c r="R66" s="18">
-        <f>GammaG*(G66+I66)+GammaQ*K66</f>
-        <v>-20.85795257196812</v>
+        <f t="shared" si="10"/>
+        <v>-45.382952571968133</v>
       </c>
       <c r="S66" s="18">
-        <f>GammaG*(F66+H66)+GammaQ*L66</f>
-        <v>-2.2073857715904337</v>
+        <f t="shared" si="11"/>
+        <v>-2.8148857715904341</v>
       </c>
       <c r="T66" s="18">
-        <f>GammaG*(G66+I66)+GammaQ*M66</f>
-        <v>-7.3579525719681129</v>
+        <f t="shared" si="12"/>
+        <v>-9.3829525719681151</v>
       </c>
       <c r="U66" s="18">
-        <f>GammaG*(F66+H66)+GammaQ*N66</f>
-        <v>-6.2573857715904344</v>
+        <f t="shared" si="13"/>
+        <v>-13.614885771590437</v>
       </c>
       <c r="V66" s="18">
-        <f>GammaG*(G66+I66)+GammaQ*O66</f>
-        <v>-20.85795257196812</v>
+        <f t="shared" si="14"/>
+        <v>-45.382952571968133</v>
       </c>
     </row>
     <row r="67" spans="2:23" x14ac:dyDescent="0.25">
@@ -2917,36 +2993,36 @@
         <v>4</v>
       </c>
       <c r="D67" s="28">
-        <f>D68+La/10</f>
+        <f t="shared" si="15"/>
         <v>2.1</v>
       </c>
       <c r="E67" s="18">
-        <f>La-D67</f>
+        <f t="shared" si="2"/>
         <v>0.89999999999999991</v>
       </c>
       <c r="F67" s="18">
-        <f>-qG_1/2*(La-D67)^2</f>
+        <f t="shared" si="3"/>
         <v>-2.6664762859840545</v>
       </c>
       <c r="G67" s="18">
-        <f>-qG_1*La*(1-D67/La)</f>
+        <f t="shared" si="4"/>
         <v>-5.9255028577423436</v>
       </c>
       <c r="H67" s="17">
-        <f>-qG_2/2*(La-D67)^2</f>
-        <v>-1.0124999999999997</v>
+        <f t="shared" si="5"/>
+        <v>-2.0249999999999995</v>
       </c>
       <c r="I67" s="17">
-        <f>-qG_2*La*(1-D67/La)</f>
-        <v>-2.2499999999999996</v>
+        <f t="shared" si="6"/>
+        <v>-4.4999999999999991</v>
       </c>
       <c r="J67" s="17">
-        <f>-qQ/2*(La-D67)^2</f>
-        <v>-6.0749999999999984</v>
+        <f t="shared" si="7"/>
+        <v>-16.199999999999996</v>
       </c>
       <c r="K67" s="17">
-        <f>-qQ*La*(1-D67/La)</f>
-        <v>-13.499999999999996</v>
+        <f t="shared" si="8"/>
+        <v>-35.999999999999993</v>
       </c>
       <c r="L67" s="3">
         <v>0</v>
@@ -2955,36 +3031,36 @@
         <v>0</v>
       </c>
       <c r="N67" s="17">
-        <f t="shared" si="0"/>
-        <v>-6.0749999999999984</v>
+        <f t="shared" si="16"/>
+        <v>-16.199999999999996</v>
       </c>
       <c r="O67" s="17">
-        <f t="shared" si="1"/>
-        <v>-13.499999999999996</v>
+        <f t="shared" si="17"/>
+        <v>-35.999999999999993</v>
       </c>
       <c r="Q67" s="18">
-        <f>GammaG*(F67+H67)+GammaQ*J67</f>
-        <v>-14.079117986078471</v>
+        <f t="shared" si="9"/>
+        <v>-30.633492986078465</v>
       </c>
       <c r="R67" s="18">
-        <f>GammaG*(G67+I67)+GammaQ*K67</f>
-        <v>-31.286928857952155</v>
+        <f t="shared" si="10"/>
+        <v>-68.074428857952142</v>
       </c>
       <c r="S67" s="18">
-        <f>GammaG*(F67+H67)+GammaQ*L67</f>
-        <v>-4.9666179860784734</v>
+        <f t="shared" si="11"/>
+        <v>-6.3334929860784737</v>
       </c>
       <c r="T67" s="18">
-        <f>GammaG*(G67+I67)+GammaQ*M67</f>
-        <v>-11.036928857952164</v>
+        <f t="shared" si="12"/>
+        <v>-14.074428857952164</v>
       </c>
       <c r="U67" s="18">
-        <f>GammaG*(F67+H67)+GammaQ*N67</f>
-        <v>-14.079117986078471</v>
+        <f t="shared" si="13"/>
+        <v>-30.633492986078465</v>
       </c>
       <c r="V67" s="18">
-        <f>GammaG*(G67+I67)+GammaQ*O67</f>
-        <v>-31.286928857952155</v>
+        <f t="shared" si="14"/>
+        <v>-68.074428857952142</v>
       </c>
     </row>
     <row r="68" spans="2:23" x14ac:dyDescent="0.25">
@@ -2993,36 +3069,36 @@
         <v>5</v>
       </c>
       <c r="D68" s="28">
-        <f>D69+La/10</f>
+        <f t="shared" si="15"/>
         <v>1.8</v>
       </c>
       <c r="E68" s="18">
-        <f>La-D68</f>
+        <f t="shared" si="2"/>
         <v>1.2</v>
       </c>
       <c r="F68" s="18">
-        <f>-qG_1/2*(La-D68)^2</f>
+        <f t="shared" si="3"/>
         <v>-4.7404022861938762</v>
       </c>
       <c r="G68" s="18">
-        <f>-qG_1*La*(1-D68/La)</f>
+        <f t="shared" si="4"/>
         <v>-7.9006704769897942</v>
       </c>
       <c r="H68" s="17">
-        <f>-qG_2/2*(La-D68)^2</f>
-        <v>-1.7999999999999998</v>
+        <f t="shared" si="5"/>
+        <v>-3.5999999999999996</v>
       </c>
       <c r="I68" s="17">
-        <f>-qG_2*La*(1-D68/La)</f>
-        <v>-3</v>
+        <f t="shared" si="6"/>
+        <v>-6</v>
       </c>
       <c r="J68" s="17">
-        <f>-qQ/2*(La-D68)^2</f>
-        <v>-10.799999999999999</v>
+        <f t="shared" si="7"/>
+        <v>-28.799999999999997</v>
       </c>
       <c r="K68" s="17">
-        <f>-qQ*La*(1-D68/La)</f>
-        <v>-18</v>
+        <f t="shared" si="8"/>
+        <v>-48</v>
       </c>
       <c r="L68" s="3">
         <v>0</v>
@@ -3031,36 +3107,36 @@
         <v>0</v>
       </c>
       <c r="N68" s="17">
-        <f t="shared" si="0"/>
-        <v>-10.799999999999999</v>
+        <f t="shared" si="16"/>
+        <v>-28.799999999999997</v>
       </c>
       <c r="O68" s="17">
-        <f t="shared" si="1"/>
-        <v>-18</v>
+        <f t="shared" si="17"/>
+        <v>-48</v>
       </c>
       <c r="Q68" s="18">
-        <f>GammaG*(F68+H68)+GammaQ*J68</f>
-        <v>-25.029543086361734</v>
+        <f t="shared" si="9"/>
+        <v>-54.459543086361727</v>
       </c>
       <c r="R68" s="18">
-        <f>GammaG*(G68+I68)+GammaQ*K68</f>
-        <v>-41.715905143936226</v>
+        <f t="shared" si="10"/>
+        <v>-90.765905143936223</v>
       </c>
       <c r="S68" s="18">
-        <f>GammaG*(F68+H68)+GammaQ*L68</f>
-        <v>-8.829543086361733</v>
+        <f t="shared" si="11"/>
+        <v>-11.259543086361733</v>
       </c>
       <c r="T68" s="18">
-        <f>GammaG*(G68+I68)+GammaQ*M68</f>
-        <v>-14.715905143936224</v>
+        <f t="shared" si="12"/>
+        <v>-18.765905143936223</v>
       </c>
       <c r="U68" s="18">
-        <f>GammaG*(F68+H68)+GammaQ*N68</f>
-        <v>-25.029543086361734</v>
+        <f t="shared" si="13"/>
+        <v>-54.459543086361727</v>
       </c>
       <c r="V68" s="18">
-        <f>GammaG*(G68+I68)+GammaQ*O68</f>
-        <v>-41.715905143936226</v>
+        <f t="shared" si="14"/>
+        <v>-90.765905143936223</v>
       </c>
     </row>
     <row r="69" spans="2:23" x14ac:dyDescent="0.25">
@@ -3069,36 +3145,36 @@
         <v>6</v>
       </c>
       <c r="D69" s="28">
-        <f>D70+La/10</f>
+        <f t="shared" si="15"/>
         <v>1.5</v>
       </c>
       <c r="E69" s="18">
-        <f>La-D69</f>
+        <f t="shared" si="2"/>
         <v>1.5</v>
       </c>
       <c r="F69" s="18">
-        <f>-qG_1/2*(La-D69)^2</f>
+        <f t="shared" si="3"/>
         <v>-7.4068785721779316</v>
       </c>
       <c r="G69" s="18">
-        <f>-qG_1*La*(1-D69/La)</f>
+        <f t="shared" si="4"/>
         <v>-9.8758380962372421</v>
       </c>
       <c r="H69" s="17">
-        <f>-qG_2/2*(La-D69)^2</f>
-        <v>-2.8125</v>
+        <f t="shared" si="5"/>
+        <v>-5.625</v>
       </c>
       <c r="I69" s="17">
-        <f>-qG_2*La*(1-D69/La)</f>
-        <v>-3.75</v>
+        <f t="shared" si="6"/>
+        <v>-7.5</v>
       </c>
       <c r="J69" s="17">
-        <f>-qQ/2*(La-D69)^2</f>
-        <v>-16.875</v>
+        <f t="shared" si="7"/>
+        <v>-45</v>
       </c>
       <c r="K69" s="17">
-        <f>-qQ*La*(1-D69/La)</f>
-        <v>-22.5</v>
+        <f t="shared" si="8"/>
+        <v>-60</v>
       </c>
       <c r="L69" s="3">
         <v>0</v>
@@ -3107,36 +3183,36 @@
         <v>0</v>
       </c>
       <c r="N69" s="17">
-        <f t="shared" si="0"/>
-        <v>-16.875</v>
+        <f t="shared" si="16"/>
+        <v>-45</v>
       </c>
       <c r="O69" s="17">
-        <f t="shared" si="1"/>
-        <v>-22.5</v>
+        <f t="shared" si="17"/>
+        <v>-60</v>
       </c>
       <c r="Q69" s="18">
-        <f>GammaG*(F69+H69)+GammaQ*J69</f>
-        <v>-39.108661072440206</v>
+        <f t="shared" si="9"/>
+        <v>-85.093036072440214</v>
       </c>
       <c r="R69" s="18">
-        <f>GammaG*(G69+I69)+GammaQ*K69</f>
-        <v>-52.144881429920275</v>
+        <f t="shared" si="10"/>
+        <v>-113.45738142992028</v>
       </c>
       <c r="S69" s="18">
-        <f>GammaG*(F69+H69)+GammaQ*L69</f>
-        <v>-13.796161072440208</v>
+        <f t="shared" si="11"/>
+        <v>-17.593036072440206</v>
       </c>
       <c r="T69" s="18">
-        <f>GammaG*(G69+I69)+GammaQ*M69</f>
-        <v>-18.394881429920279</v>
+        <f t="shared" si="12"/>
+        <v>-23.457381429920279</v>
       </c>
       <c r="U69" s="18">
-        <f>GammaG*(F69+H69)+GammaQ*N69</f>
-        <v>-39.108661072440206</v>
+        <f t="shared" si="13"/>
+        <v>-85.093036072440214</v>
       </c>
       <c r="V69" s="18">
-        <f>GammaG*(G69+I69)+GammaQ*O69</f>
-        <v>-52.144881429920275</v>
+        <f t="shared" si="14"/>
+        <v>-113.45738142992028</v>
       </c>
     </row>
     <row r="70" spans="2:23" x14ac:dyDescent="0.25">
@@ -3145,36 +3221,36 @@
         <v>7</v>
       </c>
       <c r="D70" s="28">
-        <f>D71+La/10</f>
+        <f t="shared" si="15"/>
         <v>1.2</v>
       </c>
       <c r="E70" s="18">
-        <f>La-D70</f>
+        <f t="shared" si="2"/>
         <v>1.8</v>
       </c>
       <c r="F70" s="18">
-        <f>-qG_1/2*(La-D70)^2</f>
+        <f t="shared" si="3"/>
         <v>-10.665905143936222</v>
       </c>
       <c r="G70" s="18">
-        <f>-qG_1*La*(1-D70/La)</f>
+        <f t="shared" si="4"/>
         <v>-11.851005715484693</v>
       </c>
       <c r="H70" s="17">
-        <f>-qG_2/2*(La-D70)^2</f>
-        <v>-4.0500000000000007</v>
+        <f t="shared" si="5"/>
+        <v>-8.1000000000000014</v>
       </c>
       <c r="I70" s="17">
-        <f>-qG_2*La*(1-D70/La)</f>
-        <v>-4.5000000000000009</v>
+        <f t="shared" si="6"/>
+        <v>-9.0000000000000018</v>
       </c>
       <c r="J70" s="17">
-        <f>-qQ/2*(La-D70)^2</f>
-        <v>-24.3</v>
+        <f t="shared" si="7"/>
+        <v>-64.800000000000011</v>
       </c>
       <c r="K70" s="17">
-        <f>-qQ*La*(1-D70/La)</f>
-        <v>-27.000000000000004</v>
+        <f t="shared" si="8"/>
+        <v>-72.000000000000014</v>
       </c>
       <c r="L70" s="3">
         <v>0</v>
@@ -3183,36 +3259,36 @@
         <v>0</v>
       </c>
       <c r="N70" s="17">
-        <f t="shared" si="0"/>
-        <v>-24.3</v>
+        <f t="shared" si="16"/>
+        <v>-64.800000000000011</v>
       </c>
       <c r="O70" s="17">
-        <f t="shared" si="1"/>
-        <v>-27.000000000000004</v>
+        <f t="shared" si="17"/>
+        <v>-72.000000000000014</v>
       </c>
       <c r="Q70" s="18">
-        <f>GammaG*(F70+H70)+GammaQ*J70</f>
-        <v>-56.316471944313903</v>
+        <f t="shared" si="9"/>
+        <v>-122.53397194431392</v>
       </c>
       <c r="R70" s="18">
-        <f>GammaG*(G70+I70)+GammaQ*K70</f>
-        <v>-62.573857715904339</v>
+        <f t="shared" si="10"/>
+        <v>-136.14885771590437</v>
       </c>
       <c r="S70" s="18">
-        <f>GammaG*(F70+H70)+GammaQ*L70</f>
-        <v>-19.866471944313901</v>
+        <f t="shared" si="11"/>
+        <v>-25.333971944313902</v>
       </c>
       <c r="T70" s="18">
-        <f>GammaG*(G70+I70)+GammaQ*M70</f>
-        <v>-22.073857715904335</v>
+        <f t="shared" si="12"/>
+        <v>-28.148857715904342</v>
       </c>
       <c r="U70" s="18">
-        <f>GammaG*(F70+H70)+GammaQ*N70</f>
-        <v>-56.316471944313903</v>
+        <f t="shared" si="13"/>
+        <v>-122.53397194431392</v>
       </c>
       <c r="V70" s="18">
-        <f>GammaG*(G70+I70)+GammaQ*O70</f>
-        <v>-62.573857715904339</v>
+        <f t="shared" si="14"/>
+        <v>-136.14885771590437</v>
       </c>
     </row>
     <row r="71" spans="2:23" x14ac:dyDescent="0.25">
@@ -3221,36 +3297,36 @@
         <v>8</v>
       </c>
       <c r="D71" s="28">
-        <f>D72+La/10</f>
+        <f t="shared" si="15"/>
         <v>0.89999999999999991</v>
       </c>
       <c r="E71" s="18">
-        <f>La-D71</f>
+        <f t="shared" si="2"/>
         <v>2.1</v>
       </c>
       <c r="F71" s="18">
-        <f>-qG_1/2*(La-D71)^2</f>
+        <f t="shared" si="3"/>
         <v>-14.517482001468746</v>
       </c>
       <c r="G71" s="18">
-        <f>-qG_1*La*(1-D71/La)</f>
+        <f t="shared" si="4"/>
         <v>-13.826173334732138</v>
       </c>
       <c r="H71" s="17">
-        <f>-qG_2/2*(La-D71)^2</f>
-        <v>-5.5125000000000002</v>
+        <f t="shared" si="5"/>
+        <v>-11.025</v>
       </c>
       <c r="I71" s="17">
-        <f>-qG_2*La*(1-D71/La)</f>
-        <v>-5.25</v>
+        <f t="shared" si="6"/>
+        <v>-10.5</v>
       </c>
       <c r="J71" s="17">
-        <f>-qQ/2*(La-D71)^2</f>
-        <v>-33.075000000000003</v>
+        <f t="shared" si="7"/>
+        <v>-88.2</v>
       </c>
       <c r="K71" s="17">
-        <f>-qQ*La*(1-D71/La)</f>
-        <v>-31.499999999999996</v>
+        <f t="shared" si="8"/>
+        <v>-84</v>
       </c>
       <c r="L71" s="3">
         <v>0</v>
@@ -3259,36 +3335,36 @@
         <v>0</v>
       </c>
       <c r="N71" s="17">
-        <f t="shared" si="0"/>
-        <v>-33.075000000000003</v>
+        <f t="shared" si="16"/>
+        <v>-88.2</v>
       </c>
       <c r="O71" s="17">
-        <f t="shared" si="1"/>
-        <v>-31.499999999999996</v>
+        <f t="shared" si="17"/>
+        <v>-84</v>
       </c>
       <c r="Q71" s="18">
-        <f>GammaG*(F71+H71)+GammaQ*J71</f>
-        <v>-76.652975701982811</v>
+        <f t="shared" si="9"/>
+        <v>-166.78235070198281</v>
       </c>
       <c r="R71" s="18">
-        <f>GammaG*(G71+I71)+GammaQ*K71</f>
-        <v>-73.002834001888388</v>
+        <f t="shared" si="10"/>
+        <v>-158.84033400188838</v>
       </c>
       <c r="S71" s="18">
-        <f>GammaG*(F71+H71)+GammaQ*L71</f>
-        <v>-27.040475701982807</v>
+        <f t="shared" si="11"/>
+        <v>-34.48235070198281</v>
       </c>
       <c r="T71" s="18">
-        <f>GammaG*(G71+I71)+GammaQ*M71</f>
-        <v>-25.752834001888392</v>
+        <f t="shared" si="12"/>
+        <v>-32.840334001888394</v>
       </c>
       <c r="U71" s="18">
-        <f>GammaG*(F71+H71)+GammaQ*N71</f>
-        <v>-76.652975701982811</v>
+        <f t="shared" si="13"/>
+        <v>-166.78235070198281</v>
       </c>
       <c r="V71" s="18">
-        <f>GammaG*(G71+I71)+GammaQ*O71</f>
-        <v>-73.002834001888388</v>
+        <f t="shared" si="14"/>
+        <v>-158.84033400188838</v>
       </c>
     </row>
     <row r="72" spans="2:23" x14ac:dyDescent="0.25">
@@ -3297,36 +3373,36 @@
         <v>9</v>
       </c>
       <c r="D72" s="28">
-        <f>D73+La/10</f>
+        <f t="shared" si="15"/>
         <v>0.6</v>
       </c>
       <c r="E72" s="18">
-        <f>La-D72</f>
+        <f t="shared" si="2"/>
         <v>2.4</v>
       </c>
       <c r="F72" s="18">
-        <f>-qG_1/2*(La-D72)^2</f>
+        <f t="shared" si="3"/>
         <v>-18.961609144775505</v>
       </c>
       <c r="G72" s="18">
-        <f>-qG_1*La*(1-D72/La)</f>
+        <f t="shared" si="4"/>
         <v>-15.801340953979588</v>
       </c>
       <c r="H72" s="17">
-        <f>-qG_2/2*(La-D72)^2</f>
-        <v>-7.1999999999999993</v>
+        <f t="shared" si="5"/>
+        <v>-14.399999999999999</v>
       </c>
       <c r="I72" s="17">
-        <f>-qG_2*La*(1-D72/La)</f>
-        <v>-6</v>
+        <f t="shared" si="6"/>
+        <v>-12</v>
       </c>
       <c r="J72" s="17">
-        <f>-qQ/2*(La-D72)^2</f>
-        <v>-43.199999999999996</v>
+        <f t="shared" si="7"/>
+        <v>-115.19999999999999</v>
       </c>
       <c r="K72" s="17">
-        <f>-qQ*La*(1-D72/La)</f>
-        <v>-36</v>
+        <f t="shared" si="8"/>
+        <v>-96</v>
       </c>
       <c r="L72" s="3">
         <v>0</v>
@@ -3335,36 +3411,36 @@
         <v>0</v>
       </c>
       <c r="N72" s="17">
-        <f t="shared" si="0"/>
-        <v>-43.199999999999996</v>
+        <f t="shared" si="16"/>
+        <v>-115.19999999999999</v>
       </c>
       <c r="O72" s="17">
-        <f t="shared" si="1"/>
-        <v>-36</v>
+        <f t="shared" si="17"/>
+        <v>-96</v>
       </c>
       <c r="Q72" s="18">
-        <f>GammaG*(F72+H72)+GammaQ*J72</f>
-        <v>-100.11817234544694</v>
+        <f t="shared" si="9"/>
+        <v>-217.83817234544691</v>
       </c>
       <c r="R72" s="18">
-        <f>GammaG*(G72+I72)+GammaQ*K72</f>
-        <v>-83.431810287872452</v>
+        <f t="shared" si="10"/>
+        <v>-181.53181028787245</v>
       </c>
       <c r="S72" s="18">
-        <f>GammaG*(F72+H72)+GammaQ*L72</f>
-        <v>-35.318172345446932</v>
+        <f t="shared" si="11"/>
+        <v>-45.038172345446931</v>
       </c>
       <c r="T72" s="18">
-        <f>GammaG*(G72+I72)+GammaQ*M72</f>
-        <v>-29.431810287872448</v>
+        <f t="shared" si="12"/>
+        <v>-37.531810287872446</v>
       </c>
       <c r="U72" s="18">
-        <f>GammaG*(F72+H72)+GammaQ*N72</f>
-        <v>-100.11817234544694</v>
+        <f t="shared" si="13"/>
+        <v>-217.83817234544691</v>
       </c>
       <c r="V72" s="18">
-        <f>GammaG*(G72+I72)+GammaQ*O72</f>
-        <v>-83.431810287872452</v>
+        <f t="shared" si="14"/>
+        <v>-181.53181028787245</v>
       </c>
     </row>
     <row r="73" spans="2:23" x14ac:dyDescent="0.25">
@@ -3373,36 +3449,36 @@
         <v>10</v>
       </c>
       <c r="D73" s="28">
-        <f>D74+La/10</f>
+        <f t="shared" si="15"/>
         <v>0.3</v>
       </c>
       <c r="E73" s="18">
-        <f>La-D73</f>
+        <f t="shared" si="2"/>
         <v>2.7</v>
       </c>
       <c r="F73" s="18">
-        <f>-qG_1/2*(La-D73)^2</f>
+        <f t="shared" si="3"/>
         <v>-23.9982865738565</v>
       </c>
       <c r="G73" s="18">
-        <f>-qG_1*La*(1-D73/La)</f>
+        <f t="shared" si="4"/>
         <v>-17.776508573227037</v>
       </c>
       <c r="H73" s="17">
-        <f>-qG_2/2*(La-D73)^2</f>
-        <v>-9.1125000000000007</v>
+        <f t="shared" si="5"/>
+        <v>-18.225000000000001</v>
       </c>
       <c r="I73" s="17">
-        <f>-qG_2*La*(1-D73/La)</f>
-        <v>-6.75</v>
+        <f t="shared" si="6"/>
+        <v>-13.5</v>
       </c>
       <c r="J73" s="17">
-        <f>-qQ/2*(La-D73)^2</f>
-        <v>-54.675000000000004</v>
+        <f t="shared" si="7"/>
+        <v>-145.80000000000001</v>
       </c>
       <c r="K73" s="17">
-        <f>-qQ*La*(1-D73/La)</f>
-        <v>-40.5</v>
+        <f t="shared" si="8"/>
+        <v>-108</v>
       </c>
       <c r="L73" s="3">
         <v>0</v>
@@ -3411,36 +3487,36 @@
         <v>0</v>
       </c>
       <c r="N73" s="17">
-        <f t="shared" si="0"/>
-        <v>-54.675000000000004</v>
+        <f t="shared" si="16"/>
+        <v>-145.80000000000001</v>
       </c>
       <c r="O73" s="17">
-        <f t="shared" si="1"/>
-        <v>-40.5</v>
+        <f t="shared" si="17"/>
+        <v>-108</v>
       </c>
       <c r="Q73" s="18">
-        <f>GammaG*(F73+H73)+GammaQ*J73</f>
-        <v>-126.71206187470628</v>
+        <f t="shared" si="9"/>
+        <v>-275.7014368747063</v>
       </c>
       <c r="R73" s="18">
-        <f>GammaG*(G73+I73)+GammaQ*K73</f>
-        <v>-93.860786573856501</v>
+        <f t="shared" si="10"/>
+        <v>-204.22328657385651</v>
       </c>
       <c r="S73" s="18">
-        <f>GammaG*(F73+H73)+GammaQ*L73</f>
-        <v>-44.699561874706276</v>
+        <f t="shared" si="11"/>
+        <v>-57.001436874706279</v>
       </c>
       <c r="T73" s="18">
-        <f>GammaG*(G73+I73)+GammaQ*M73</f>
-        <v>-33.110786573856501</v>
+        <f t="shared" si="12"/>
+        <v>-42.223286573856505</v>
       </c>
       <c r="U73" s="18">
-        <f>GammaG*(F73+H73)+GammaQ*N73</f>
-        <v>-126.71206187470628</v>
+        <f t="shared" si="13"/>
+        <v>-275.7014368747063</v>
       </c>
       <c r="V73" s="18">
-        <f>GammaG*(G73+I73)+GammaQ*O73</f>
-        <v>-93.860786573856501</v>
+        <f t="shared" si="14"/>
+        <v>-204.22328657385651</v>
       </c>
     </row>
     <row r="74" spans="2:23" x14ac:dyDescent="0.25">
@@ -3452,32 +3528,32 @@
         <v>0</v>
       </c>
       <c r="E74" s="18">
-        <f>La-D74</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="F74" s="18">
-        <f>-qG_1/2*(La-D74)^2</f>
+        <f t="shared" si="3"/>
         <v>-29.627514288711726</v>
       </c>
       <c r="G74" s="18">
-        <f>-qG_1*La*(1-D74/La)</f>
+        <f t="shared" si="4"/>
         <v>-19.751676192474484</v>
       </c>
       <c r="H74" s="17">
-        <f>-qG_2/2*(La-D74)^2</f>
-        <v>-11.25</v>
+        <f t="shared" si="5"/>
+        <v>-22.5</v>
       </c>
       <c r="I74" s="17">
-        <f>-qG_2*La*(1-D74/La)</f>
-        <v>-7.5</v>
+        <f t="shared" si="6"/>
+        <v>-15</v>
       </c>
       <c r="J74" s="17">
-        <f>-qQ/2*(La-D74)^2</f>
-        <v>-67.5</v>
+        <f t="shared" si="7"/>
+        <v>-180</v>
       </c>
       <c r="K74" s="17">
-        <f>-qQ*La*(1-D74/La)</f>
-        <v>-45</v>
+        <f t="shared" si="8"/>
+        <v>-120</v>
       </c>
       <c r="L74" s="3">
         <v>0</v>
@@ -3486,36 +3562,36 @@
         <v>0</v>
       </c>
       <c r="N74" s="17">
-        <f t="shared" si="0"/>
-        <v>-67.5</v>
+        <f t="shared" si="16"/>
+        <v>-180</v>
       </c>
       <c r="O74" s="17">
-        <f t="shared" si="1"/>
-        <v>-45</v>
+        <f t="shared" si="17"/>
+        <v>-120</v>
       </c>
       <c r="Q74" s="18">
-        <f>GammaG*(F74+H74)+GammaQ*J74</f>
-        <v>-156.43464428976083</v>
+        <f t="shared" si="9"/>
+        <v>-340.37214428976085</v>
       </c>
       <c r="R74" s="18">
-        <f>GammaG*(G74+I74)+GammaQ*K74</f>
-        <v>-104.28976285984055</v>
+        <f t="shared" si="10"/>
+        <v>-226.91476285984055</v>
       </c>
       <c r="S74" s="18">
-        <f>GammaG*(F74+H74)+GammaQ*L74</f>
-        <v>-55.184644289760833</v>
+        <f t="shared" si="11"/>
+        <v>-70.372144289760826</v>
       </c>
       <c r="T74" s="18">
-        <f>GammaG*(G74+I74)+GammaQ*M74</f>
-        <v>-36.789762859840557</v>
+        <f t="shared" si="12"/>
+        <v>-46.914762859840557</v>
       </c>
       <c r="U74" s="18">
-        <f>GammaG*(F74+H74)+GammaQ*N74</f>
-        <v>-156.43464428976083</v>
+        <f t="shared" si="13"/>
+        <v>-340.37214428976085</v>
       </c>
       <c r="V74" s="18">
-        <f>GammaG*(G74+I74)+GammaQ*O74</f>
-        <v>-104.28976285984055</v>
+        <f t="shared" si="14"/>
+        <v>-226.91476285984055</v>
       </c>
     </row>
     <row r="75" spans="2:23" x14ac:dyDescent="0.25">
@@ -3529,71 +3605,71 @@
         <v>0</v>
       </c>
       <c r="F75" s="18">
-        <f>-qG_1*La^2/2*(LL-D75)/LL+qG_1*(D75*(LL-D75))/2</f>
+        <f t="shared" ref="F75:F95" si="18">-qG_1*La^2/2*(LL-D75)/LL+qG_1*(D75*(LL-D75))/2</f>
         <v>-29.62751428871173</v>
       </c>
       <c r="G75" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D75)</f>
+        <f t="shared" ref="G75:G95" si="19">+qG_1*La^2/2/LL+qG_1/2*(LL-2*D75)</f>
         <v>35.882211749661977</v>
       </c>
       <c r="H75" s="17">
-        <f>-qG_2*La^2/2*(LL-D75)/LL+qG_2*(D75*(LL-D75))/2</f>
-        <v>-11.25</v>
+        <f t="shared" ref="H75:H95" si="20">-qG_2*La^2/2*(LL-D75)/LL+qG_2*(D75*(LL-D75))/2</f>
+        <v>-22.5</v>
       </c>
       <c r="I75" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D75)</f>
-        <v>13.625</v>
+        <f t="shared" ref="I75:I95" si="21">+qG_2*La^2/2/LL+qG_2/2*(LL-2*D75)</f>
+        <v>27.25</v>
       </c>
       <c r="J75" s="17">
-        <f>-qQ*La^2/2*(LL-D75)/LL</f>
-        <v>-67.5</v>
+        <f t="shared" ref="J75:J95" si="22">-qQ*La^2/2*(LL-D75)/LL</f>
+        <v>-180</v>
       </c>
       <c r="K75" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" ref="K75:K95" si="23">+qQ*La^2/2/LL</f>
+        <v>18</v>
       </c>
       <c r="L75" s="17">
-        <f>qQ*(D75*(LL-D75))/2</f>
+        <f t="shared" ref="L75:L95" si="24">qQ*(D75*(LL-D75))/2</f>
         <v>0</v>
       </c>
       <c r="M75" s="17">
-        <f>qQ/2*(LL-2*D75)</f>
-        <v>75</v>
+        <f t="shared" ref="M75:M95" si="25">qQ/2*(LL-2*D75)</f>
+        <v>200</v>
       </c>
       <c r="N75" s="17">
-        <f t="shared" ref="N75:N95" si="2">J75+L75</f>
-        <v>-67.5</v>
+        <f t="shared" ref="N75:N95" si="26">J75+L75</f>
+        <v>-180</v>
       </c>
       <c r="O75" s="17">
-        <f t="shared" ref="O75:O95" si="3">K75+M75</f>
-        <v>81.75</v>
+        <f t="shared" ref="O75:O95" si="27">K75+M75</f>
+        <v>218</v>
       </c>
       <c r="Q75" s="18">
-        <f>GammaG*(F75+H75)+GammaQ*J75</f>
-        <v>-156.43464428976085</v>
+        <f t="shared" si="9"/>
+        <v>-340.37214428976085</v>
       </c>
       <c r="R75" s="18">
-        <f>GammaG*(G75+I75)+GammaQ*K75</f>
-        <v>76.959735862043672</v>
+        <f t="shared" si="10"/>
+        <v>112.22848586204367</v>
       </c>
       <c r="S75" s="18">
-        <f>GammaG*(F75+H75)+GammaQ*L75</f>
-        <v>-55.18464428976084</v>
+        <f t="shared" si="11"/>
+        <v>-70.37214428976084</v>
       </c>
       <c r="T75" s="18">
-        <f>GammaG*(G75+I75)+GammaQ*M75</f>
-        <v>179.33473586204366</v>
+        <f t="shared" si="12"/>
+        <v>385.22848586204367</v>
       </c>
       <c r="U75" s="18">
-        <f>GammaG*(F75+H75)+GammaQ*N75</f>
-        <v>-156.43464428976085</v>
+        <f t="shared" si="13"/>
+        <v>-340.37214428976085</v>
       </c>
       <c r="V75" s="18">
-        <f>GammaG*(G75+I75)+GammaQ*O75</f>
-        <v>189.45973586204366</v>
+        <f t="shared" si="14"/>
+        <v>412.22848586204367</v>
       </c>
       <c r="W75" s="18">
-        <f>D75</f>
+        <f t="shared" ref="W75:W95" si="28">D75</f>
         <v>0</v>
       </c>
     </row>
@@ -3603,75 +3679,75 @@
         <v>2</v>
       </c>
       <c r="D76" s="18">
-        <f>D75+LL/20</f>
+        <f t="shared" ref="D76:D95" si="29">D75+LL/20</f>
         <v>0.5</v>
       </c>
       <c r="F76" s="18">
-        <f>-qG_1*La^2/2*(LL-D76)/LL+qG_1*(D76*(LL-D76))/2</f>
+        <f t="shared" si="18"/>
         <v>-12.509394921900512</v>
       </c>
       <c r="G76" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D76)</f>
+        <f t="shared" si="19"/>
         <v>32.590265717582902</v>
       </c>
       <c r="H76" s="17">
-        <f>-qG_2*La^2/2*(LL-D76)/LL+qG_2*(D76*(LL-D76))/2</f>
-        <v>-4.75</v>
+        <f t="shared" si="20"/>
+        <v>-9.5</v>
       </c>
       <c r="I76" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D76)</f>
-        <v>12.375</v>
+        <f t="shared" si="21"/>
+        <v>24.75</v>
       </c>
       <c r="J76" s="17">
-        <f>-qQ*La^2/2*(LL-D76)/LL</f>
-        <v>-64.125</v>
+        <f t="shared" si="22"/>
+        <v>-171</v>
       </c>
       <c r="K76" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L76" s="17">
-        <f>qQ*(D76*(LL-D76))/2</f>
-        <v>35.625</v>
+        <f t="shared" si="24"/>
+        <v>95</v>
       </c>
       <c r="M76" s="17">
-        <f>qQ/2*(LL-2*D76)</f>
-        <v>67.5</v>
+        <f t="shared" si="25"/>
+        <v>180</v>
       </c>
       <c r="N76" s="17">
-        <f t="shared" si="2"/>
-        <v>-28.5</v>
+        <f t="shared" si="26"/>
+        <v>-76</v>
       </c>
       <c r="O76" s="17">
-        <f t="shared" si="3"/>
-        <v>74.25</v>
+        <f t="shared" si="27"/>
+        <v>198</v>
       </c>
       <c r="Q76" s="18">
-        <f>GammaG*(F76+H76)+GammaQ*J76</f>
-        <v>-119.48768314456569</v>
+        <f t="shared" si="9"/>
+        <v>-286.21268314456569</v>
       </c>
       <c r="R76" s="18">
-        <f>GammaG*(G76+I76)+GammaQ*K76</f>
-        <v>70.828108718736928</v>
+        <f t="shared" si="10"/>
+        <v>104.40935871873693</v>
       </c>
       <c r="S76" s="18">
-        <f>GammaG*(F76+H76)+GammaQ*L76</f>
-        <v>30.137316855434307</v>
+        <f t="shared" si="11"/>
+        <v>112.78731685543431</v>
       </c>
       <c r="T76" s="18">
-        <f>GammaG*(G76+I76)+GammaQ*M76</f>
-        <v>161.95310871873693</v>
+        <f t="shared" si="12"/>
+        <v>347.40935871873694</v>
       </c>
       <c r="U76" s="18">
-        <f>GammaG*(F76+H76)+GammaQ*N76</f>
-        <v>-66.050183144565693</v>
+        <f t="shared" si="13"/>
+        <v>-143.71268314456569</v>
       </c>
       <c r="V76" s="18">
-        <f>GammaG*(G76+I76)+GammaQ*O76</f>
-        <v>172.07810871873693</v>
+        <f t="shared" si="14"/>
+        <v>374.40935871873694</v>
       </c>
       <c r="W76" s="18">
-        <f>D76</f>
+        <f t="shared" si="28"/>
         <v>0.5</v>
       </c>
     </row>
@@ -3681,75 +3757,75 @@
         <v>3</v>
       </c>
       <c r="D77" s="18">
-        <f>D76+LL/20</f>
+        <f t="shared" si="29"/>
         <v>1</v>
       </c>
       <c r="F77" s="18">
-        <f>-qG_1*La^2/2*(LL-D77)/LL+qG_1*(D77*(LL-D77))/2</f>
+        <f t="shared" si="18"/>
         <v>2.9627514288711687</v>
       </c>
       <c r="G77" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D77)</f>
+        <f t="shared" si="19"/>
         <v>29.298319685503817</v>
       </c>
       <c r="H77" s="17">
-        <f>-qG_2*La^2/2*(LL-D77)/LL+qG_2*(D77*(LL-D77))/2</f>
-        <v>1.125</v>
+        <f t="shared" si="20"/>
+        <v>2.25</v>
       </c>
       <c r="I77" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D77)</f>
-        <v>11.125</v>
+        <f t="shared" si="21"/>
+        <v>22.25</v>
       </c>
       <c r="J77" s="17">
-        <f>-qQ*La^2/2*(LL-D77)/LL</f>
-        <v>-60.75</v>
+        <f t="shared" si="22"/>
+        <v>-162</v>
       </c>
       <c r="K77" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L77" s="17">
-        <f>qQ*(D77*(LL-D77))/2</f>
-        <v>67.5</v>
+        <f t="shared" si="24"/>
+        <v>180</v>
       </c>
       <c r="M77" s="17">
-        <f>qQ/2*(LL-2*D77)</f>
-        <v>60</v>
+        <f t="shared" si="25"/>
+        <v>160</v>
       </c>
       <c r="N77" s="17">
-        <f t="shared" si="2"/>
-        <v>6.75</v>
+        <f t="shared" si="26"/>
+        <v>18</v>
       </c>
       <c r="O77" s="17">
-        <f t="shared" si="3"/>
-        <v>66.75</v>
+        <f t="shared" si="27"/>
+        <v>178</v>
       </c>
       <c r="Q77" s="18">
-        <f>GammaG*(F77+H77)+GammaQ*J77</f>
-        <v>-85.606535571023926</v>
+        <f t="shared" si="9"/>
+        <v>-235.96278557102391</v>
       </c>
       <c r="R77" s="18">
-        <f>GammaG*(G77+I77)+GammaQ*K77</f>
-        <v>64.696481575430141</v>
+        <f t="shared" si="10"/>
+        <v>96.590231575430153</v>
       </c>
       <c r="S77" s="18">
-        <f>GammaG*(F77+H77)+GammaQ*L77</f>
-        <v>106.76846442897607</v>
+        <f t="shared" si="11"/>
+        <v>277.03721442897609</v>
       </c>
       <c r="T77" s="18">
-        <f>GammaG*(G77+I77)+GammaQ*M77</f>
-        <v>144.57148157543014</v>
+        <f t="shared" si="12"/>
+        <v>309.59023157543015</v>
       </c>
       <c r="U77" s="18">
-        <f>GammaG*(F77+H77)+GammaQ*N77</f>
-        <v>15.643464428976078</v>
+        <f t="shared" si="13"/>
+        <v>34.037214428976078</v>
       </c>
       <c r="V77" s="18">
-        <f>GammaG*(G77+I77)+GammaQ*O77</f>
-        <v>154.69648157543014</v>
+        <f t="shared" si="14"/>
+        <v>336.59023157543015</v>
       </c>
       <c r="W77" s="18">
-        <f>D77</f>
+        <f t="shared" si="28"/>
         <v>1</v>
       </c>
     </row>
@@ -3759,75 +3835,75 @@
         <v>4</v>
       </c>
       <c r="D78" s="18">
-        <f>D77+LL/20</f>
+        <f t="shared" si="29"/>
         <v>1.5</v>
       </c>
       <c r="F78" s="18">
-        <f>-qG_1*La^2/2*(LL-D78)/LL+qG_1*(D78*(LL-D78))/2</f>
+        <f t="shared" si="18"/>
         <v>16.788924763603308</v>
       </c>
       <c r="G78" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D78)</f>
+        <f t="shared" si="19"/>
         <v>26.006373653424735</v>
       </c>
       <c r="H78" s="17">
-        <f>-qG_2*La^2/2*(LL-D78)/LL+qG_2*(D78*(LL-D78))/2</f>
-        <v>6.375</v>
+        <f t="shared" si="20"/>
+        <v>12.75</v>
       </c>
       <c r="I78" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D78)</f>
-        <v>9.875</v>
+        <f t="shared" si="21"/>
+        <v>19.75</v>
       </c>
       <c r="J78" s="17">
-        <f>-qQ*La^2/2*(LL-D78)/LL</f>
-        <v>-57.375</v>
+        <f t="shared" si="22"/>
+        <v>-153</v>
       </c>
       <c r="K78" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L78" s="17">
-        <f>qQ*(D78*(LL-D78))/2</f>
-        <v>95.625</v>
+        <f t="shared" si="24"/>
+        <v>255</v>
       </c>
       <c r="M78" s="17">
-        <f>qQ/2*(LL-2*D78)</f>
-        <v>52.5</v>
+        <f t="shared" si="25"/>
+        <v>140</v>
       </c>
       <c r="N78" s="17">
-        <f t="shared" si="2"/>
-        <v>38.25</v>
+        <f t="shared" si="26"/>
+        <v>102</v>
       </c>
       <c r="O78" s="17">
-        <f t="shared" si="3"/>
-        <v>59.25</v>
+        <f t="shared" si="27"/>
+        <v>158</v>
       </c>
       <c r="Q78" s="18">
-        <f>GammaG*(F78+H78)+GammaQ*J78</f>
-        <v>-54.791201569135531</v>
+        <f t="shared" si="9"/>
+        <v>-189.62245156913554</v>
       </c>
       <c r="R78" s="18">
-        <f>GammaG*(G78+I78)+GammaQ*K78</f>
-        <v>58.56485443212339</v>
+        <f t="shared" si="10"/>
+        <v>88.771104432123394</v>
       </c>
       <c r="S78" s="18">
-        <f>GammaG*(F78+H78)+GammaQ*L78</f>
-        <v>174.70879843086448</v>
+        <f t="shared" si="11"/>
+        <v>422.37754843086446</v>
       </c>
       <c r="T78" s="18">
-        <f>GammaG*(G78+I78)+GammaQ*M78</f>
-        <v>127.18985443212338</v>
+        <f t="shared" si="12"/>
+        <v>271.77110443212337</v>
       </c>
       <c r="U78" s="18">
-        <f>GammaG*(F78+H78)+GammaQ*N78</f>
-        <v>88.646298430864476</v>
+        <f t="shared" si="13"/>
+        <v>192.87754843086446</v>
       </c>
       <c r="V78" s="18">
-        <f>GammaG*(G78+I78)+GammaQ*O78</f>
-        <v>137.31485443212338</v>
+        <f t="shared" si="14"/>
+        <v>298.77110443212337</v>
       </c>
       <c r="W78" s="18">
-        <f>D78</f>
+        <f t="shared" si="28"/>
         <v>1.5</v>
       </c>
     </row>
@@ -3837,75 +3913,75 @@
         <v>5</v>
       </c>
       <c r="D79" s="18">
-        <f>D78+LL/20</f>
+        <f t="shared" si="29"/>
         <v>2</v>
       </c>
       <c r="F79" s="18">
-        <f>-qG_1*La^2/2*(LL-D79)/LL+qG_1*(D79*(LL-D79))/2</f>
+        <f t="shared" si="18"/>
         <v>28.969125082295907</v>
       </c>
       <c r="G79" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D79)</f>
+        <f t="shared" si="19"/>
         <v>22.714427621345656</v>
       </c>
       <c r="H79" s="17">
-        <f>-qG_2*La^2/2*(LL-D79)/LL+qG_2*(D79*(LL-D79))/2</f>
-        <v>11</v>
+        <f t="shared" si="20"/>
+        <v>22</v>
       </c>
       <c r="I79" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D79)</f>
-        <v>8.625</v>
+        <f t="shared" si="21"/>
+        <v>17.25</v>
       </c>
       <c r="J79" s="17">
-        <f>-qQ*La^2/2*(LL-D79)/LL</f>
-        <v>-54</v>
+        <f t="shared" si="22"/>
+        <v>-144</v>
       </c>
       <c r="K79" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L79" s="17">
-        <f>qQ*(D79*(LL-D79))/2</f>
+        <f t="shared" si="24"/>
+        <v>320</v>
+      </c>
+      <c r="M79" s="17">
+        <f t="shared" si="25"/>
         <v>120</v>
       </c>
-      <c r="M79" s="17">
-        <f>qQ/2*(LL-2*D79)</f>
-        <v>45</v>
-      </c>
       <c r="N79" s="17">
-        <f t="shared" si="2"/>
-        <v>66</v>
+        <f t="shared" si="26"/>
+        <v>176</v>
       </c>
       <c r="O79" s="17">
-        <f t="shared" si="3"/>
-        <v>51.75</v>
+        <f t="shared" si="27"/>
+        <v>138</v>
       </c>
       <c r="Q79" s="18">
-        <f>GammaG*(F79+H79)+GammaQ*J79</f>
-        <v>-27.041681138900529</v>
+        <f t="shared" si="9"/>
+        <v>-147.19168113890052</v>
       </c>
       <c r="R79" s="18">
-        <f>GammaG*(G79+I79)+GammaQ*K79</f>
-        <v>52.433227288816639</v>
+        <f t="shared" si="10"/>
+        <v>80.951977288816636</v>
       </c>
       <c r="S79" s="18">
-        <f>GammaG*(F79+H79)+GammaQ*L79</f>
-        <v>233.95831886109949</v>
+        <f t="shared" si="11"/>
+        <v>548.80831886109945</v>
       </c>
       <c r="T79" s="18">
-        <f>GammaG*(G79+I79)+GammaQ*M79</f>
-        <v>109.80822728881664</v>
+        <f t="shared" si="12"/>
+        <v>233.95197728881664</v>
       </c>
       <c r="U79" s="18">
-        <f>GammaG*(F79+H79)+GammaQ*N79</f>
-        <v>152.95831886109949</v>
+        <f t="shared" si="13"/>
+        <v>332.80831886109945</v>
       </c>
       <c r="V79" s="18">
-        <f>GammaG*(G79+I79)+GammaQ*O79</f>
-        <v>119.93322728881664</v>
+        <f t="shared" si="14"/>
+        <v>260.95197728881664</v>
       </c>
       <c r="W79" s="18">
-        <f>D79</f>
+        <f t="shared" si="28"/>
         <v>2</v>
       </c>
     </row>
@@ -3915,75 +3991,75 @@
         <v>6</v>
       </c>
       <c r="D80" s="18">
-        <f>D79+LL/20</f>
+        <f t="shared" si="29"/>
         <v>2.5</v>
       </c>
       <c r="F80" s="18">
-        <f>-qG_1*La^2/2*(LL-D80)/LL+qG_1*(D80*(LL-D80))/2</f>
+        <f t="shared" si="18"/>
         <v>39.503352384948968</v>
       </c>
       <c r="G80" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D80)</f>
+        <f t="shared" si="19"/>
         <v>19.422481589266575</v>
       </c>
       <c r="H80" s="17">
-        <f>-qG_2*La^2/2*(LL-D80)/LL+qG_2*(D80*(LL-D80))/2</f>
-        <v>15</v>
+        <f t="shared" si="20"/>
+        <v>30</v>
       </c>
       <c r="I80" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D80)</f>
-        <v>7.375</v>
+        <f t="shared" si="21"/>
+        <v>14.75</v>
       </c>
       <c r="J80" s="17">
-        <f>-qQ*La^2/2*(LL-D80)/LL</f>
-        <v>-50.625</v>
+        <f t="shared" si="22"/>
+        <v>-135</v>
       </c>
       <c r="K80" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L80" s="17">
-        <f>qQ*(D80*(LL-D80))/2</f>
-        <v>140.625</v>
+        <f t="shared" si="24"/>
+        <v>375</v>
       </c>
       <c r="M80" s="17">
-        <f>qQ/2*(LL-2*D80)</f>
-        <v>37.5</v>
+        <f t="shared" si="25"/>
+        <v>100</v>
       </c>
       <c r="N80" s="17">
-        <f t="shared" si="2"/>
-        <v>90</v>
+        <f t="shared" si="26"/>
+        <v>240</v>
       </c>
       <c r="O80" s="17">
-        <f t="shared" si="3"/>
-        <v>44.25</v>
+        <f t="shared" si="27"/>
+        <v>118</v>
       </c>
       <c r="Q80" s="18">
-        <f>GammaG*(F80+H80)+GammaQ*J80</f>
-        <v>-2.357974280318885</v>
+        <f t="shared" si="9"/>
+        <v>-108.67047428031889</v>
       </c>
       <c r="R80" s="18">
-        <f>GammaG*(G80+I80)+GammaQ*K80</f>
-        <v>46.30160014550988</v>
+        <f t="shared" si="10"/>
+        <v>73.132850145509877</v>
       </c>
       <c r="S80" s="18">
-        <f>GammaG*(F80+H80)+GammaQ*L80</f>
-        <v>284.5170257196811</v>
+        <f t="shared" si="11"/>
+        <v>656.3295257196811</v>
       </c>
       <c r="T80" s="18">
-        <f>GammaG*(G80+I80)+GammaQ*M80</f>
-        <v>92.42660014550988</v>
+        <f t="shared" si="12"/>
+        <v>196.13285014550988</v>
       </c>
       <c r="U80" s="18">
-        <f>GammaG*(F80+H80)+GammaQ*N80</f>
-        <v>208.5795257196811</v>
+        <f t="shared" si="13"/>
+        <v>453.8295257196811</v>
       </c>
       <c r="V80" s="18">
-        <f>GammaG*(G80+I80)+GammaQ*O80</f>
-        <v>102.55160014550988</v>
+        <f t="shared" si="14"/>
+        <v>223.13285014550988</v>
       </c>
       <c r="W80" s="18">
-        <f>D80</f>
+        <f t="shared" si="28"/>
         <v>2.5</v>
       </c>
     </row>
@@ -3993,75 +4069,75 @@
         <v>7</v>
       </c>
       <c r="D81" s="18">
-        <f>D80+LL/20</f>
+        <f t="shared" si="29"/>
         <v>3</v>
       </c>
       <c r="F81" s="18">
-        <f>-qG_1*La^2/2*(LL-D81)/LL+qG_1*(D81*(LL-D81))/2</f>
+        <f t="shared" si="18"/>
         <v>48.391606671562485</v>
       </c>
       <c r="G81" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D81)</f>
+        <f t="shared" si="19"/>
         <v>16.130535557187496</v>
       </c>
       <c r="H81" s="17">
-        <f>-qG_2*La^2/2*(LL-D81)/LL+qG_2*(D81*(LL-D81))/2</f>
-        <v>18.375</v>
+        <f t="shared" si="20"/>
+        <v>36.75</v>
       </c>
       <c r="I81" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D81)</f>
-        <v>6.125</v>
+        <f t="shared" si="21"/>
+        <v>12.25</v>
       </c>
       <c r="J81" s="17">
-        <f>-qQ*La^2/2*(LL-D81)/LL</f>
-        <v>-47.25</v>
+        <f t="shared" si="22"/>
+        <v>-126</v>
       </c>
       <c r="K81" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L81" s="17">
-        <f>qQ*(D81*(LL-D81))/2</f>
-        <v>157.5</v>
+        <f t="shared" si="24"/>
+        <v>420</v>
       </c>
       <c r="M81" s="17">
-        <f>qQ/2*(LL-2*D81)</f>
-        <v>30</v>
+        <f t="shared" si="25"/>
+        <v>80</v>
       </c>
       <c r="N81" s="17">
-        <f t="shared" si="2"/>
-        <v>110.25</v>
+        <f t="shared" si="26"/>
+        <v>294</v>
       </c>
       <c r="O81" s="17">
-        <f t="shared" si="3"/>
-        <v>36.75</v>
+        <f t="shared" si="27"/>
+        <v>98</v>
       </c>
       <c r="Q81" s="18">
-        <f>GammaG*(F81+H81)+GammaQ*J81</f>
-        <v>19.259919006609366</v>
+        <f t="shared" si="9"/>
+        <v>-74.058830993390643</v>
       </c>
       <c r="R81" s="18">
-        <f>GammaG*(G81+I81)+GammaQ*K81</f>
-        <v>40.169973002203122</v>
+        <f t="shared" si="10"/>
+        <v>65.313723002203119</v>
       </c>
       <c r="S81" s="18">
-        <f>GammaG*(F81+H81)+GammaQ*L81</f>
-        <v>326.38491900660938</v>
+        <f t="shared" si="11"/>
+        <v>744.94116900660936</v>
       </c>
       <c r="T81" s="18">
-        <f>GammaG*(G81+I81)+GammaQ*M81</f>
-        <v>75.044973002203122</v>
+        <f t="shared" si="12"/>
+        <v>158.31372300220312</v>
       </c>
       <c r="U81" s="18">
-        <f>GammaG*(F81+H81)+GammaQ*N81</f>
-        <v>255.50991900660938</v>
+        <f t="shared" si="13"/>
+        <v>555.94116900660936</v>
       </c>
       <c r="V81" s="18">
-        <f>GammaG*(G81+I81)+GammaQ*O81</f>
-        <v>85.169973002203122</v>
+        <f t="shared" si="14"/>
+        <v>185.31372300220312</v>
       </c>
       <c r="W81" s="18">
-        <f>D81</f>
+        <f t="shared" si="28"/>
         <v>3</v>
       </c>
     </row>
@@ -4071,75 +4147,75 @@
         <v>8</v>
       </c>
       <c r="D82" s="18">
-        <f>D81+LL/20</f>
+        <f t="shared" si="29"/>
         <v>3.5</v>
       </c>
       <c r="F82" s="18">
-        <f>-qG_1*La^2/2*(LL-D82)/LL+qG_1*(D82*(LL-D82))/2</f>
+        <f t="shared" si="18"/>
         <v>55.633887942136468</v>
       </c>
       <c r="G82" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D82)</f>
+        <f t="shared" si="19"/>
         <v>12.838589525108414</v>
       </c>
       <c r="H82" s="17">
-        <f>-qG_2*La^2/2*(LL-D82)/LL+qG_2*(D82*(LL-D82))/2</f>
-        <v>21.125</v>
+        <f t="shared" si="20"/>
+        <v>42.25</v>
       </c>
       <c r="I82" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D82)</f>
-        <v>4.875</v>
+        <f t="shared" si="21"/>
+        <v>9.75</v>
       </c>
       <c r="J82" s="17">
-        <f>-qQ*La^2/2*(LL-D82)/LL</f>
-        <v>-43.875</v>
+        <f t="shared" si="22"/>
+        <v>-117</v>
       </c>
       <c r="K82" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L82" s="17">
-        <f>qQ*(D82*(LL-D82))/2</f>
-        <v>170.625</v>
+        <f t="shared" si="24"/>
+        <v>455</v>
       </c>
       <c r="M82" s="17">
-        <f>qQ/2*(LL-2*D82)</f>
-        <v>22.5</v>
+        <f t="shared" si="25"/>
+        <v>60</v>
       </c>
       <c r="N82" s="17">
-        <f t="shared" si="2"/>
-        <v>126.75</v>
+        <f t="shared" si="26"/>
+        <v>338</v>
       </c>
       <c r="O82" s="17">
-        <f t="shared" si="3"/>
-        <v>29.25</v>
+        <f t="shared" si="27"/>
+        <v>78</v>
       </c>
       <c r="Q82" s="18">
-        <f>GammaG*(F82+H82)+GammaQ*J82</f>
-        <v>37.811998721884237</v>
+        <f t="shared" si="9"/>
+        <v>-43.356751278115752</v>
       </c>
       <c r="R82" s="18">
-        <f>GammaG*(G82+I82)+GammaQ*K82</f>
-        <v>34.038345858896363</v>
+        <f t="shared" si="10"/>
+        <v>57.494595858896361</v>
       </c>
       <c r="S82" s="18">
-        <f>GammaG*(F82+H82)+GammaQ*L82</f>
-        <v>359.56199872188427</v>
+        <f t="shared" si="11"/>
+        <v>814.64324872188422</v>
       </c>
       <c r="T82" s="18">
-        <f>GammaG*(G82+I82)+GammaQ*M82</f>
-        <v>57.663345858896363</v>
+        <f t="shared" si="12"/>
+        <v>120.49459585889636</v>
       </c>
       <c r="U82" s="18">
-        <f>GammaG*(F82+H82)+GammaQ*N82</f>
-        <v>293.74949872188427</v>
+        <f t="shared" si="13"/>
+        <v>639.14324872188422</v>
       </c>
       <c r="V82" s="18">
-        <f>GammaG*(G82+I82)+GammaQ*O82</f>
-        <v>67.788345858896363</v>
+        <f t="shared" si="14"/>
+        <v>147.49459585889636</v>
       </c>
       <c r="W82" s="18">
-        <f>D82</f>
+        <f t="shared" si="28"/>
         <v>3.5</v>
       </c>
     </row>
@@ -4149,75 +4225,75 @@
         <v>9</v>
       </c>
       <c r="D83" s="18">
-        <f>D82+LL/20</f>
+        <f t="shared" si="29"/>
         <v>4</v>
       </c>
       <c r="F83" s="18">
-        <f>-qG_1*La^2/2*(LL-D83)/LL+qG_1*(D83*(LL-D83))/2</f>
+        <f t="shared" si="18"/>
         <v>61.230196196670903</v>
       </c>
       <c r="G83" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D83)</f>
+        <f t="shared" si="19"/>
         <v>9.5466434930293342</v>
       </c>
       <c r="H83" s="17">
-        <f>-qG_2*La^2/2*(LL-D83)/LL+qG_2*(D83*(LL-D83))/2</f>
-        <v>23.25</v>
+        <f t="shared" si="20"/>
+        <v>46.5</v>
       </c>
       <c r="I83" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D83)</f>
-        <v>3.625</v>
+        <f t="shared" si="21"/>
+        <v>7.25</v>
       </c>
       <c r="J83" s="17">
-        <f>-qQ*La^2/2*(LL-D83)/LL</f>
-        <v>-40.5</v>
+        <f t="shared" si="22"/>
+        <v>-108</v>
       </c>
       <c r="K83" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L83" s="17">
-        <f>qQ*(D83*(LL-D83))/2</f>
-        <v>180</v>
+        <f t="shared" si="24"/>
+        <v>480</v>
       </c>
       <c r="M83" s="17">
-        <f>qQ/2*(LL-2*D83)</f>
-        <v>15</v>
+        <f t="shared" si="25"/>
+        <v>40</v>
       </c>
       <c r="N83" s="17">
-        <f t="shared" si="2"/>
-        <v>139.5</v>
+        <f t="shared" si="26"/>
+        <v>372</v>
       </c>
       <c r="O83" s="17">
-        <f t="shared" si="3"/>
-        <v>21.75</v>
+        <f t="shared" si="27"/>
+        <v>58</v>
       </c>
       <c r="Q83" s="18">
-        <f>GammaG*(F83+H83)+GammaQ*J83</f>
-        <v>53.298264865505729</v>
+        <f t="shared" si="9"/>
+        <v>-16.564235134494282</v>
       </c>
       <c r="R83" s="18">
-        <f>GammaG*(G83+I83)+GammaQ*K83</f>
-        <v>27.906718715589601</v>
+        <f t="shared" si="10"/>
+        <v>49.675468715589602</v>
       </c>
       <c r="S83" s="18">
-        <f>GammaG*(F83+H83)+GammaQ*L83</f>
-        <v>384.04826486550576</v>
+        <f t="shared" si="11"/>
+        <v>865.43576486550569</v>
       </c>
       <c r="T83" s="18">
-        <f>GammaG*(G83+I83)+GammaQ*M83</f>
-        <v>40.281718715589605</v>
+        <f t="shared" si="12"/>
+        <v>82.675468715589602</v>
       </c>
       <c r="U83" s="18">
-        <f>GammaG*(F83+H83)+GammaQ*N83</f>
-        <v>323.29826486550576</v>
+        <f t="shared" si="13"/>
+        <v>703.43576486550569</v>
       </c>
       <c r="V83" s="18">
-        <f>GammaG*(G83+I83)+GammaQ*O83</f>
-        <v>50.406718715589605</v>
+        <f t="shared" si="14"/>
+        <v>109.6754687155896</v>
       </c>
       <c r="W83" s="18">
-        <f>D83</f>
+        <f t="shared" si="28"/>
         <v>4</v>
       </c>
     </row>
@@ -4227,75 +4303,75 @@
         <v>10</v>
       </c>
       <c r="D84" s="18">
-        <f>D83+LL/20</f>
+        <f t="shared" si="29"/>
         <v>4.5</v>
       </c>
       <c r="F84" s="18">
-        <f>-qG_1*La^2/2*(LL-D84)/LL+qG_1*(D84*(LL-D84))/2</f>
+        <f t="shared" si="18"/>
         <v>65.18053143516579</v>
       </c>
       <c r="G84" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D84)</f>
+        <f t="shared" si="19"/>
         <v>6.2546974609502533</v>
       </c>
       <c r="H84" s="17">
-        <f>-qG_2*La^2/2*(LL-D84)/LL+qG_2*(D84*(LL-D84))/2</f>
-        <v>24.75</v>
+        <f t="shared" si="20"/>
+        <v>49.5</v>
       </c>
       <c r="I84" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D84)</f>
-        <v>2.375</v>
+        <f t="shared" si="21"/>
+        <v>4.75</v>
       </c>
       <c r="J84" s="17">
-        <f>-qQ*La^2/2*(LL-D84)/LL</f>
-        <v>-37.125</v>
+        <f t="shared" si="22"/>
+        <v>-99</v>
       </c>
       <c r="K84" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L84" s="17">
-        <f>qQ*(D84*(LL-D84))/2</f>
-        <v>185.625</v>
+        <f t="shared" si="24"/>
+        <v>495</v>
       </c>
       <c r="M84" s="17">
-        <f>qQ/2*(LL-2*D84)</f>
-        <v>7.5</v>
+        <f t="shared" si="25"/>
+        <v>20</v>
       </c>
       <c r="N84" s="17">
-        <f t="shared" si="2"/>
-        <v>148.5</v>
+        <f t="shared" si="26"/>
+        <v>396</v>
       </c>
       <c r="O84" s="17">
-        <f t="shared" si="3"/>
-        <v>14.25</v>
+        <f t="shared" si="27"/>
+        <v>38</v>
       </c>
       <c r="Q84" s="18">
-        <f>GammaG*(F84+H84)+GammaQ*J84</f>
-        <v>65.718717437473828</v>
+        <f t="shared" si="9"/>
+        <v>6.318717437473822</v>
       </c>
       <c r="R84" s="18">
-        <f>GammaG*(G84+I84)+GammaQ*K84</f>
-        <v>21.775091572282843</v>
+        <f t="shared" si="10"/>
+        <v>41.856341572282844</v>
       </c>
       <c r="S84" s="18">
-        <f>GammaG*(F84+H84)+GammaQ*L84</f>
-        <v>399.84371743747386</v>
+        <f t="shared" si="11"/>
+        <v>897.31871743747388</v>
       </c>
       <c r="T84" s="18">
-        <f>GammaG*(G84+I84)+GammaQ*M84</f>
-        <v>22.900091572282843</v>
+        <f t="shared" si="12"/>
+        <v>44.856341572282844</v>
       </c>
       <c r="U84" s="18">
-        <f>GammaG*(F84+H84)+GammaQ*N84</f>
-        <v>344.15621743747386</v>
+        <f t="shared" si="13"/>
+        <v>748.81871743747388</v>
       </c>
       <c r="V84" s="18">
-        <f>GammaG*(G84+I84)+GammaQ*O84</f>
-        <v>33.025091572282847</v>
+        <f t="shared" si="14"/>
+        <v>71.856341572282844</v>
       </c>
       <c r="W84" s="18">
-        <f>D84</f>
+        <f t="shared" si="28"/>
         <v>4.5</v>
       </c>
     </row>
@@ -4305,75 +4381,75 @@
         <v>11</v>
       </c>
       <c r="D85" s="18">
-        <f>D84+LL/20</f>
+        <f t="shared" si="29"/>
         <v>5</v>
       </c>
       <c r="F85" s="18">
-        <f>-qG_1*La^2/2*(LL-D85)/LL+qG_1*(D85*(LL-D85))/2</f>
+        <f t="shared" si="18"/>
         <v>67.484893657621157</v>
       </c>
       <c r="G85" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D85)</f>
+        <f t="shared" si="19"/>
         <v>2.9627514288711727</v>
       </c>
       <c r="H85" s="17">
-        <f>-qG_2*La^2/2*(LL-D85)/LL+qG_2*(D85*(LL-D85))/2</f>
-        <v>25.625</v>
+        <f t="shared" si="20"/>
+        <v>51.25</v>
       </c>
       <c r="I85" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D85)</f>
-        <v>1.125</v>
+        <f t="shared" si="21"/>
+        <v>2.25</v>
       </c>
       <c r="J85" s="17">
-        <f>-qQ*La^2/2*(LL-D85)/LL</f>
-        <v>-33.75</v>
+        <f t="shared" si="22"/>
+        <v>-90</v>
       </c>
       <c r="K85" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L85" s="17">
-        <f>qQ*(D85*(LL-D85))/2</f>
-        <v>187.5</v>
+        <f t="shared" si="24"/>
+        <v>500</v>
       </c>
       <c r="M85" s="17">
-        <f>qQ/2*(LL-2*D85)</f>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="N85" s="17">
-        <f t="shared" si="2"/>
-        <v>153.75</v>
+        <f t="shared" si="26"/>
+        <v>410</v>
       </c>
       <c r="O85" s="17">
-        <f t="shared" si="3"/>
-        <v>6.75</v>
+        <f t="shared" si="27"/>
+        <v>18</v>
       </c>
       <c r="Q85" s="18">
-        <f>GammaG*(F85+H85)+GammaQ*J85</f>
-        <v>75.073356437788576</v>
+        <f t="shared" si="9"/>
+        <v>25.292106437788561</v>
       </c>
       <c r="R85" s="18">
-        <f>GammaG*(G85+I85)+GammaQ*K85</f>
-        <v>15.643464428976083</v>
+        <f t="shared" si="10"/>
+        <v>34.037214428976085</v>
       </c>
       <c r="S85" s="18">
-        <f>GammaG*(F85+H85)+GammaQ*L85</f>
-        <v>406.94835643778856</v>
+        <f t="shared" si="11"/>
+        <v>910.29210643778856</v>
       </c>
       <c r="T85" s="18">
-        <f>GammaG*(G85+I85)+GammaQ*M85</f>
-        <v>5.5184644289760829</v>
+        <f t="shared" si="12"/>
+        <v>7.0372144289760827</v>
       </c>
       <c r="U85" s="18">
-        <f>GammaG*(F85+H85)+GammaQ*N85</f>
-        <v>356.32335643778856</v>
+        <f t="shared" si="13"/>
+        <v>775.29210643778856</v>
       </c>
       <c r="V85" s="18">
-        <f>GammaG*(G85+I85)+GammaQ*O85</f>
-        <v>15.643464428976083</v>
+        <f t="shared" si="14"/>
+        <v>34.037214428976085</v>
       </c>
       <c r="W85" s="18">
-        <f>D85</f>
+        <f t="shared" si="28"/>
         <v>5</v>
       </c>
     </row>
@@ -4383,75 +4459,75 @@
         <v>12</v>
       </c>
       <c r="D86" s="18">
-        <f>D85+LL/20</f>
+        <f t="shared" si="29"/>
         <v>5.5</v>
       </c>
       <c r="F86" s="18">
-        <f>-qG_1*La^2/2*(LL-D86)/LL+qG_1*(D86*(LL-D86))/2</f>
+        <f t="shared" si="18"/>
         <v>68.143282864036962</v>
       </c>
       <c r="G86" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D86)</f>
+        <f t="shared" si="19"/>
         <v>-0.32919460320790783</v>
       </c>
       <c r="H86" s="17">
-        <f>-qG_2*La^2/2*(LL-D86)/LL+qG_2*(D86*(LL-D86))/2</f>
-        <v>25.875</v>
+        <f t="shared" si="20"/>
+        <v>51.75</v>
       </c>
       <c r="I86" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D86)</f>
-        <v>-0.125</v>
+        <f t="shared" si="21"/>
+        <v>-0.25</v>
       </c>
       <c r="J86" s="17">
-        <f>-qQ*La^2/2*(LL-D86)/LL</f>
-        <v>-30.375</v>
+        <f t="shared" si="22"/>
+        <v>-81</v>
       </c>
       <c r="K86" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L86" s="17">
-        <f>qQ*(D86*(LL-D86))/2</f>
-        <v>185.625</v>
+        <f t="shared" si="24"/>
+        <v>495</v>
       </c>
       <c r="M86" s="17">
-        <f>qQ/2*(LL-2*D86)</f>
-        <v>-7.5</v>
+        <f t="shared" si="25"/>
+        <v>-20</v>
       </c>
       <c r="N86" s="17">
-        <f t="shared" si="2"/>
-        <v>155.25</v>
+        <f t="shared" si="26"/>
+        <v>414</v>
       </c>
       <c r="O86" s="17">
-        <f t="shared" si="3"/>
-        <v>-0.75</v>
+        <f t="shared" si="27"/>
+        <v>-2</v>
       </c>
       <c r="Q86" s="18">
-        <f>GammaG*(F86+H86)+GammaQ*J86</f>
-        <v>81.362181866449902</v>
+        <f t="shared" si="9"/>
+        <v>40.355931866449907</v>
       </c>
       <c r="R86" s="18">
-        <f>GammaG*(G86+I86)+GammaQ*K86</f>
-        <v>9.5118372856693245</v>
+        <f t="shared" si="10"/>
+        <v>26.218087285669323</v>
       </c>
       <c r="S86" s="18">
-        <f>GammaG*(F86+H86)+GammaQ*L86</f>
-        <v>405.36218186644987</v>
+        <f t="shared" si="11"/>
+        <v>904.35593186644996</v>
       </c>
       <c r="T86" s="18">
-        <f>GammaG*(G86+I86)+GammaQ*M86</f>
-        <v>-11.863162714330675</v>
+        <f t="shared" si="12"/>
+        <v>-30.781912714330677</v>
       </c>
       <c r="U86" s="18">
-        <f>GammaG*(F86+H86)+GammaQ*N86</f>
-        <v>359.79968186644987</v>
+        <f t="shared" si="13"/>
+        <v>782.85593186644996</v>
       </c>
       <c r="V86" s="18">
-        <f>GammaG*(G86+I86)+GammaQ*O86</f>
-        <v>-1.7381627143306755</v>
+        <f t="shared" si="14"/>
+        <v>-3.7819127143306757</v>
       </c>
       <c r="W86" s="18">
-        <f>D86</f>
+        <f t="shared" si="28"/>
         <v>5.5</v>
       </c>
     </row>
@@ -4461,75 +4537,75 @@
         <v>13</v>
       </c>
       <c r="D87" s="18">
-        <f>D86+LL/20</f>
+        <f t="shared" si="29"/>
         <v>6</v>
       </c>
       <c r="F87" s="18">
-        <f>-qG_1*La^2/2*(LL-D87)/LL+qG_1*(D87*(LL-D87))/2</f>
+        <f t="shared" si="18"/>
         <v>67.155699054413247</v>
       </c>
       <c r="G87" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D87)</f>
+        <f t="shared" si="19"/>
         <v>-3.6211406352869884</v>
       </c>
       <c r="H87" s="17">
-        <f>-qG_2*La^2/2*(LL-D87)/LL+qG_2*(D87*(LL-D87))/2</f>
-        <v>25.5</v>
+        <f t="shared" si="20"/>
+        <v>51</v>
       </c>
       <c r="I87" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D87)</f>
-        <v>-1.375</v>
+        <f t="shared" si="21"/>
+        <v>-2.75</v>
       </c>
       <c r="J87" s="17">
-        <f>-qQ*La^2/2*(LL-D87)/LL</f>
-        <v>-27</v>
+        <f t="shared" si="22"/>
+        <v>-72</v>
       </c>
       <c r="K87" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L87" s="17">
-        <f>qQ*(D87*(LL-D87))/2</f>
-        <v>180</v>
+        <f t="shared" si="24"/>
+        <v>480</v>
       </c>
       <c r="M87" s="17">
-        <f>qQ/2*(LL-2*D87)</f>
-        <v>-15</v>
+        <f t="shared" si="25"/>
+        <v>-40</v>
       </c>
       <c r="N87" s="17">
-        <f t="shared" si="2"/>
-        <v>153</v>
+        <f t="shared" si="26"/>
+        <v>408</v>
       </c>
       <c r="O87" s="17">
-        <f t="shared" si="3"/>
-        <v>-8.25</v>
+        <f t="shared" si="27"/>
+        <v>-22</v>
       </c>
       <c r="Q87" s="18">
-        <f>GammaG*(F87+H87)+GammaQ*J87</f>
-        <v>84.585193723457891</v>
+        <f t="shared" si="9"/>
+        <v>51.510193723457888</v>
       </c>
       <c r="R87" s="18">
-        <f>GammaG*(G87+I87)+GammaQ*K87</f>
-        <v>3.3802101423625661</v>
+        <f t="shared" si="10"/>
+        <v>18.398960142362565</v>
       </c>
       <c r="S87" s="18">
-        <f>GammaG*(F87+H87)+GammaQ*L87</f>
-        <v>395.08519372345791</v>
+        <f t="shared" si="11"/>
+        <v>879.51019372345786</v>
       </c>
       <c r="T87" s="18">
-        <f>GammaG*(G87+I87)+GammaQ*M87</f>
-        <v>-29.244789857637436</v>
+        <f t="shared" si="12"/>
+        <v>-68.601039857637431</v>
       </c>
       <c r="U87" s="18">
-        <f>GammaG*(F87+H87)+GammaQ*N87</f>
-        <v>354.58519372345791</v>
+        <f t="shared" si="13"/>
+        <v>771.51019372345786</v>
       </c>
       <c r="V87" s="18">
-        <f>GammaG*(G87+I87)+GammaQ*O87</f>
-        <v>-19.119789857637436</v>
+        <f t="shared" si="14"/>
+        <v>-41.601039857637431</v>
       </c>
       <c r="W87" s="18">
-        <f>D87</f>
+        <f t="shared" si="28"/>
         <v>6</v>
       </c>
     </row>
@@ -4539,75 +4615,75 @@
         <v>14</v>
       </c>
       <c r="D88" s="18">
-        <f>D87+LL/20</f>
+        <f t="shared" si="29"/>
         <v>6.5</v>
       </c>
       <c r="F88" s="18">
-        <f>-qG_1*La^2/2*(LL-D88)/LL+qG_1*(D88*(LL-D88))/2</f>
+        <f t="shared" si="18"/>
         <v>64.522142228749985</v>
       </c>
       <c r="G88" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D88)</f>
+        <f t="shared" si="19"/>
         <v>-6.9130866673660698</v>
       </c>
       <c r="H88" s="17">
-        <f>-qG_2*La^2/2*(LL-D88)/LL+qG_2*(D88*(LL-D88))/2</f>
-        <v>24.5</v>
+        <f t="shared" si="20"/>
+        <v>49</v>
       </c>
       <c r="I88" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D88)</f>
-        <v>-2.625</v>
+        <f t="shared" si="21"/>
+        <v>-5.25</v>
       </c>
       <c r="J88" s="17">
-        <f>-qQ*La^2/2*(LL-D88)/LL</f>
-        <v>-23.625</v>
+        <f t="shared" si="22"/>
+        <v>-63</v>
       </c>
       <c r="K88" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L88" s="17">
-        <f>qQ*(D88*(LL-D88))/2</f>
-        <v>170.625</v>
+        <f t="shared" si="24"/>
+        <v>455</v>
       </c>
       <c r="M88" s="17">
-        <f>qQ/2*(LL-2*D88)</f>
-        <v>-22.5</v>
+        <f t="shared" si="25"/>
+        <v>-60</v>
       </c>
       <c r="N88" s="17">
-        <f t="shared" si="2"/>
-        <v>147</v>
+        <f t="shared" si="26"/>
+        <v>392</v>
       </c>
       <c r="O88" s="17">
-        <f t="shared" si="3"/>
-        <v>-15.75</v>
+        <f t="shared" si="27"/>
+        <v>-42</v>
       </c>
       <c r="Q88" s="18">
-        <f>GammaG*(F88+H88)+GammaQ*J88</f>
-        <v>84.742392008812487</v>
+        <f t="shared" si="9"/>
+        <v>58.754892008812476</v>
       </c>
       <c r="R88" s="18">
-        <f>GammaG*(G88+I88)+GammaQ*K88</f>
-        <v>-2.7514170009441958</v>
+        <f t="shared" si="10"/>
+        <v>10.579832999055803</v>
       </c>
       <c r="S88" s="18">
-        <f>GammaG*(F88+H88)+GammaQ*L88</f>
-        <v>376.11739200881249</v>
+        <f t="shared" si="11"/>
+        <v>835.75489200881248</v>
       </c>
       <c r="T88" s="18">
-        <f>GammaG*(G88+I88)+GammaQ*M88</f>
-        <v>-46.626417000944194</v>
+        <f t="shared" si="12"/>
+        <v>-106.42016700094419</v>
       </c>
       <c r="U88" s="18">
-        <f>GammaG*(F88+H88)+GammaQ*N88</f>
-        <v>340.67989200881249</v>
+        <f t="shared" si="13"/>
+        <v>741.25489200881248</v>
       </c>
       <c r="V88" s="18">
-        <f>GammaG*(G88+I88)+GammaQ*O88</f>
-        <v>-36.501417000944194</v>
+        <f t="shared" si="14"/>
+        <v>-79.42016700094419</v>
       </c>
       <c r="W88" s="18">
-        <f>D88</f>
+        <f t="shared" si="28"/>
         <v>6.5</v>
       </c>
     </row>
@@ -4617,75 +4693,75 @@
         <v>15</v>
       </c>
       <c r="D89" s="18">
-        <f>D88+LL/20</f>
+        <f t="shared" si="29"/>
         <v>7</v>
       </c>
       <c r="F89" s="18">
-        <f>-qG_1*La^2/2*(LL-D89)/LL+qG_1*(D89*(LL-D89))/2</f>
+        <f t="shared" si="18"/>
         <v>60.242612387047174</v>
       </c>
       <c r="G89" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D89)</f>
+        <f t="shared" si="19"/>
         <v>-10.20503269944515</v>
       </c>
       <c r="H89" s="17">
-        <f>-qG_2*La^2/2*(LL-D89)/LL+qG_2*(D89*(LL-D89))/2</f>
-        <v>22.875</v>
+        <f t="shared" si="20"/>
+        <v>45.75</v>
       </c>
       <c r="I89" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D89)</f>
-        <v>-3.875</v>
+        <f t="shared" si="21"/>
+        <v>-7.75</v>
       </c>
       <c r="J89" s="17">
-        <f>-qQ*La^2/2*(LL-D89)/LL</f>
-        <v>-20.25</v>
+        <f t="shared" si="22"/>
+        <v>-54</v>
       </c>
       <c r="K89" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L89" s="17">
-        <f>qQ*(D89*(LL-D89))/2</f>
-        <v>157.5</v>
+        <f t="shared" si="24"/>
+        <v>420</v>
       </c>
       <c r="M89" s="17">
-        <f>qQ/2*(LL-2*D89)</f>
-        <v>-30</v>
+        <f t="shared" si="25"/>
+        <v>-80</v>
       </c>
       <c r="N89" s="17">
-        <f t="shared" si="2"/>
-        <v>137.25</v>
+        <f t="shared" si="26"/>
+        <v>366</v>
       </c>
       <c r="O89" s="17">
-        <f t="shared" si="3"/>
-        <v>-23.25</v>
+        <f t="shared" si="27"/>
+        <v>-62</v>
       </c>
       <c r="Q89" s="18">
-        <f>GammaG*(F89+H89)+GammaQ*J89</f>
-        <v>81.83377672251369</v>
+        <f t="shared" si="9"/>
+        <v>62.090026722513699</v>
       </c>
       <c r="R89" s="18">
-        <f>GammaG*(G89+I89)+GammaQ*K89</f>
-        <v>-8.8830441442509525</v>
+        <f t="shared" si="10"/>
+        <v>2.7607058557490483</v>
       </c>
       <c r="S89" s="18">
-        <f>GammaG*(F89+H89)+GammaQ*L89</f>
-        <v>348.45877672251368</v>
+        <f t="shared" si="11"/>
+        <v>773.0900267225137</v>
       </c>
       <c r="T89" s="18">
-        <f>GammaG*(G89+I89)+GammaQ*M89</f>
-        <v>-64.00804414425096</v>
+        <f t="shared" si="12"/>
+        <v>-144.23929414425095</v>
       </c>
       <c r="U89" s="18">
-        <f>GammaG*(F89+H89)+GammaQ*N89</f>
-        <v>318.08377672251368</v>
+        <f t="shared" si="13"/>
+        <v>692.0900267225137</v>
       </c>
       <c r="V89" s="18">
-        <f>GammaG*(G89+I89)+GammaQ*O89</f>
-        <v>-53.883044144250952</v>
+        <f t="shared" si="14"/>
+        <v>-117.23929414425095</v>
       </c>
       <c r="W89" s="18">
-        <f>D89</f>
+        <f t="shared" si="28"/>
         <v>7</v>
       </c>
     </row>
@@ -4695,75 +4771,75 @@
         <v>16</v>
       </c>
       <c r="D90" s="18">
-        <f>D89+LL/20</f>
+        <f t="shared" si="29"/>
         <v>7.5</v>
       </c>
       <c r="F90" s="18">
-        <f>-qG_1*La^2/2*(LL-D90)/LL+qG_1*(D90*(LL-D90))/2</f>
+        <f t="shared" si="18"/>
         <v>54.31710952930483</v>
       </c>
       <c r="G90" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D90)</f>
+        <f t="shared" si="19"/>
         <v>-13.49697873152423</v>
       </c>
       <c r="H90" s="17">
-        <f>-qG_2*La^2/2*(LL-D90)/LL+qG_2*(D90*(LL-D90))/2</f>
-        <v>20.625</v>
+        <f t="shared" si="20"/>
+        <v>41.25</v>
       </c>
       <c r="I90" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D90)</f>
-        <v>-5.125</v>
+        <f t="shared" si="21"/>
+        <v>-10.25</v>
       </c>
       <c r="J90" s="17">
-        <f>-qQ*La^2/2*(LL-D90)/LL</f>
-        <v>-16.875</v>
+        <f t="shared" si="22"/>
+        <v>-45</v>
       </c>
       <c r="K90" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L90" s="17">
-        <f>qQ*(D90*(LL-D90))/2</f>
-        <v>140.625</v>
+        <f t="shared" si="24"/>
+        <v>375</v>
       </c>
       <c r="M90" s="17">
-        <f>qQ/2*(LL-2*D90)</f>
-        <v>-37.5</v>
+        <f t="shared" si="25"/>
+        <v>-100</v>
       </c>
       <c r="N90" s="17">
-        <f t="shared" si="2"/>
-        <v>123.75</v>
+        <f t="shared" si="26"/>
+        <v>330</v>
       </c>
       <c r="O90" s="17">
-        <f t="shared" si="3"/>
-        <v>-30.75</v>
+        <f t="shared" si="27"/>
+        <v>-82</v>
       </c>
       <c r="Q90" s="18">
-        <f>GammaG*(F90+H90)+GammaQ*J90</f>
-        <v>75.859347864561528</v>
+        <f t="shared" si="9"/>
+        <v>61.515597864561528</v>
       </c>
       <c r="R90" s="18">
-        <f>GammaG*(G90+I90)+GammaQ*K90</f>
-        <v>-15.014671287557711</v>
+        <f t="shared" si="10"/>
+        <v>-5.0584212875577137</v>
       </c>
       <c r="S90" s="18">
-        <f>GammaG*(F90+H90)+GammaQ*L90</f>
-        <v>312.10934786456153</v>
+        <f t="shared" si="11"/>
+        <v>691.51559786456153</v>
       </c>
       <c r="T90" s="18">
-        <f>GammaG*(G90+I90)+GammaQ*M90</f>
-        <v>-81.389671287557718</v>
+        <f t="shared" si="12"/>
+        <v>-182.05842128755771</v>
       </c>
       <c r="U90" s="18">
-        <f>GammaG*(F90+H90)+GammaQ*N90</f>
-        <v>286.79684786456153</v>
+        <f t="shared" si="13"/>
+        <v>624.01559786456153</v>
       </c>
       <c r="V90" s="18">
-        <f>GammaG*(G90+I90)+GammaQ*O90</f>
-        <v>-71.264671287557718</v>
+        <f t="shared" si="14"/>
+        <v>-155.05842128755771</v>
       </c>
       <c r="W90" s="18">
-        <f>D90</f>
+        <f t="shared" si="28"/>
         <v>7.5</v>
       </c>
     </row>
@@ -4773,75 +4849,75 @@
         <v>17</v>
       </c>
       <c r="D91" s="18">
-        <f>D90+LL/20</f>
+        <f t="shared" si="29"/>
         <v>8</v>
       </c>
       <c r="F91" s="18">
-        <f>-qG_1*La^2/2*(LL-D91)/LL+qG_1*(D91*(LL-D91))/2</f>
+        <f t="shared" si="18"/>
         <v>46.745633655522944</v>
       </c>
       <c r="G91" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D91)</f>
+        <f t="shared" si="19"/>
         <v>-16.788924763603312</v>
       </c>
       <c r="H91" s="17">
-        <f>-qG_2*La^2/2*(LL-D91)/LL+qG_2*(D91*(LL-D91))/2</f>
-        <v>17.75</v>
+        <f t="shared" si="20"/>
+        <v>35.5</v>
       </c>
       <c r="I91" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D91)</f>
-        <v>-6.375</v>
+        <f t="shared" si="21"/>
+        <v>-12.75</v>
       </c>
       <c r="J91" s="17">
-        <f>-qQ*La^2/2*(LL-D91)/LL</f>
-        <v>-13.5</v>
+        <f t="shared" si="22"/>
+        <v>-36</v>
       </c>
       <c r="K91" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L91" s="17">
-        <f>qQ*(D91*(LL-D91))/2</f>
-        <v>120</v>
+        <f t="shared" si="24"/>
+        <v>320</v>
       </c>
       <c r="M91" s="17">
-        <f>qQ/2*(LL-2*D91)</f>
-        <v>-45</v>
+        <f t="shared" si="25"/>
+        <v>-120</v>
       </c>
       <c r="N91" s="17">
-        <f t="shared" si="2"/>
-        <v>106.5</v>
+        <f t="shared" si="26"/>
+        <v>284</v>
       </c>
       <c r="O91" s="17">
-        <f t="shared" si="3"/>
-        <v>-38.25</v>
+        <f t="shared" si="27"/>
+        <v>-102</v>
       </c>
       <c r="Q91" s="18">
-        <f>GammaG*(F91+H91)+GammaQ*J91</f>
-        <v>66.819105434955972</v>
+        <f t="shared" si="9"/>
+        <v>57.031605434955978</v>
       </c>
       <c r="R91" s="18">
-        <f>GammaG*(G91+I91)+GammaQ*K91</f>
-        <v>-21.146298430864473</v>
+        <f t="shared" si="10"/>
+        <v>-12.877548430864472</v>
       </c>
       <c r="S91" s="18">
-        <f>GammaG*(F91+H91)+GammaQ*L91</f>
-        <v>267.06910543495599</v>
+        <f t="shared" si="11"/>
+        <v>591.03160543495596</v>
       </c>
       <c r="T91" s="18">
-        <f>GammaG*(G91+I91)+GammaQ*M91</f>
-        <v>-98.771298430864476</v>
+        <f t="shared" si="12"/>
+        <v>-219.87754843086446</v>
       </c>
       <c r="U91" s="18">
-        <f>GammaG*(F91+H91)+GammaQ*N91</f>
-        <v>246.81910543495599</v>
+        <f t="shared" si="13"/>
+        <v>537.03160543495596</v>
       </c>
       <c r="V91" s="18">
-        <f>GammaG*(G91+I91)+GammaQ*O91</f>
-        <v>-88.646298430864476</v>
+        <f t="shared" si="14"/>
+        <v>-192.87754843086446</v>
       </c>
       <c r="W91" s="18">
-        <f>D91</f>
+        <f t="shared" si="28"/>
         <v>8</v>
       </c>
     </row>
@@ -4851,75 +4927,75 @@
         <v>18</v>
       </c>
       <c r="D92" s="18">
-        <f>D91+LL/20</f>
+        <f t="shared" si="29"/>
         <v>8.5</v>
       </c>
       <c r="F92" s="18">
-        <f>-qG_1*La^2/2*(LL-D92)/LL+qG_1*(D92*(LL-D92))/2</f>
+        <f t="shared" si="18"/>
         <v>37.528184765701518</v>
       </c>
       <c r="G92" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D92)</f>
+        <f t="shared" si="19"/>
         <v>-20.08087079568239</v>
       </c>
       <c r="H92" s="17">
-        <f>-qG_2*La^2/2*(LL-D92)/LL+qG_2*(D92*(LL-D92))/2</f>
-        <v>14.25</v>
+        <f t="shared" si="20"/>
+        <v>28.5</v>
       </c>
       <c r="I92" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D92)</f>
-        <v>-7.625</v>
+        <f t="shared" si="21"/>
+        <v>-15.25</v>
       </c>
       <c r="J92" s="17">
-        <f>-qQ*La^2/2*(LL-D92)/LL</f>
-        <v>-10.125</v>
+        <f t="shared" si="22"/>
+        <v>-27</v>
       </c>
       <c r="K92" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L92" s="17">
-        <f>qQ*(D92*(LL-D92))/2</f>
-        <v>95.625</v>
+        <f t="shared" si="24"/>
+        <v>255</v>
       </c>
       <c r="M92" s="17">
-        <f>qQ/2*(LL-2*D92)</f>
-        <v>-52.5</v>
+        <f t="shared" si="25"/>
+        <v>-140</v>
       </c>
       <c r="N92" s="17">
-        <f t="shared" si="2"/>
-        <v>85.5</v>
+        <f t="shared" si="26"/>
+        <v>228</v>
       </c>
       <c r="O92" s="17">
-        <f t="shared" si="3"/>
-        <v>-45.75</v>
+        <f t="shared" si="27"/>
+        <v>-122</v>
       </c>
       <c r="Q92" s="18">
-        <f>GammaG*(F92+H92)+GammaQ*J92</f>
-        <v>54.713049433697051</v>
+        <f t="shared" si="9"/>
+        <v>48.638049433697063</v>
       </c>
       <c r="R92" s="18">
-        <f>GammaG*(G92+I92)+GammaQ*K92</f>
-        <v>-27.277925574171228</v>
+        <f t="shared" si="10"/>
+        <v>-20.696675574171223</v>
       </c>
       <c r="S92" s="18">
-        <f>GammaG*(F92+H92)+GammaQ*L92</f>
-        <v>213.33804943369705</v>
+        <f t="shared" si="11"/>
+        <v>471.63804943369706</v>
       </c>
       <c r="T92" s="18">
-        <f>GammaG*(G92+I92)+GammaQ*M92</f>
-        <v>-116.15292557417123</v>
+        <f t="shared" si="12"/>
+        <v>-257.69667557417119</v>
       </c>
       <c r="U92" s="18">
-        <f>GammaG*(F92+H92)+GammaQ*N92</f>
-        <v>198.15054943369705</v>
+        <f t="shared" si="13"/>
+        <v>431.13804943369706</v>
       </c>
       <c r="V92" s="18">
-        <f>GammaG*(G92+I92)+GammaQ*O92</f>
-        <v>-106.02792557417123</v>
+        <f t="shared" si="14"/>
+        <v>-230.69667557417122</v>
       </c>
       <c r="W92" s="18">
-        <f>D92</f>
+        <f t="shared" si="28"/>
         <v>8.5</v>
       </c>
     </row>
@@ -4929,75 +5005,75 @@
         <v>19</v>
       </c>
       <c r="D93" s="18">
-        <f>D92+LL/20</f>
+        <f t="shared" si="29"/>
         <v>9</v>
       </c>
       <c r="F93" s="18">
-        <f>-qG_1*La^2/2*(LL-D93)/LL+qG_1*(D93*(LL-D93))/2</f>
+        <f t="shared" si="18"/>
         <v>26.664762859840554</v>
       </c>
       <c r="G93" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D93)</f>
+        <f t="shared" si="19"/>
         <v>-23.372816827761472</v>
       </c>
       <c r="H93" s="17">
-        <f>-qG_2*La^2/2*(LL-D93)/LL+qG_2*(D93*(LL-D93))/2</f>
-        <v>10.125</v>
+        <f t="shared" si="20"/>
+        <v>20.25</v>
       </c>
       <c r="I93" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D93)</f>
-        <v>-8.875</v>
+        <f t="shared" si="21"/>
+        <v>-17.75</v>
       </c>
       <c r="J93" s="17">
-        <f>-qQ*La^2/2*(LL-D93)/LL</f>
-        <v>-6.75</v>
+        <f t="shared" si="22"/>
+        <v>-18</v>
       </c>
       <c r="K93" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L93" s="17">
-        <f>qQ*(D93*(LL-D93))/2</f>
-        <v>67.5</v>
+        <f t="shared" si="24"/>
+        <v>180</v>
       </c>
       <c r="M93" s="17">
-        <f>qQ/2*(LL-2*D93)</f>
-        <v>-60</v>
+        <f t="shared" si="25"/>
+        <v>-160</v>
       </c>
       <c r="N93" s="17">
-        <f t="shared" si="2"/>
-        <v>60.75</v>
+        <f t="shared" si="26"/>
+        <v>162</v>
       </c>
       <c r="O93" s="17">
-        <f t="shared" si="3"/>
-        <v>-53.25</v>
+        <f t="shared" si="27"/>
+        <v>-142</v>
       </c>
       <c r="Q93" s="18">
-        <f>GammaG*(F93+H93)+GammaQ*J93</f>
-        <v>39.541179860784744</v>
+        <f t="shared" si="9"/>
+        <v>36.334929860784747</v>
       </c>
       <c r="R93" s="18">
-        <f>GammaG*(G93+I93)+GammaQ*K93</f>
-        <v>-33.409552717477986</v>
+        <f t="shared" si="10"/>
+        <v>-28.515802717477989</v>
       </c>
       <c r="S93" s="18">
-        <f>GammaG*(F93+H93)+GammaQ*L93</f>
-        <v>150.91617986078475</v>
+        <f t="shared" si="11"/>
+        <v>333.33492986078477</v>
       </c>
       <c r="T93" s="18">
-        <f>GammaG*(G93+I93)+GammaQ*M93</f>
-        <v>-133.53455271747799</v>
+        <f t="shared" si="12"/>
+        <v>-295.51580271747798</v>
       </c>
       <c r="U93" s="18">
-        <f>GammaG*(F93+H93)+GammaQ*N93</f>
-        <v>140.79117986078475</v>
+        <f t="shared" si="13"/>
+        <v>306.33492986078477</v>
       </c>
       <c r="V93" s="18">
-        <f>GammaG*(G93+I93)+GammaQ*O93</f>
-        <v>-123.40955271747799</v>
+        <f t="shared" si="14"/>
+        <v>-268.51580271747798</v>
       </c>
       <c r="W93" s="18">
-        <f>D93</f>
+        <f t="shared" si="28"/>
         <v>9</v>
       </c>
     </row>
@@ -5007,75 +5083,75 @@
         <v>20</v>
       </c>
       <c r="D94" s="18">
-        <f>D93+LL/20</f>
+        <f t="shared" si="29"/>
         <v>9.5</v>
       </c>
       <c r="F94" s="18">
-        <f>-qG_1*La^2/2*(LL-D94)/LL+qG_1*(D94*(LL-D94))/2</f>
+        <f t="shared" si="18"/>
         <v>14.155367937940046</v>
       </c>
       <c r="G94" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D94)</f>
+        <f t="shared" si="19"/>
         <v>-26.664762859840554</v>
       </c>
       <c r="H94" s="17">
-        <f>-qG_2*La^2/2*(LL-D94)/LL+qG_2*(D94*(LL-D94))/2</f>
-        <v>5.375</v>
+        <f t="shared" si="20"/>
+        <v>10.75</v>
       </c>
       <c r="I94" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D94)</f>
-        <v>-10.125</v>
+        <f t="shared" si="21"/>
+        <v>-20.25</v>
       </c>
       <c r="J94" s="17">
-        <f>-qQ*La^2/2*(LL-D94)/LL</f>
-        <v>-3.375</v>
+        <f t="shared" si="22"/>
+        <v>-9</v>
       </c>
       <c r="K94" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L94" s="17">
-        <f>qQ*(D94*(LL-D94))/2</f>
-        <v>35.625</v>
+        <f t="shared" si="24"/>
+        <v>95</v>
       </c>
       <c r="M94" s="17">
-        <f>qQ/2*(LL-2*D94)</f>
-        <v>-67.5</v>
+        <f t="shared" si="25"/>
+        <v>-180</v>
       </c>
       <c r="N94" s="17">
-        <f t="shared" si="2"/>
-        <v>32.25</v>
+        <f t="shared" si="26"/>
+        <v>86</v>
       </c>
       <c r="O94" s="17">
-        <f t="shared" si="3"/>
-        <v>-60.75</v>
+        <f t="shared" si="27"/>
+        <v>-162</v>
       </c>
       <c r="Q94" s="18">
-        <f>GammaG*(F94+H94)+GammaQ*J94</f>
-        <v>21.303496716219062</v>
+        <f t="shared" si="9"/>
+        <v>20.122246716219067</v>
       </c>
       <c r="R94" s="18">
-        <f>GammaG*(G94+I94)+GammaQ*K94</f>
-        <v>-39.541179860784744</v>
+        <f t="shared" si="10"/>
+        <v>-36.334929860784747</v>
       </c>
       <c r="S94" s="18">
-        <f>GammaG*(F94+H94)+GammaQ*L94</f>
-        <v>79.803496716219058</v>
+        <f t="shared" si="11"/>
+        <v>176.12224671621908</v>
       </c>
       <c r="T94" s="18">
-        <f>GammaG*(G94+I94)+GammaQ*M94</f>
-        <v>-150.91617986078475</v>
+        <f t="shared" si="12"/>
+        <v>-333.33492986078477</v>
       </c>
       <c r="U94" s="18">
-        <f>GammaG*(F94+H94)+GammaQ*N94</f>
-        <v>74.740996716219058</v>
+        <f t="shared" si="13"/>
+        <v>162.62224671621908</v>
       </c>
       <c r="V94" s="18">
-        <f>GammaG*(G94+I94)+GammaQ*O94</f>
-        <v>-140.79117986078475</v>
+        <f t="shared" si="14"/>
+        <v>-306.33492986078477</v>
       </c>
       <c r="W94" s="18">
-        <f>D94</f>
+        <f t="shared" si="28"/>
         <v>9.5</v>
       </c>
     </row>
@@ -5085,75 +5161,75 @@
         <v>21</v>
       </c>
       <c r="D95" s="18">
-        <f>D94+LL/20</f>
+        <f t="shared" si="29"/>
         <v>10</v>
       </c>
       <c r="F95" s="18">
-        <f>-qG_1*La^2/2*(LL-D95)/LL+qG_1*(D95*(LL-D95))/2</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="G95" s="18">
-        <f>+qG_1*La^2/2/LL+qG_1/2*(LL-2*D95)</f>
+        <f t="shared" si="19"/>
         <v>-29.956708891919632</v>
       </c>
       <c r="H95" s="17">
-        <f>-qG_2*La^2/2*(LL-D95)/LL+qG_2*(D95*(LL-D95))/2</f>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="I95" s="17">
-        <f>+qG_2*La^2/2/LL+qG_2/2*(LL-2*D95)</f>
-        <v>-11.375</v>
+        <f t="shared" si="21"/>
+        <v>-22.75</v>
       </c>
       <c r="J95" s="17">
-        <f>-qQ*La^2/2*(LL-D95)/LL</f>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="K95" s="17">
-        <f>+qQ*La^2/2/LL</f>
-        <v>6.75</v>
+        <f t="shared" si="23"/>
+        <v>18</v>
       </c>
       <c r="L95" s="17">
-        <f>qQ*(D95*(LL-D95))/2</f>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="M95" s="17">
-        <f>qQ/2*(LL-2*D95)</f>
-        <v>-75</v>
+        <f t="shared" si="25"/>
+        <v>-200</v>
       </c>
       <c r="N95" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="O95" s="17">
-        <f t="shared" si="3"/>
-        <v>-68.25</v>
+        <f t="shared" si="27"/>
+        <v>-182</v>
       </c>
       <c r="Q95" s="18">
-        <f>GammaG*(F95+H95)+GammaQ*J95</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="R95" s="18">
-        <f>GammaG*(G95+I95)+GammaQ*K95</f>
-        <v>-45.67280700409151</v>
+        <f t="shared" si="10"/>
+        <v>-44.154057004091513</v>
       </c>
       <c r="S95" s="18">
-        <f>GammaG*(F95+H95)+GammaQ*L95</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="T95" s="18">
-        <f>GammaG*(G95+I95)+GammaQ*M95</f>
-        <v>-168.29780700409151</v>
+        <f t="shared" si="12"/>
+        <v>-371.1540570040915</v>
       </c>
       <c r="U95" s="18">
-        <f>GammaG*(F95+H95)+GammaQ*N95</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="V95" s="18">
-        <f>GammaG*(G95+I95)+GammaQ*O95</f>
-        <v>-158.17280700409151</v>
+        <f t="shared" si="14"/>
+        <v>-344.1540570040915</v>
       </c>
       <c r="W95" s="18">
-        <f>D95</f>
+        <f t="shared" si="28"/>
         <v>10</v>
       </c>
     </row>
@@ -5165,7 +5241,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="C4:J61"/>
+  <dimension ref="C4:J76"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="4" spans="3:6" x14ac:dyDescent="0.25">
@@ -5503,7 +5579,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="50" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C50" s="2" t="s">
         <v>167</v>
       </c>
@@ -5517,47 +5593,49 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C51" s="2" t="s">
         <v>168</v>
       </c>
       <c r="D51" s="18">
         <f>MAX(Feuil1!Q75:Q95)</f>
-        <v>84.742392008812487</v>
+        <v>62.090026722513699</v>
       </c>
       <c r="E51" s="18">
         <f>MAX(Feuil1!S75:S95)</f>
-        <v>406.94835643778856</v>
+        <v>910.29210643778856</v>
       </c>
       <c r="F51" s="18">
         <f>MAX(Feuil1!U75:U95)</f>
-        <v>359.79968186644987</v>
-      </c>
-    </row>
-    <row r="52" spans="3:6" x14ac:dyDescent="0.25">
+        <v>782.85593186644996</v>
+      </c>
+    </row>
+    <row r="52" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C52" s="2" t="s">
         <v>169</v>
       </c>
       <c r="D52" s="3">
-        <f>VLOOKUP(Connexion!D51,Feuil1!Q75:W95,7,FALSE)</f>
-        <v>6.5</v>
+        <v>7.1</v>
       </c>
       <c r="E52" s="3">
-        <f>VLOOKUP(Connexion!E51,Feuil1!S75:W95,5,FALSE)</f>
         <v>5</v>
       </c>
       <c r="F52" s="3">
-        <f>VLOOKUP(Connexion!F51,Feuil1!U75:W95,3,FALSE)</f>
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="53" spans="3:6" x14ac:dyDescent="0.25">
+        <v>5.3</v>
+      </c>
+      <c r="H52" s="63">
+        <v>7</v>
+      </c>
+      <c r="I52" s="63"/>
+      <c r="J52" s="63"/>
+    </row>
+    <row r="53" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C53" s="2" t="s">
         <v>170</v>
       </c>
       <c r="D53" s="18">
         <f>($D$36-$D$43)*$G$36+(D52-$D$36-$D$44)*$G$37</f>
-        <v>1854.3489689609494</v>
+        <v>2092.7644356040828</v>
       </c>
       <c r="E53" s="18">
         <f t="shared" ref="E53:F53" si="0">($D$36-$D$43)*$G$36+(E52-$D$36-$D$44)*$G$37</f>
@@ -5565,16 +5643,16 @@
       </c>
       <c r="F53" s="18">
         <f t="shared" si="0"/>
-        <v>1456.9898578890602</v>
-      </c>
-    </row>
-    <row r="54" spans="3:6" x14ac:dyDescent="0.25">
+        <v>1377.5180356746823</v>
+      </c>
+    </row>
+    <row r="54" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C54" s="2" t="s">
         <v>171</v>
       </c>
       <c r="D54" s="18">
         <f>(LL-D52)*$G$37</f>
-        <v>1390.7568887516113</v>
+        <v>1152.3414221084781</v>
       </c>
       <c r="E54" s="18">
         <f>(LL-E52)*$G$37</f>
@@ -5582,16 +5660,16 @@
       </c>
       <c r="F54" s="18">
         <f>(LL-F52)*$G$37</f>
-        <v>1788.1159998235003</v>
-      </c>
-    </row>
-    <row r="55" spans="3:6" x14ac:dyDescent="0.25">
+        <v>1867.5878220378781</v>
+      </c>
+    </row>
+    <row r="55" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C55" s="2" t="s">
         <v>172</v>
       </c>
       <c r="D55" s="18">
         <f>MIN(D53:D54)</f>
-        <v>1390.7568887516113</v>
+        <v>1152.3414221084781</v>
       </c>
       <c r="E55" s="18">
         <f t="shared" ref="E55:F55" si="1">MIN(E53:E54)</f>
@@ -5599,16 +5677,16 @@
       </c>
       <c r="F55" s="18">
         <f t="shared" si="1"/>
-        <v>1456.9898578890602</v>
-      </c>
-    </row>
-    <row r="56" spans="3:6" x14ac:dyDescent="0.25">
+        <v>1377.5180356746823</v>
+      </c>
+    </row>
+    <row r="56" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C56" s="2"/>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C57" s="2" t="s">
         <v>47</v>
       </c>
@@ -5621,7 +5699,7 @@
       </c>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C58" s="2" t="s">
         <v>43</v>
       </c>
@@ -5634,13 +5712,13 @@
       </c>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C59" s="2" t="s">
         <v>133</v>
       </c>
       <c r="D59" s="62">
         <f>D55/MIN($D$57:$D$58)</f>
-        <v>0.53865887356756348</v>
+        <v>0.44631735238455267</v>
       </c>
       <c r="E59" s="62">
         <f t="shared" ref="E59:F59" si="2">E55/MIN($D$57:$D$58)</f>
@@ -5648,19 +5726,155 @@
       </c>
       <c r="F59" s="62">
         <f t="shared" si="2"/>
-        <v>0.56431179453251967</v>
-      </c>
-    </row>
-    <row r="60" spans="3:6" x14ac:dyDescent="0.25">
+        <v>0.53353128747151601</v>
+      </c>
+    </row>
+    <row r="60" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C60" s="2"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C61" s="15" t="s">
         <v>173</v>
       </c>
+    </row>
+    <row r="64" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C64" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D64" s="7">
+        <f>Nc</f>
+        <v>3034.4999999999995</v>
+      </c>
+      <c r="E64" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="65" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C65" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D65" s="11">
+        <f>Na</f>
+        <v>2581.8880129841023</v>
+      </c>
+      <c r="E65" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="66" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C66" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D66" s="7">
+        <f>Nf</f>
+        <v>766.44500000000005</v>
+      </c>
+      <c r="E66" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="67" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C67" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D67" s="14">
+        <f>Nc*D59</f>
+        <v>1354.3500058109248</v>
+      </c>
+      <c r="E67" s="14">
+        <f>Nc*E59</f>
+        <v>1478.8955188173918</v>
+      </c>
+      <c r="F67" s="14">
+        <f>Nc*F59</f>
+        <v>1619.0006918323152</v>
+      </c>
+    </row>
+    <row r="69" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C69" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="D69" s="6" t="str">
+        <f>IF(Na-2*Nf&lt;=D67,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="E69" s="6" t="str">
+        <f>IF(Na-2*Nf&lt;=E67,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="F69" s="6" t="str">
+        <f>IF(Na-2*Nf&lt;=F67,oui,non)</f>
+        <v>oui</v>
+      </c>
+    </row>
+    <row r="71" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C71" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D71" s="24">
+        <f>(Na-D67)/2/Nf</f>
+        <v>0.80079980114240246</v>
+      </c>
+      <c r="E71" s="24">
+        <f>(Na-E67)/2/Nf</f>
+        <v>0.71955097506455801</v>
+      </c>
+      <c r="F71" s="24">
+        <f>(Na-F67)/2/Nf</f>
+        <v>0.62815160980356521</v>
+      </c>
+    </row>
+    <row r="72" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C72" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D72" s="14">
+        <f>D71*tf</f>
+        <v>10.17015747450851</v>
+      </c>
+      <c r="E72" s="14">
+        <f>E71*tf</f>
+        <v>9.1382973833198857</v>
+      </c>
+      <c r="F72" s="14">
+        <f>F71*tf</f>
+        <v>7.9775254445052779</v>
+      </c>
+    </row>
+    <row r="73" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C73" s="2"/>
+      <c r="D73" s="3"/>
+      <c r="E73" s="3"/>
+      <c r="F73" s="3"/>
+    </row>
+    <row r="74" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C74" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D74" s="65">
+        <f>(D67*(td-tc/2*D59)+Na*Ht/2-(Na-D59*Nc)*D72/2)/1000</f>
+        <v>612.80229895647165</v>
+      </c>
+      <c r="E74" s="65">
+        <f>(E67*(td-tc/2*E59)+Na*Ht/2-(Na-E59*Nc)*E72/2)/1000</f>
+        <v>626.00933229871885</v>
+      </c>
+      <c r="F74" s="65">
+        <f>(F67*(td-tc/2*F59)+Na*Ht/2-(Na-F59*Nc)*F72/2)/1000</f>
+        <v>640.27285237589899</v>
+      </c>
+    </row>
+    <row r="75" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C75" s="2"/>
+      <c r="D75" s="3"/>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+    </row>
+    <row r="76" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C76" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Test TU MV C05 en cours
</commit_message>
<xml_diff>
--- a/Manuel Validation/CAS C05/TEST C05.xlsx
+++ b/Manuel Validation/CAS C05/TEST C05.xlsx
@@ -21,17 +21,17 @@
     <definedName name="Av">Feuil1!$E$20</definedName>
     <definedName name="Avmin">Feuil1!$J$36</definedName>
     <definedName name="b">Feuil1!$E$12</definedName>
-    <definedName name="bb">Feuil1!$E$26</definedName>
+    <definedName name="bb">Feuil1!$E$27</definedName>
     <definedName name="beff_1">Feuil1!$O$4</definedName>
     <definedName name="beff_a">Feuil1!$O$5</definedName>
-    <definedName name="bm">Feuil1!$E$31</definedName>
-    <definedName name="bt">Feuil1!$E$27</definedName>
-    <definedName name="c_z">Feuil1!$E$40</definedName>
+    <definedName name="bm">Feuil1!$E$32</definedName>
+    <definedName name="bt">Feuil1!$E$28</definedName>
+    <definedName name="c_z">Feuil1!$E$41</definedName>
     <definedName name="d">Feuil1!$E$6</definedName>
     <definedName name="dsc">Connexion!$D$4</definedName>
     <definedName name="dw">Feuil1!$E$19</definedName>
-    <definedName name="e_s">Feuil1!$E$39</definedName>
-    <definedName name="ebac">Feuil1!$E$25</definedName>
+    <definedName name="e_s">Feuil1!$E$40</definedName>
+    <definedName name="ebac">Feuil1!$E$26</definedName>
     <definedName name="Ecm">Feuil1!$J$9</definedName>
     <definedName name="Eta">Feuil1!$J$35</definedName>
     <definedName name="Ey">Feuil1!$J$6</definedName>
@@ -40,7 +40,7 @@
     <definedName name="Fsk">Feuil1!$J$8</definedName>
     <definedName name="Fusc">Connexion!$D$6</definedName>
     <definedName name="Fy">Feuil1!$J$4</definedName>
-    <definedName name="fybac">Feuil1!$E$29</definedName>
+    <definedName name="fybac">Feuil1!$E$30</definedName>
     <definedName name="g">Feuil1!$J$28</definedName>
     <definedName name="GammaC">Feuil1!$J$16</definedName>
     <definedName name="GammaG">Feuil1!$J$20</definedName>
@@ -49,18 +49,20 @@
     <definedName name="GammaQ">Feuil1!$J$21</definedName>
     <definedName name="GammaS">Feuil1!$J$17</definedName>
     <definedName name="GammaV">Feuil1!$J$18</definedName>
-    <definedName name="hbac">Feuil1!$E$24</definedName>
+    <definedName name="hbac">Feuil1!$E$25</definedName>
     <definedName name="hsc">Connexion!$D$5</definedName>
     <definedName name="Ht">Feuil1!$E$11</definedName>
     <definedName name="hw">Feuil1!$E$18</definedName>
     <definedName name="kC">Feuil1!$O$53</definedName>
     <definedName name="La">Feuil1!$E$5</definedName>
+    <definedName name="Le">Connexion!$H$60</definedName>
     <definedName name="Le_1">Feuil1!$O$7</definedName>
     <definedName name="Le_a">Feuil1!$O$8</definedName>
     <definedName name="LL">Feuil1!$E$4</definedName>
+    <definedName name="MplaRd">Connexion!$M$78</definedName>
     <definedName name="MplRd_1">Feuil1!$O$19</definedName>
     <definedName name="MplRd_app">Feuil1!$O$37</definedName>
-    <definedName name="mubac">Feuil1!$E$30</definedName>
+    <definedName name="mubac">Feuil1!$E$31</definedName>
     <definedName name="Na">Feuil1!$O$15</definedName>
     <definedName name="Nc">Feuil1!$O$14</definedName>
     <definedName name="Nf">Feuil1!$O$29</definedName>
@@ -72,7 +74,7 @@
     <definedName name="oui">Feuil1!$T$2</definedName>
     <definedName name="p_1">Feuil1!$O$40</definedName>
     <definedName name="p_w">Feuil1!$R$40</definedName>
-    <definedName name="PhiS">Feuil1!$E$38</definedName>
+    <definedName name="PhiS">Feuil1!$E$39</definedName>
     <definedName name="PRd_dp">Connexion!$D$12</definedName>
     <definedName name="PRda">Connexion!$D$10</definedName>
     <definedName name="PRdc">Connexion!$D$11</definedName>
@@ -82,12 +84,13 @@
     <definedName name="RhoA">Feuil1!$J$26</definedName>
     <definedName name="RhoC">Feuil1!$J$27</definedName>
     <definedName name="rr">Feuil1!$E$15</definedName>
-    <definedName name="tbac">Feuil1!$E$28</definedName>
-    <definedName name="tc">Feuil1!$E$36</definedName>
-    <definedName name="td">Feuil1!$E$35</definedName>
+    <definedName name="tbac">Feuil1!$E$29</definedName>
+    <definedName name="tc">Feuil1!$E$37</definedName>
+    <definedName name="td">Feuil1!$E$36</definedName>
     <definedName name="tf">Feuil1!$E$13</definedName>
     <definedName name="tw">Feuil1!$E$14</definedName>
     <definedName name="VplRd">Feuil1!$J$37</definedName>
+    <definedName name="Wpl">Feuil1!$E$21</definedName>
     <definedName name="zn">Feuil1!$O$17</definedName>
     <definedName name="zR">Feuil1!$O$52</definedName>
   </definedNames>
@@ -101,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="205">
   <si>
     <t>Portee principale</t>
   </si>
@@ -635,6 +638,87 @@
   </si>
   <si>
     <t>Avec prise en compte degre connexion</t>
+  </si>
+  <si>
+    <t>Mmax</t>
+  </si>
+  <si>
+    <t>Mmin</t>
+  </si>
+  <si>
+    <t>Vmax</t>
+  </si>
+  <si>
+    <t>Vmin</t>
+  </si>
+  <si>
+    <t>MedMax</t>
+  </si>
+  <si>
+    <t>MedMin</t>
+  </si>
+  <si>
+    <t>VedMax</t>
+  </si>
+  <si>
+    <t>VEdMin</t>
+  </si>
+  <si>
+    <t>EtaMin</t>
+  </si>
+  <si>
+    <t>Le</t>
+  </si>
+  <si>
+    <t>Résistance en flexion dans la travée principale</t>
+  </si>
+  <si>
+    <t>Moment positif</t>
+  </si>
+  <si>
+    <t>Prise en compte du degré de connexion effectif</t>
+  </si>
+  <si>
+    <t>zone</t>
+  </si>
+  <si>
+    <t>nPRd</t>
+  </si>
+  <si>
+    <t>ANP</t>
+  </si>
+  <si>
+    <t>Sem sup ?</t>
+  </si>
+  <si>
+    <t>congés ?</t>
+  </si>
+  <si>
+    <t>âme</t>
+  </si>
+  <si>
+    <t>Wpl</t>
+  </si>
+  <si>
+    <t>cm3</t>
+  </si>
+  <si>
+    <t>MplaRd</t>
+  </si>
+  <si>
+    <t>knM</t>
+  </si>
+  <si>
+    <t>Vérification</t>
+  </si>
+  <si>
+    <t>ELU01</t>
+  </si>
+  <si>
+    <t>ELU02</t>
+  </si>
+  <si>
+    <t>ELU03</t>
   </si>
 </sst>
 </file>
@@ -699,7 +783,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -772,8 +856,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -877,11 +979,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1047,6 +1167,60 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1062,6 +1236,1119 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="0"/>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Connexion!$F$111:$F$131</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>9.5</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>10</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Connexion!$H$111:$H$131</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.0924322715763612E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4.2139778043996684E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>6.5037999143746292E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8.1348128469880418E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>9.5708419354080018E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.10468774189632066</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.10810484895720011</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.11801875693717821</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.10424054280510127</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>8.2430316448273755E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4.9581000014427924E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-BBF6-4FD4-A32B-5377AA8F4B77}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="1"/>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Connexion!$F$111:$F$131</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>9.5</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>10</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Connexion!$J$111:$J$131</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.31178680245873286</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.76583564231427137</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.1676112964404883</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.4539371349002377</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.5682385622298081</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.6539071204016087</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.7217044403359252</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.5648287898116933</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.5513590131514212</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.5166592555208547</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.4574685207869096</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.3889776577757806</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.3613977823260401</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.3034790521486443</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.2152395791273385</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.2230554418386614</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.010809579186094</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.75621182858928992</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.43396332626910178</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-BBF6-4FD4-A32B-5377AA8F4B77}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="2"/>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Connexion!$F$111:$F$131</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>9.5</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>10</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Connexion!$L$111:$L$131</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.4091734312778549E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.53318649443907851</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.8816964994263139</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.0843835832795394</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.2342921779589113</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.3507946835153533</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.2719101536274235</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.2946198980788115</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.2917325555667576</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.2616579786808397</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.2184172843880545</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.2074625895321531</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.1669078902211643</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.0966180008948236</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.1113101590958148</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.92401041612833945</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.69495896384919753</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.40069947111244736</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-BBF6-4FD4-A32B-5377AA8F4B77}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="929533439"/>
+        <c:axId val="929533855"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="929533439"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="929533855"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="929533855"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="929533439"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="0"/>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Connexion!$C$84:$C$104</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>9.5</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>10</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Connexion!$G$84:$G$104</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>361.745</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>361.745</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>361.745</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>361.745</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>377.46358194417815</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>418.51382916287656</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>450.41294025369427</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>473.16091521663122</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>553.05460284230173</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>578.40816331396184</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>600.19553048860269</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>620.49774589860397</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>633.20686895126073</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>613.89470649854354</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>593.09739228118656</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>569.03643507162406</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>483.24187540217946</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>466.59436074345575</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>440.79570995685128</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>405.84592304236605</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>361.745</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-20C7-419E-931F-E0C071ED7371}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="929533439"/>
+        <c:axId val="929533855"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="929533439"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="929533855"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="929533855"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="929533439"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>157162</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>118</xdr:row>
+      <xdr:rowOff>42862</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Graphique 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>371475</xdr:colOff>
+      <xdr:row>104</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>371475</xdr:colOff>
+      <xdr:row>118</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Graphique 2"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1327,7 +2614,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:AB95"/>
+  <dimension ref="B2:AB107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="3:24" x14ac:dyDescent="0.25">
@@ -1809,6 +3096,15 @@
       </c>
     </row>
     <row r="21" spans="3:28" x14ac:dyDescent="0.25">
+      <c r="D21" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="E21" s="4">
+        <v>1019</v>
+      </c>
+      <c r="F21" t="s">
+        <v>198</v>
+      </c>
       <c r="I21" s="2" t="s">
         <v>28</v>
       </c>
@@ -1818,12 +3114,6 @@
       <c r="N21" s="2"/>
     </row>
     <row r="22" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C22" s="5"/>
-      <c r="D22" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
       <c r="I22" s="2"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9" t="s">
@@ -1842,6 +3132,12 @@
       </c>
     </row>
     <row r="23" spans="3:28" x14ac:dyDescent="0.25">
+      <c r="C23" s="5"/>
+      <c r="D23" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
       <c r="I23" s="2"/>
       <c r="V23" s="2" t="s">
         <v>124</v>
@@ -1853,15 +3149,6 @@
       </c>
     </row>
     <row r="24" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="D24" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E24" s="4">
-        <v>58</v>
-      </c>
-      <c r="F24" t="s">
-        <v>2</v>
-      </c>
       <c r="H24" s="5"/>
       <c r="I24" s="5" t="s">
         <v>100</v>
@@ -1892,10 +3179,10 @@
     </row>
     <row r="25" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D25" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E25" s="4">
-        <v>207</v>
+        <v>58</v>
       </c>
       <c r="F25" t="s">
         <v>2</v>
@@ -1914,10 +3201,10 @@
     </row>
     <row r="26" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D26" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E26" s="4">
-        <v>62</v>
+        <v>207</v>
       </c>
       <c r="F26" t="s">
         <v>2</v>
@@ -1947,10 +3234,10 @@
     </row>
     <row r="27" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D27" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E27" s="4">
-        <v>101</v>
+        <v>62</v>
       </c>
       <c r="F27" t="s">
         <v>2</v>
@@ -1989,10 +3276,10 @@
     </row>
     <row r="28" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D28" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E28" s="4">
-        <v>0.75</v>
+        <v>101</v>
       </c>
       <c r="F28" t="s">
         <v>2</v>
@@ -2024,13 +3311,13 @@
     </row>
     <row r="29" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D29" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E29" s="4">
-        <v>355</v>
+        <v>0.75</v>
       </c>
       <c r="F29" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="I29" s="2"/>
       <c r="N29" s="15" t="s">
@@ -2058,13 +3345,13 @@
     </row>
     <row r="30" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D30" s="2" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="E30" s="4">
-        <v>8.5299999999999994</v>
+        <v>355</v>
       </c>
       <c r="F30" t="s">
-        <v>97</v>
+        <v>17</v>
       </c>
       <c r="I30" s="2"/>
       <c r="N30" s="15" t="s">
@@ -2080,14 +3367,13 @@
     </row>
     <row r="31" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D31" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="E31" s="4">
-        <f>(bb+bt)/2</f>
-        <v>81.5</v>
+        <v>8.5299999999999994</v>
       </c>
       <c r="F31" t="s">
-        <v>2</v>
+        <v>97</v>
       </c>
       <c r="I31" s="2"/>
       <c r="N31" s="15" t="s">
@@ -2102,6 +3388,16 @@
       </c>
     </row>
     <row r="32" spans="3:28" x14ac:dyDescent="0.25">
+      <c r="D32" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E32" s="4">
+        <f>(bb+bt)/2</f>
+        <v>81.5</v>
+      </c>
+      <c r="F32" t="s">
+        <v>2</v>
+      </c>
       <c r="I32" s="2"/>
       <c r="U32" s="52" t="s">
         <v>135</v>
@@ -2109,12 +3405,6 @@
       <c r="V32" s="51"/>
     </row>
     <row r="33" spans="3:25" x14ac:dyDescent="0.25">
-      <c r="C33" s="5"/>
-      <c r="D33" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
       <c r="H33" s="9"/>
       <c r="I33" s="9" t="s">
         <v>131</v>
@@ -2139,6 +3429,12 @@
       </c>
     </row>
     <row r="34" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="C34" s="5"/>
+      <c r="D34" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
       <c r="N34" s="2" t="s">
         <v>68</v>
       </c>
@@ -2167,15 +3463,6 @@
       </c>
     </row>
     <row r="35" spans="3:25" x14ac:dyDescent="0.25">
-      <c r="D35" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E35" s="4">
-        <v>130</v>
-      </c>
-      <c r="F35" t="s">
-        <v>2</v>
-      </c>
       <c r="I35" s="2" t="s">
         <v>133</v>
       </c>
@@ -2207,11 +3494,10 @@
     </row>
     <row r="36" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D36" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E36" s="7">
-        <f>td-hbac</f>
-        <v>72</v>
+        <v>35</v>
+      </c>
+      <c r="E36" s="4">
+        <v>130</v>
       </c>
       <c r="F36" t="s">
         <v>2</v>
@@ -2240,7 +3526,14 @@
     </row>
     <row r="37" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D37" s="2" t="s">
-        <v>58</v>
+        <v>36</v>
+      </c>
+      <c r="E37" s="7">
+        <f>td-hbac</f>
+        <v>72</v>
+      </c>
+      <c r="F37" t="s">
+        <v>2</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>132</v>
@@ -2277,13 +3570,7 @@
     </row>
     <row r="38" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D38" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E38" s="4">
-        <v>16</v>
-      </c>
-      <c r="F38" t="s">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="V38" t="s">
         <v>108</v>
@@ -2302,11 +3589,11 @@
       </c>
     </row>
     <row r="39" spans="3:25" x14ac:dyDescent="0.25">
-      <c r="D39" s="15" t="s">
-        <v>25</v>
+      <c r="D39" s="2" t="s">
+        <v>56</v>
       </c>
       <c r="E39" s="4">
-        <v>180</v>
+        <v>16</v>
       </c>
       <c r="F39" t="s">
         <v>2</v>
@@ -2335,10 +3622,10 @@
     </row>
     <row r="40" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D40" s="15" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="E40" s="4">
-        <v>20</v>
+        <v>180</v>
       </c>
       <c r="F40" t="s">
         <v>2</v>
@@ -2359,6 +3646,15 @@
       </c>
     </row>
     <row r="41" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="D41" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E41" s="4">
+        <v>20</v>
+      </c>
+      <c r="F41" t="s">
+        <v>2</v>
+      </c>
       <c r="V41" t="s">
         <v>128</v>
       </c>
@@ -5231,6 +6527,206 @@
       <c r="W95" s="18">
         <f t="shared" si="28"/>
         <v>10</v>
+      </c>
+    </row>
+    <row r="98" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E98" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F98" s="25">
+        <f>MAX(F$64:F$95)</f>
+        <v>68.143282864036962</v>
+      </c>
+      <c r="H98" s="25">
+        <f>MAX(H$64:H$95)</f>
+        <v>51.75</v>
+      </c>
+      <c r="J98" s="25">
+        <f>MAX(J$64:J$95)</f>
+        <v>0</v>
+      </c>
+      <c r="L98" s="25">
+        <f>MAX(L$64:L$95)</f>
+        <v>500</v>
+      </c>
+      <c r="N98" s="25">
+        <f>MAX(N$64:N$95)</f>
+        <v>414</v>
+      </c>
+      <c r="Q98" s="25">
+        <f>MAX(Q$64:Q$95)</f>
+        <v>62.090026722513699</v>
+      </c>
+      <c r="S98" s="25">
+        <f>MAX(S$64:S$95)</f>
+        <v>910.29210643778856</v>
+      </c>
+      <c r="U98" s="25">
+        <f>MAX(U$64:U$95)</f>
+        <v>782.85593186644996</v>
+      </c>
+    </row>
+    <row r="99" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E99" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F99" s="25">
+        <f>MIN(F$64:F$95)</f>
+        <v>-29.62751428871173</v>
+      </c>
+      <c r="H99" s="25">
+        <f>MIN(H$64:H$95)</f>
+        <v>-22.5</v>
+      </c>
+      <c r="J99" s="25">
+        <f>MIN(J$64:J$95)</f>
+        <v>-180</v>
+      </c>
+      <c r="L99" s="25">
+        <f>MIN(L$64:L$95)</f>
+        <v>0</v>
+      </c>
+      <c r="N99" s="25">
+        <f>MIN(N$64:N$95)</f>
+        <v>-180</v>
+      </c>
+      <c r="Q99" s="25">
+        <f>MIN(Q$64:Q$95)</f>
+        <v>-340.37214428976085</v>
+      </c>
+      <c r="S99" s="25">
+        <f>MIN(S$64:S$95)</f>
+        <v>-70.37214428976084</v>
+      </c>
+      <c r="U99" s="25">
+        <f>MIN(U$64:U$95)</f>
+        <v>-340.37214428976085</v>
+      </c>
+    </row>
+    <row r="100" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E100" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="F100" s="3"/>
+      <c r="G100" s="25">
+        <f>MAX(G$64:G$95)</f>
+        <v>35.882211749661977</v>
+      </c>
+      <c r="H100" s="3"/>
+      <c r="I100" s="25">
+        <f>MAX(I$64:I$95)</f>
+        <v>27.25</v>
+      </c>
+      <c r="J100" s="3"/>
+      <c r="K100" s="25">
+        <f>MAX(K$64:K$95)</f>
+        <v>18</v>
+      </c>
+      <c r="L100" s="3"/>
+      <c r="M100" s="25">
+        <f>MAX(M$64:M$95)</f>
+        <v>200</v>
+      </c>
+      <c r="N100" s="3"/>
+      <c r="O100" s="25">
+        <f>MAX(O$64:O$95)</f>
+        <v>218</v>
+      </c>
+      <c r="Q100" s="3"/>
+      <c r="R100" s="25">
+        <f>MAX(R$64:R$95)</f>
+        <v>112.22848586204367</v>
+      </c>
+      <c r="S100" s="3"/>
+      <c r="T100" s="25">
+        <f>MAX(T$64:T$95)</f>
+        <v>385.22848586204367</v>
+      </c>
+      <c r="U100" s="3"/>
+      <c r="V100" s="25">
+        <f>MAX(V$64:V$95)</f>
+        <v>412.22848586204367</v>
+      </c>
+    </row>
+    <row r="101" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E101" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="F101" s="3"/>
+      <c r="G101" s="25">
+        <f>MIN(G$64:G$95)</f>
+        <v>-29.956708891919632</v>
+      </c>
+      <c r="H101" s="3"/>
+      <c r="I101" s="25">
+        <f>MIN(I$64:I$95)</f>
+        <v>-22.75</v>
+      </c>
+      <c r="J101" s="3"/>
+      <c r="K101" s="25">
+        <f>MIN(K$64:K$95)</f>
+        <v>-120</v>
+      </c>
+      <c r="L101" s="3"/>
+      <c r="M101" s="25">
+        <f>MIN(M$64:M$95)</f>
+        <v>-200</v>
+      </c>
+      <c r="N101" s="3"/>
+      <c r="O101" s="25">
+        <f>MIN(O$64:O$95)</f>
+        <v>-182</v>
+      </c>
+      <c r="Q101" s="3"/>
+      <c r="R101" s="25">
+        <f>MIN(R$64:R$95)</f>
+        <v>-226.91476285984055</v>
+      </c>
+      <c r="S101" s="3"/>
+      <c r="T101" s="25">
+        <f>MIN(T$64:T$95)</f>
+        <v>-371.1540570040915</v>
+      </c>
+      <c r="U101" s="3"/>
+      <c r="V101" s="25">
+        <f>MIN(V$64:V$95)</f>
+        <v>-344.1540570040915</v>
+      </c>
+    </row>
+    <row r="104" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="P104" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="Q104" s="25">
+        <f>MAX(Q98:U98)</f>
+        <v>910.29210643778856</v>
+      </c>
+    </row>
+    <row r="105" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="P105" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q105" s="25">
+        <f>MIN(Q99:U99)</f>
+        <v>-340.37214428976085</v>
+      </c>
+    </row>
+    <row r="106" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="P106" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q106" s="25">
+        <f>MAX(R100:V100)</f>
+        <v>412.22848586204367</v>
+      </c>
+    </row>
+    <row r="107" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="P107" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="Q107" s="25">
+        <f>MIN(R101:V101)</f>
+        <v>-371.1540570040915</v>
       </c>
     </row>
   </sheetData>
@@ -5241,7 +6737,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="C4:J76"/>
+  <dimension ref="B4:T134"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="4" spans="3:6" x14ac:dyDescent="0.25">
@@ -5730,10 +7226,25 @@
       </c>
     </row>
     <row r="60" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C60" s="2"/>
-      <c r="D60" s="3"/>
+      <c r="C60" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D60" s="69">
+        <f>MAX(0.4,1-(355/Fy)*(0.75-0.03*Le))</f>
+        <v>0.505</v>
+      </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
+      <c r="G60" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="H60" s="68">
+        <f>0.85*LL</f>
+        <v>8.5</v>
+      </c>
+      <c r="I60" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="61" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C61" s="15" t="s">
@@ -5752,7 +7263,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="65" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C65" s="2" t="s">
         <v>47</v>
       </c>
@@ -5764,7 +7275,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="66" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C66" s="15" t="s">
         <v>62</v>
       </c>
@@ -5775,8 +7286,12 @@
       <c r="E66" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="67" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="I66">
+        <f>Nw</f>
+        <v>848.02400000000011</v>
+      </c>
+    </row>
+    <row r="67" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C67" s="1" t="s">
         <v>174</v>
       </c>
@@ -5793,7 +7308,7 @@
         <v>1619.0006918323152</v>
       </c>
     </row>
-    <row r="69" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C69" s="15" t="s">
         <v>175</v>
       </c>
@@ -5810,7 +7325,7 @@
         <v>oui</v>
       </c>
     </row>
-    <row r="71" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C71" s="2" t="s">
         <v>74</v>
       </c>
@@ -5827,7 +7342,7 @@
         <v>0.62815160980356521</v>
       </c>
     </row>
-    <row r="72" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C72" s="2" t="s">
         <v>50</v>
       </c>
@@ -5844,13 +7359,13 @@
         <v>7.9775254445052779</v>
       </c>
     </row>
-    <row r="73" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C73" s="2"/>
       <c r="D73" s="3"/>
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C74" s="2" t="s">
         <v>176</v>
       </c>
@@ -5867,17 +7382,2416 @@
         <v>640.27285237589899</v>
       </c>
     </row>
-    <row r="75" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C75" s="2"/>
       <c r="D75" s="3"/>
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C76" s="2"/>
+    </row>
+    <row r="78" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="L78" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="M78" s="68">
+        <f>Wpl*Fy/GammaM0/1000</f>
+        <v>361.745</v>
+      </c>
+      <c r="N78" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="79" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="C79" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="80" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="C80" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="81" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C81" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="82" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="I82" s="70" t="s">
+        <v>193</v>
+      </c>
+      <c r="J82" s="71"/>
+      <c r="K82" s="71"/>
+      <c r="L82" s="72"/>
+      <c r="M82" s="76" t="s">
+        <v>193</v>
+      </c>
+      <c r="N82" s="77"/>
+      <c r="O82" s="77"/>
+      <c r="P82" s="78"/>
+      <c r="Q82" s="82" t="s">
+        <v>193</v>
+      </c>
+      <c r="R82" s="83"/>
+      <c r="S82" s="83"/>
+      <c r="T82" s="84"/>
+    </row>
+    <row r="83" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C83" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E83" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F83" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="G83" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I83" s="73" t="s">
+        <v>194</v>
+      </c>
+      <c r="J83" s="74" t="s">
+        <v>74</v>
+      </c>
+      <c r="K83" s="74" t="s">
+        <v>50</v>
+      </c>
+      <c r="L83" s="75" t="s">
+        <v>51</v>
+      </c>
+      <c r="M83" s="79" t="s">
+        <v>195</v>
+      </c>
+      <c r="N83" s="80" t="s">
+        <v>74</v>
+      </c>
+      <c r="O83" s="80" t="s">
+        <v>50</v>
+      </c>
+      <c r="P83" s="81" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q83" s="85" t="s">
+        <v>196</v>
+      </c>
+      <c r="R83" s="86" t="s">
+        <v>74</v>
+      </c>
+      <c r="S83" s="86" t="s">
+        <v>50</v>
+      </c>
+      <c r="T83" s="87" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="84" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B84" s="3">
+        <f>Feuil1!C75</f>
+        <v>1</v>
+      </c>
+      <c r="C84" s="18">
+        <f>Feuil1!D75</f>
+        <v>0</v>
+      </c>
+      <c r="D84" s="3">
+        <f>IF(C84&lt;$D$36,1,2)</f>
+        <v>2</v>
+      </c>
+      <c r="E84" s="13">
+        <f>IF(D84=1,IF(C84&lt;=$D$43,0,C84*$G$36),IF(C84-$D$36&lt;$D$44,0,MIN((C84-$D$36-$D$44)*$G$37,(LL-C84)*$G$37)))</f>
+        <v>0</v>
+      </c>
+      <c r="F84" s="17">
+        <f>E84/MIN($D$57:$D$58)</f>
+        <v>0</v>
+      </c>
+      <c r="G84" s="18">
+        <f>IF(I84=oui,L84,IF(M84=oui,P84,T84))</f>
+        <v>361.745</v>
+      </c>
+      <c r="I84" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E84,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J84" s="17">
+        <f>(Na-E84)/(2*Nf)</f>
+        <v>1.6843269986653329</v>
+      </c>
+      <c r="K84" s="17">
+        <f>J84*tf</f>
+        <v>21.390952883049724</v>
+      </c>
+      <c r="L84" s="17">
+        <f>(E84*(td-tc/2*F84)+Na*Ht/2-(Na-F84*Nc)*K84/2)/1000</f>
+        <v>437.12531991961151</v>
+      </c>
+      <c r="M84" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E84,E84&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N84" s="17">
+        <f>(E84-Nw)/(2*Nr)</f>
+        <v>-4.2195704181270575</v>
+      </c>
+      <c r="O84" s="18">
+        <f>dw/2+N84*rr</f>
+        <v>73.347732473712981</v>
+      </c>
+      <c r="P84" s="13">
+        <f>MplaRd+E84*(td-F84*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E84)*O84/1000</f>
+        <v>360.64064588328802</v>
+      </c>
+      <c r="Q84" s="67" t="str">
+        <f>IF(Nw&gt;E84,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R84" s="17">
+        <f>E84/2/Nw</f>
+        <v>0</v>
+      </c>
+      <c r="S84" s="13">
+        <f>R84*dw</f>
+        <v>0</v>
+      </c>
+      <c r="T84" s="13">
+        <f>MplaRd+E84*(Ht/2+td/2-F84*tc-S84/2)/1000</f>
+        <v>361.745</v>
+      </c>
+    </row>
+    <row r="85" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B85" s="3">
+        <f>Feuil1!C76</f>
+        <v>2</v>
+      </c>
+      <c r="C85" s="18">
+        <f>Feuil1!D76</f>
+        <v>0.5</v>
+      </c>
+      <c r="D85" s="3">
+        <f t="shared" ref="D85:D104" si="3">IF(C85&lt;$D$36,1,2)</f>
+        <v>2</v>
+      </c>
+      <c r="E85" s="13">
+        <f>IF(D85=1,IF(C85&lt;=$D$43,0,C85*$G$36),IF(C85-$D$36&lt;$D$44,0,MIN((C85-$D$36-$D$44)*$G$37,(LL-C85)*$G$37)))</f>
+        <v>0</v>
+      </c>
+      <c r="F85" s="17">
+        <f t="shared" ref="F85:F104" si="4">E85/MIN($D$57:$D$58)</f>
+        <v>0</v>
+      </c>
+      <c r="G85" s="18">
+        <f>IF(I85=oui,L85,IF(M85=oui,P85,T85))</f>
+        <v>361.745</v>
+      </c>
+      <c r="I85" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E85,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J85" s="17">
+        <f>(Na-E85)/(2*Nf)</f>
+        <v>1.6843269986653329</v>
+      </c>
+      <c r="K85" s="17">
+        <f>J85*tf</f>
+        <v>21.390952883049724</v>
+      </c>
+      <c r="L85" s="17">
+        <f>(E85*(td-tc/2*F85)+Na*Ht/2-(Na-F85*Nc)*K85/2)/1000</f>
+        <v>437.12531991961151</v>
+      </c>
+      <c r="M85" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E85,E85&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N85" s="17">
+        <f>(E85-Nw)/(2*Nr)</f>
+        <v>-4.2195704181270575</v>
+      </c>
+      <c r="O85" s="18">
+        <f>dw/2+N85*rr</f>
+        <v>73.347732473712981</v>
+      </c>
+      <c r="P85" s="13">
+        <f>MplaRd+E85*(td-F85*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E85)*O85/1000</f>
+        <v>360.64064588328802</v>
+      </c>
+      <c r="Q85" s="67" t="str">
+        <f>IF(Nw&gt;E85,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R85" s="17">
+        <f>E85/2/Nw</f>
+        <v>0</v>
+      </c>
+      <c r="S85" s="13">
+        <f>R85*dw</f>
+        <v>0</v>
+      </c>
+      <c r="T85" s="13">
+        <f>MplaRd+E85*(Ht/2+td/2-F85*tc-S85/2)/1000</f>
+        <v>361.745</v>
+      </c>
+    </row>
+    <row r="86" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B86" s="3">
+        <f>Feuil1!C77</f>
+        <v>3</v>
+      </c>
+      <c r="C86" s="18">
+        <f>Feuil1!D77</f>
+        <v>1</v>
+      </c>
+      <c r="D86" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E86" s="13">
+        <f>IF(D86=1,IF(C86&lt;=$D$43,0,C86*$G$36),IF(C86-$D$36&lt;$D$44,0,MIN((C86-$D$36-$D$44)*$G$37,(LL-C86)*$G$37)))</f>
+        <v>0</v>
+      </c>
+      <c r="F86" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G86" s="18">
+        <f>IF(I86=oui,L86,IF(M86=oui,P86,T86))</f>
+        <v>361.745</v>
+      </c>
+      <c r="I86" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E86,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J86" s="17">
+        <f>(Na-E86)/(2*Nf)</f>
+        <v>1.6843269986653329</v>
+      </c>
+      <c r="K86" s="17">
+        <f>J86*tf</f>
+        <v>21.390952883049724</v>
+      </c>
+      <c r="L86" s="17">
+        <f>(E86*(td-tc/2*F86)+Na*Ht/2-(Na-F86*Nc)*K86/2)/1000</f>
+        <v>437.12531991961151</v>
+      </c>
+      <c r="M86" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E86,E86&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N86" s="17">
+        <f>(E86-Nw)/(2*Nr)</f>
+        <v>-4.2195704181270575</v>
+      </c>
+      <c r="O86" s="18">
+        <f>dw/2+N86*rr</f>
+        <v>73.347732473712981</v>
+      </c>
+      <c r="P86" s="13">
+        <f>MplaRd+E86*(td-F86*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E86)*O86/1000</f>
+        <v>360.64064588328802</v>
+      </c>
+      <c r="Q86" s="67" t="str">
+        <f>IF(Nw&gt;E86,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R86" s="17">
+        <f>E86/2/Nw</f>
+        <v>0</v>
+      </c>
+      <c r="S86" s="13">
+        <f>R86*dw</f>
+        <v>0</v>
+      </c>
+      <c r="T86" s="13">
+        <f>MplaRd+E86*(Ht/2+td/2-F86*tc-S86/2)/1000</f>
+        <v>361.745</v>
+      </c>
+    </row>
+    <row r="87" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B87" s="3">
+        <f>Feuil1!C78</f>
+        <v>4</v>
+      </c>
+      <c r="C87" s="18">
+        <f>Feuil1!D78</f>
+        <v>1.5</v>
+      </c>
+      <c r="D87" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E87" s="13">
+        <f>IF(D87=1,IF(C87&lt;=$D$43,0,C87*$G$36),IF(C87-$D$36&lt;$D$44,0,MIN((C87-$D$36-$D$44)*$G$37,(LL-C87)*$G$37)))</f>
+        <v>0</v>
+      </c>
+      <c r="F87" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G87" s="18">
+        <f>IF(I87=oui,L87,IF(M87=oui,P87,T87))</f>
+        <v>361.745</v>
+      </c>
+      <c r="I87" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E87,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J87" s="17">
+        <f>(Na-E87)/(2*Nf)</f>
+        <v>1.6843269986653329</v>
+      </c>
+      <c r="K87" s="17">
+        <f>J87*tf</f>
+        <v>21.390952883049724</v>
+      </c>
+      <c r="L87" s="17">
+        <f>(E87*(td-tc/2*F87)+Na*Ht/2-(Na-F87*Nc)*K87/2)/1000</f>
+        <v>437.12531991961151</v>
+      </c>
+      <c r="M87" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E87,E87&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N87" s="17">
+        <f>(E87-Nw)/(2*Nr)</f>
+        <v>-4.2195704181270575</v>
+      </c>
+      <c r="O87" s="18">
+        <f>dw/2+N87*rr</f>
+        <v>73.347732473712981</v>
+      </c>
+      <c r="P87" s="13">
+        <f>MplaRd+E87*(td-F87*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E87)*O87/1000</f>
+        <v>360.64064588328802</v>
+      </c>
+      <c r="Q87" s="67" t="str">
+        <f>IF(Nw&gt;E87,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R87" s="17">
+        <f>E87/2/Nw</f>
+        <v>0</v>
+      </c>
+      <c r="S87" s="13">
+        <f>R87*dw</f>
+        <v>0</v>
+      </c>
+      <c r="T87" s="13">
+        <f>MplaRd+E87*(Ht/2+td/2-F87*tc-S87/2)/1000</f>
+        <v>361.745</v>
+      </c>
+    </row>
+    <row r="88" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B88" s="3">
+        <f>Feuil1!C79</f>
+        <v>5</v>
+      </c>
+      <c r="C88" s="18">
+        <f>Feuil1!D79</f>
+        <v>2</v>
+      </c>
+      <c r="D88" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E88" s="13">
+        <f>IF(D88=1,IF(C88&lt;=$D$43,0,C88*$G$36),IF(C88-$D$36&lt;$D$44,0,MIN((C88-$D$36-$D$44)*$G$37,(LL-C88)*$G$37)))</f>
+        <v>66.232969137448919</v>
+      </c>
+      <c r="F88" s="17">
+        <f t="shared" si="4"/>
+        <v>2.5652920964956177E-2</v>
+      </c>
+      <c r="G88" s="18">
+        <f>IF(I88=oui,L88,IF(M88=oui,P88,T88))</f>
+        <v>377.46358194417815</v>
+      </c>
+      <c r="I88" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E88,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J88" s="17">
+        <f>(Na-E88)/(2*Nf)</f>
+        <v>1.6411190912894293</v>
+      </c>
+      <c r="K88" s="17">
+        <f>J88*tf</f>
+        <v>20.842212459375752</v>
+      </c>
+      <c r="L88" s="17">
+        <f>(E88*(td-tc/2*F88)+Na*Ht/2-(Na-F88*Nc)*K88/2)/1000</f>
+        <v>447.19405097116191</v>
+      </c>
+      <c r="M88" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E88,E88&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N88" s="17">
+        <f>(E88-Nw)/(2*Nr)</f>
+        <v>-3.8900105503908828</v>
+      </c>
+      <c r="O88" s="18">
+        <f>dw/2+N88*rr</f>
+        <v>79.279810092964127</v>
+      </c>
+      <c r="P88" s="13">
+        <f>MplaRd+E88*(td-F88*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E88)*O88/1000</f>
+        <v>380.8913068033628</v>
+      </c>
+      <c r="Q88" s="67" t="str">
+        <f>IF(Nw&gt;E88,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R88" s="17">
+        <f>E88/2/Nw</f>
+        <v>3.9051352990863999E-2</v>
+      </c>
+      <c r="S88" s="13">
+        <f>R88*dw</f>
+        <v>11.66073400307199</v>
+      </c>
+      <c r="T88" s="13">
+        <f>MplaRd+E88*(Ht/2+td/2-F88*tc-S88/2)/1000</f>
+        <v>377.46358194417815</v>
+      </c>
+    </row>
+    <row r="89" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B89" s="3">
+        <f>Feuil1!C80</f>
+        <v>6</v>
+      </c>
+      <c r="C89" s="18">
+        <f>Feuil1!D80</f>
+        <v>2.5</v>
+      </c>
+      <c r="D89" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E89" s="13">
+        <f>IF(D89=1,IF(C89&lt;=$D$43,0,C89*$G$36),IF(C89-$D$36&lt;$D$44,0,MIN((C89-$D$36-$D$44)*$G$37,(LL-C89)*$G$37)))</f>
+        <v>264.91252467339336</v>
+      </c>
+      <c r="F89" s="17">
+        <f t="shared" si="4"/>
+        <v>0.10260418861746523</v>
+      </c>
+      <c r="G89" s="18">
+        <f>IF(I89=oui,L89,IF(M89=oui,P89,T89))</f>
+        <v>418.51382916287656</v>
+      </c>
+      <c r="I89" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E89,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J89" s="17">
+        <f>(Na-E89)/(2*Nf)</f>
+        <v>1.511507993600786</v>
+      </c>
+      <c r="K89" s="17">
+        <f>J89*tf</f>
+        <v>19.19615151872998</v>
+      </c>
+      <c r="L89" s="17">
+        <f>(E89*(td-tc/2*F89)+Na*Ht/2-(Na-F89*Nc)*K89/2)/1000</f>
+        <v>476.40717696900123</v>
+      </c>
+      <c r="M89" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E89,E89&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N89" s="17">
+        <f>(E89-Nw)/(2*Nr)</f>
+        <v>-2.9014272376236696</v>
+      </c>
+      <c r="O89" s="18">
+        <f>dw/2+N89*rr</f>
+        <v>97.074309722773961</v>
+      </c>
+      <c r="P89" s="13">
+        <f>MplaRd+E89*(td-F89*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E89)*O89/1000</f>
+        <v>436.18951416015676</v>
+      </c>
+      <c r="Q89" s="67" t="str">
+        <f>IF(Nw&gt;E89,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R89" s="17">
+        <f>E89/2/Nw</f>
+        <v>0.15619400198189753</v>
+      </c>
+      <c r="S89" s="13">
+        <f>R89*dw</f>
+        <v>46.639528991794606</v>
+      </c>
+      <c r="T89" s="13">
+        <f>MplaRd+E89*(Ht/2+td/2-F89*tc-S89/2)/1000</f>
+        <v>418.51382916287656</v>
+      </c>
+    </row>
+    <row r="90" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B90" s="3">
+        <f>Feuil1!C81</f>
+        <v>7</v>
+      </c>
+      <c r="C90" s="18">
+        <f>Feuil1!D81</f>
+        <v>3</v>
+      </c>
+      <c r="D90" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E90" s="13">
+        <f>IF(D90=1,IF(C90&lt;=$D$43,0,C90*$G$36),IF(C90-$D$36&lt;$D$44,0,MIN((C90-$D$36-$D$44)*$G$37,(LL-C90)*$G$37)))</f>
+        <v>463.59208020933784</v>
+      </c>
+      <c r="F90" s="17">
+        <f t="shared" si="4"/>
+        <v>0.17955545626997432</v>
+      </c>
+      <c r="G90" s="18">
+        <f>IF(I90=oui,L90,IF(M90=oui,P90,T90))</f>
+        <v>450.41294025369427</v>
+      </c>
+      <c r="I90" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E90,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J90" s="17">
+        <f>(Na-E90)/(2*Nf)</f>
+        <v>1.3818968959121427</v>
+      </c>
+      <c r="K90" s="17">
+        <f>J90*tf</f>
+        <v>17.550090578084212</v>
+      </c>
+      <c r="L90" s="17">
+        <f>(E90*(td-tc/2*F90)+Na*Ht/2-(Na-F90*Nc)*K90/2)/1000</f>
+        <v>504.13515120220092</v>
+      </c>
+      <c r="M90" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E90,E90&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N90" s="17">
+        <f>(E90-Nw)/(2*Nr)</f>
+        <v>-1.9128439248564568</v>
+      </c>
+      <c r="O90" s="18">
+        <f>dw/2+N90*rr</f>
+        <v>114.86880935258378</v>
+      </c>
+      <c r="P90" s="13">
+        <f>MplaRd+E90*(td-F90*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E90)*O90/1000</f>
+        <v>483.31613261891124</v>
+      </c>
+      <c r="Q90" s="67" t="str">
+        <f>IF(Nw&gt;E90,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R90" s="17">
+        <f>E90/2/Nw</f>
+        <v>0.27333665097293108</v>
+      </c>
+      <c r="S90" s="13">
+        <f>R90*dw</f>
+        <v>81.618323980517232</v>
+      </c>
+      <c r="T90" s="13">
+        <f>MplaRd+E90*(Ht/2+td/2-F90*tc-S90/2)/1000</f>
+        <v>450.41294025369427</v>
+      </c>
+    </row>
+    <row r="91" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B91" s="3">
+        <f>Feuil1!C82</f>
+        <v>8</v>
+      </c>
+      <c r="C91" s="18">
+        <f>Feuil1!D82</f>
+        <v>3.5</v>
+      </c>
+      <c r="D91" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E91" s="13">
+        <f>IF(D91=1,IF(C91&lt;=$D$43,0,C91*$G$36),IF(C91-$D$36&lt;$D$44,0,MIN((C91-$D$36-$D$44)*$G$37,(LL-C91)*$G$37)))</f>
+        <v>662.27163574528231</v>
+      </c>
+      <c r="F91" s="17">
+        <f t="shared" si="4"/>
+        <v>0.25650672392248336</v>
+      </c>
+      <c r="G91" s="18">
+        <f>IF(I91=oui,L91,IF(M91=oui,P91,T91))</f>
+        <v>473.16091521663122</v>
+      </c>
+      <c r="I91" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E91,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J91" s="17">
+        <f>(Na-E91)/(2*Nf)</f>
+        <v>1.2522857982234994</v>
+      </c>
+      <c r="K91" s="17">
+        <f>J91*tf</f>
+        <v>15.904029637438441</v>
+      </c>
+      <c r="L91" s="17">
+        <f>(E91*(td-tc/2*F91)+Na*Ht/2-(Na-F91*Nc)*K91/2)/1000</f>
+        <v>530.37797367076087</v>
+      </c>
+      <c r="M91" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E91,E91&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N91" s="17">
+        <f>(E91-Nw)/(2*Nr)</f>
+        <v>-0.92426061208924393</v>
+      </c>
+      <c r="O91" s="18">
+        <f>dw/2+N91*rr</f>
+        <v>132.66330898239363</v>
+      </c>
+      <c r="P91" s="13">
+        <f>MplaRd+E91*(td-F91*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E91)*O91/1000</f>
+        <v>522.27116217962623</v>
+      </c>
+      <c r="Q91" s="67" t="str">
+        <f>IF(Nw&gt;E91,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R91" s="17">
+        <f>E91/2/Nw</f>
+        <v>0.39047929996396458</v>
+      </c>
+      <c r="S91" s="13">
+        <f>R91*dw</f>
+        <v>116.59711896923983</v>
+      </c>
+      <c r="T91" s="13">
+        <f>MplaRd+E91*(Ht/2+td/2-F91*tc-S91/2)/1000</f>
+        <v>473.16091521663122</v>
+      </c>
+    </row>
+    <row r="92" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B92" s="3">
+        <f>Feuil1!C83</f>
+        <v>9</v>
+      </c>
+      <c r="C92" s="18">
+        <f>Feuil1!D83</f>
+        <v>4</v>
+      </c>
+      <c r="D92" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E92" s="13">
+        <f>IF(D92=1,IF(C92&lt;=$D$43,0,C92*$G$36),IF(C92-$D$36&lt;$D$44,0,MIN((C92-$D$36-$D$44)*$G$37,(LL-C92)*$G$37)))</f>
+        <v>860.95119128122678</v>
+      </c>
+      <c r="F92" s="17">
+        <f t="shared" si="4"/>
+        <v>0.33345799157499245</v>
+      </c>
+      <c r="G92" s="18">
+        <f>IF(I92=oui,L92,IF(M92=oui,P92,T92))</f>
+        <v>553.05460284230173</v>
+      </c>
+      <c r="I92" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E92,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J92" s="17">
+        <f>(Na-E92)/(2*Nf)</f>
+        <v>1.1226747005348561</v>
+      </c>
+      <c r="K92" s="17">
+        <f>J92*tf</f>
+        <v>14.257968696792672</v>
+      </c>
+      <c r="L92" s="17">
+        <f>(E92*(td-tc/2*F92)+Na*Ht/2-(Na-F92*Nc)*K92/2)/1000</f>
+        <v>555.13564437468119</v>
+      </c>
+      <c r="M92" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E92,E92&gt;=Nw),oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="N92" s="17">
+        <f>(E92-Nw)/(2*Nr)</f>
+        <v>6.4322700677969094E-2</v>
+      </c>
+      <c r="O92" s="18">
+        <f>dw/2+N92*rr</f>
+        <v>150.45780861220345</v>
+      </c>
+      <c r="P92" s="13">
+        <f>MplaRd+E92*(td-F92*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E92)*O92/1000</f>
+        <v>553.05460284230173</v>
+      </c>
+      <c r="Q92" s="67" t="str">
+        <f>IF(Nw&gt;E92,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="R92" s="17">
+        <f>E92/2/Nw</f>
+        <v>0.50762194895499813</v>
+      </c>
+      <c r="S92" s="13">
+        <f>R92*dw</f>
+        <v>151.57591395796246</v>
+      </c>
+      <c r="T92" s="13">
+        <f>MplaRd+E92*(Ht/2+td/2-F92*tc-S92/2)/1000</f>
+        <v>486.75775405168736</v>
+      </c>
+    </row>
+    <row r="93" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B93" s="3">
+        <f>Feuil1!C84</f>
+        <v>10</v>
+      </c>
+      <c r="C93" s="18">
+        <f>Feuil1!D84</f>
+        <v>4.5</v>
+      </c>
+      <c r="D93" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E93" s="13">
+        <f>IF(D93=1,IF(C93&lt;=$D$43,0,C93*$G$36),IF(C93-$D$36&lt;$D$44,0,MIN((C93-$D$36-$D$44)*$G$37,(LL-C93)*$G$37)))</f>
+        <v>1059.6307468171713</v>
+      </c>
+      <c r="F93" s="17">
+        <f t="shared" si="4"/>
+        <v>0.41040925922750154</v>
+      </c>
+      <c r="G93" s="18">
+        <f>IF(I93=oui,L93,IF(M93=oui,P93,T93))</f>
+        <v>578.40816331396184</v>
+      </c>
+      <c r="I93" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E93,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="J93" s="17">
+        <f>(Na-E93)/(2*Nf)</f>
+        <v>0.99306360284621265</v>
+      </c>
+      <c r="K93" s="17">
+        <f>J93*tf</f>
+        <v>12.6119077561469</v>
+      </c>
+      <c r="L93" s="17">
+        <f>(E93*(td-tc/2*F93)+Na*Ht/2-(Na-F93*Nc)*K93/2)/1000</f>
+        <v>578.40816331396184</v>
+      </c>
+      <c r="M93" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E93,E93&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N93" s="17">
+        <f>(E93-Nw)/(2*Nr)</f>
+        <v>1.052906013445182</v>
+      </c>
+      <c r="O93" s="18">
+        <f>dw/2+N93*rr</f>
+        <v>168.25230824201327</v>
+      </c>
+      <c r="P93" s="13">
+        <f>MplaRd+E93*(td-F93*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E93)*O93/1000</f>
+        <v>575.66645460693769</v>
+      </c>
+      <c r="Q93" s="67" t="str">
+        <f>IF(Nw&gt;E93,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="R93" s="17">
+        <f>E93/2/Nw</f>
+        <v>0.62476459794603167</v>
+      </c>
+      <c r="S93" s="13">
+        <f>R93*dw</f>
+        <v>186.55470894668508</v>
+      </c>
+      <c r="T93" s="13">
+        <f>MplaRd+E93*(Ht/2+td/2-F93*tc-S93/2)/1000</f>
+        <v>491.20345675886279</v>
+      </c>
+    </row>
+    <row r="94" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B94" s="3">
+        <f>Feuil1!C85</f>
+        <v>11</v>
+      </c>
+      <c r="C94" s="18">
+        <f>Feuil1!D85</f>
+        <v>5</v>
+      </c>
+      <c r="D94" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E94" s="13">
+        <f>IF(D94=1,IF(C94&lt;=$D$43,0,C94*$G$36),IF(C94-$D$36&lt;$D$44,0,MIN((C94-$D$36-$D$44)*$G$37,(LL-C94)*$G$37)))</f>
+        <v>1258.3103023531157</v>
+      </c>
+      <c r="F94" s="17">
+        <f t="shared" si="4"/>
+        <v>0.48736052688001058</v>
+      </c>
+      <c r="G94" s="18">
+        <f>IF(I94=oui,L94,IF(M94=oui,P94,T94))</f>
+        <v>600.19553048860269</v>
+      </c>
+      <c r="I94" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E94,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="J94" s="17">
+        <f>(Na-E94)/(2*Nf)</f>
+        <v>0.86345250515756933</v>
+      </c>
+      <c r="K94" s="17">
+        <f>J94*tf</f>
+        <v>10.965846815501131</v>
+      </c>
+      <c r="L94" s="17">
+        <f>(E94*(td-tc/2*F94)+Na*Ht/2-(Na-F94*Nc)*K94/2)/1000</f>
+        <v>600.19553048860269</v>
+      </c>
+      <c r="M94" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E94,E94&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N94" s="17">
+        <f>(E94-Nw)/(2*Nr)</f>
+        <v>2.0414893262123952</v>
+      </c>
+      <c r="O94" s="18">
+        <f>dw/2+N94*rr</f>
+        <v>186.04680787182312</v>
+      </c>
+      <c r="P94" s="13">
+        <f>MplaRd+E94*(td-F94*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E94)*O94/1000</f>
+        <v>590.1067174735341</v>
+      </c>
+      <c r="Q94" s="67" t="str">
+        <f>IF(Nw&gt;E94,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="R94" s="17">
+        <f>E94/2/Nw</f>
+        <v>0.74190724693706522</v>
+      </c>
+      <c r="S94" s="13">
+        <f>R94*dw</f>
+        <v>221.53350393540768</v>
+      </c>
+      <c r="T94" s="13">
+        <f>MplaRd+E94*(Ht/2+td/2-F94*tc-S94/2)/1000</f>
+        <v>486.49802333815745</v>
+      </c>
+    </row>
+    <row r="95" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B95" s="3">
+        <f>Feuil1!C86</f>
+        <v>12</v>
+      </c>
+      <c r="C95" s="18">
+        <f>Feuil1!D86</f>
+        <v>5.5</v>
+      </c>
+      <c r="D95" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E95" s="13">
+        <f>IF(D95=1,IF(C95&lt;=$D$43,0,C95*$G$36),IF(C95-$D$36&lt;$D$44,0,MIN((C95-$D$36-$D$44)*$G$37,(LL-C95)*$G$37)))</f>
+        <v>1456.9898578890602</v>
+      </c>
+      <c r="F95" s="17">
+        <f t="shared" si="4"/>
+        <v>0.56431179453251967</v>
+      </c>
+      <c r="G95" s="18">
+        <f>IF(I95=oui,L95,IF(M95=oui,P95,T95))</f>
+        <v>620.49774589860397</v>
+      </c>
+      <c r="I95" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E95,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="J95" s="17">
+        <f>(Na-E95)/(2*Nf)</f>
+        <v>0.73384140746892601</v>
+      </c>
+      <c r="K95" s="17">
+        <f>J95*tf</f>
+        <v>9.3197858748553593</v>
+      </c>
+      <c r="L95" s="17">
+        <f>(E95*(td-tc/2*F95)+Na*Ht/2-(Na-F95*Nc)*K95/2)/1000</f>
+        <v>620.49774589860397</v>
+      </c>
+      <c r="M95" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E95,E95&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N95" s="17">
+        <f>(E95-Nw)/(2*Nr)</f>
+        <v>3.030072638979608</v>
+      </c>
+      <c r="O95" s="18">
+        <f>dw/2+N95*rr</f>
+        <v>203.84130750163297</v>
+      </c>
+      <c r="P95" s="13">
+        <f>MplaRd+E95*(td-F95*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E95)*O95/1000</f>
+        <v>596.37539144209109</v>
+      </c>
+      <c r="Q95" s="67" t="str">
+        <f>IF(Nw&gt;E95,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="R95" s="17">
+        <f>E95/2/Nw</f>
+        <v>0.85904989592809877</v>
+      </c>
+      <c r="S95" s="13">
+        <f>R95*dw</f>
+        <v>256.51229892413033</v>
+      </c>
+      <c r="T95" s="13">
+        <f>MplaRd+E95*(Ht/2+td/2-F95*tc-S95/2)/1000</f>
+        <v>472.6414537895713</v>
+      </c>
+    </row>
+    <row r="96" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B96" s="3">
+        <f>Feuil1!C87</f>
+        <v>13</v>
+      </c>
+      <c r="C96" s="18">
+        <f>Feuil1!D87</f>
+        <v>6</v>
+      </c>
+      <c r="D96" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E96" s="13">
+        <f>IF(D96=1,IF(C96&lt;=$D$43,0,C96*$G$36),IF(C96-$D$36&lt;$D$44,0,MIN((C96-$D$36-$D$44)*$G$37,(LL-C96)*$G$37)))</f>
+        <v>1589.4364442875558</v>
+      </c>
+      <c r="F96" s="17">
+        <f t="shared" si="4"/>
+        <v>0.61561014122007263</v>
+      </c>
+      <c r="G96" s="18">
+        <f>IF(I96=oui,L96,IF(M96=oui,P96,T96))</f>
+        <v>633.20686895126073</v>
+      </c>
+      <c r="I96" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E96,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="J96" s="17">
+        <f>(Na-E96)/(2*Nf)</f>
+        <v>0.64743821715618632</v>
+      </c>
+      <c r="K96" s="17">
+        <f>J96*tf</f>
+        <v>8.222465357883566</v>
+      </c>
+      <c r="L96" s="17">
+        <f>(E96*(td-tc/2*F96)+Na*Ht/2-(Na-F96*Nc)*K96/2)/1000</f>
+        <v>633.20686895126073</v>
+      </c>
+      <c r="M96" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E96,E96&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N96" s="17">
+        <f>(E96-Nw)/(2*Nr)</f>
+        <v>3.6890960840106466</v>
+      </c>
+      <c r="O96" s="18">
+        <f>dw/2+N96*rr</f>
+        <v>215.70372951219164</v>
+      </c>
+      <c r="P96" s="13">
+        <f>MplaRd+E96*(td-F96*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E96)*O96/1000</f>
+        <v>596.01484180815157</v>
+      </c>
+      <c r="Q96" s="67" t="str">
+        <f>IF(Nw&gt;E96,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="R96" s="17">
+        <f>E96/2/Nw</f>
+        <v>0.93714119192826828</v>
+      </c>
+      <c r="S96" s="13">
+        <f>R96*dw</f>
+        <v>279.83035990978095</v>
+      </c>
+      <c r="T96" s="13">
+        <f>MplaRd+E96*(Ht/2+td/2-F96*tc-S96/2)/1000</f>
+        <v>458.32057275826674</v>
+      </c>
+    </row>
+    <row r="97" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B97" s="3">
+        <f>Feuil1!C88</f>
+        <v>14</v>
+      </c>
+      <c r="C97" s="18">
+        <f>Feuil1!D88</f>
+        <v>6.5</v>
+      </c>
+      <c r="D97" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E97" s="13">
+        <f>IF(D97=1,IF(C97&lt;=$D$43,0,C97*$G$36),IF(C97-$D$36&lt;$D$44,0,MIN((C97-$D$36-$D$44)*$G$37,(LL-C97)*$G$37)))</f>
+        <v>1390.7568887516113</v>
+      </c>
+      <c r="F97" s="17">
+        <f t="shared" si="4"/>
+        <v>0.53865887356756348</v>
+      </c>
+      <c r="G97" s="18">
+        <f>IF(I97=oui,L97,IF(M97=oui,P97,T97))</f>
+        <v>613.89470649854354</v>
+      </c>
+      <c r="I97" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E97,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="J97" s="17">
+        <f>(Na-E97)/(2*Nf)</f>
+        <v>0.77704931484482964</v>
+      </c>
+      <c r="K97" s="17">
+        <f>J97*tf</f>
+        <v>9.8685262985293356</v>
+      </c>
+      <c r="L97" s="17">
+        <f>(E97*(td-tc/2*F97)+Na*Ht/2-(Na-F97*Nc)*K97/2)/1000</f>
+        <v>613.89470649854354</v>
+      </c>
+      <c r="M97" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E97,E97&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N97" s="17">
+        <f>(E97-Nw)/(2*Nr)</f>
+        <v>2.7005127712434334</v>
+      </c>
+      <c r="O97" s="18">
+        <f>dw/2+N97*rr</f>
+        <v>197.90922988238179</v>
+      </c>
+      <c r="P97" s="13">
+        <f>MplaRd+E97*(td-F97*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E97)*O97/1000</f>
+        <v>595.19362846068191</v>
+      </c>
+      <c r="Q97" s="67" t="str">
+        <f>IF(Nw&gt;E97,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="R97" s="17">
+        <f>E97/2/Nw</f>
+        <v>0.81999854293723473</v>
+      </c>
+      <c r="S97" s="13">
+        <f>R97*dw</f>
+        <v>244.8515649210583</v>
+      </c>
+      <c r="T97" s="13">
+        <f>MplaRd+E97*(Ht/2+td/2-F97*tc-S97/2)/1000</f>
+        <v>478.27760261106607</v>
+      </c>
+    </row>
+    <row r="98" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B98" s="3">
+        <f>Feuil1!C89</f>
+        <v>15</v>
+      </c>
+      <c r="C98" s="18">
+        <f>Feuil1!D89</f>
+        <v>7</v>
+      </c>
+      <c r="D98" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E98" s="13">
+        <f>IF(D98=1,IF(C98&lt;=$D$43,0,C98*$G$36),IF(C98-$D$36&lt;$D$44,0,MIN((C98-$D$36-$D$44)*$G$37,(LL-C98)*$G$37)))</f>
+        <v>1192.0773332156668</v>
+      </c>
+      <c r="F98" s="17">
+        <f t="shared" si="4"/>
+        <v>0.46170760591505444</v>
+      </c>
+      <c r="G98" s="18">
+        <f>IF(I98=oui,L98,IF(M98=oui,P98,T98))</f>
+        <v>593.09739228118656</v>
+      </c>
+      <c r="I98" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E98,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="J98" s="17">
+        <f>(Na-E98)/(2*Nf)</f>
+        <v>0.90666041253347296</v>
+      </c>
+      <c r="K98" s="17">
+        <f>J98*tf</f>
+        <v>11.514587239175105</v>
+      </c>
+      <c r="L98" s="17">
+        <f>(E98*(td-tc/2*F98)+Na*Ht/2-(Na-F98*Nc)*K98/2)/1000</f>
+        <v>593.09739228118656</v>
+      </c>
+      <c r="M98" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E98,E98&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N98" s="17">
+        <f>(E98-Nw)/(2*Nr)</f>
+        <v>1.7119294584762206</v>
+      </c>
+      <c r="O98" s="18">
+        <f>dw/2+N98*rr</f>
+        <v>180.11473025257197</v>
+      </c>
+      <c r="P98" s="13">
+        <f>MplaRd+E98*(td-F98*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E98)*O98/1000</f>
+        <v>586.2008262151727</v>
+      </c>
+      <c r="Q98" s="67" t="str">
+        <f>IF(Nw&gt;E98,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="R98" s="17">
+        <f>E98/2/Nw</f>
+        <v>0.70285589394620118</v>
+      </c>
+      <c r="S98" s="13">
+        <f>R98*dw</f>
+        <v>209.8727699323357</v>
+      </c>
+      <c r="T98" s="13">
+        <f>MplaRd+E98*(Ht/2+td/2-F98*tc-S98/2)/1000</f>
+        <v>489.08349633598465</v>
+      </c>
+    </row>
+    <row r="99" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B99" s="3">
+        <f>Feuil1!C90</f>
+        <v>16</v>
+      </c>
+      <c r="C99" s="18">
+        <f>Feuil1!D90</f>
+        <v>7.5</v>
+      </c>
+      <c r="D99" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E99" s="13">
+        <f>IF(D99=1,IF(C99&lt;=$D$43,0,C99*$G$36),IF(C99-$D$36&lt;$D$44,0,MIN((C99-$D$36-$D$44)*$G$37,(LL-C99)*$G$37)))</f>
+        <v>993.39777767972237</v>
+      </c>
+      <c r="F99" s="17">
+        <f t="shared" si="4"/>
+        <v>0.38475633826254535</v>
+      </c>
+      <c r="G99" s="18">
+        <f>IF(I99=oui,L99,IF(M99=oui,P99,T99))</f>
+        <v>569.03643507162406</v>
+      </c>
+      <c r="I99" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E99,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J99" s="17">
+        <f>(Na-E99)/(2*Nf)</f>
+        <v>1.0362715102221163</v>
+      </c>
+      <c r="K99" s="17">
+        <f>J99*tf</f>
+        <v>13.160648179820877</v>
+      </c>
+      <c r="L99" s="17">
+        <f>(E99*(td-tc/2*F99)+Na*Ht/2-(Na-F99*Nc)*K99/2)/1000</f>
+        <v>570.81492629918989</v>
+      </c>
+      <c r="M99" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E99,E99&gt;=Nw),oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="N99" s="17">
+        <f>(E99-Nw)/(2*Nr)</f>
+        <v>0.72334614570900757</v>
+      </c>
+      <c r="O99" s="18">
+        <f>dw/2+N99*rr</f>
+        <v>162.32023062276215</v>
+      </c>
+      <c r="P99" s="13">
+        <f>MplaRd+E99*(td-F99*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E99)*O99/1000</f>
+        <v>569.03643507162406</v>
+      </c>
+      <c r="Q99" s="67" t="str">
+        <f>IF(Nw&gt;E99,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="R99" s="17">
+        <f>E99/2/Nw</f>
+        <v>0.58571324495516763</v>
+      </c>
+      <c r="S99" s="13">
+        <f>R99*dw</f>
+        <v>174.89397494361307</v>
+      </c>
+      <c r="T99" s="13">
+        <f>MplaRd+E99*(Ht/2+td/2-F99*tc-S99/2)/1000</f>
+        <v>490.73825393302246</v>
+      </c>
+    </row>
+    <row r="100" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B100" s="3">
+        <f>Feuil1!C91</f>
+        <v>17</v>
+      </c>
+      <c r="C100" s="18">
+        <f>Feuil1!D91</f>
+        <v>8</v>
+      </c>
+      <c r="D100" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E100" s="13">
+        <f>IF(D100=1,IF(C100&lt;=$D$43,0,C100*$G$36),IF(C100-$D$36&lt;$D$44,0,MIN((C100-$D$36-$D$44)*$G$37,(LL-C100)*$G$37)))</f>
+        <v>794.71822214377789</v>
+      </c>
+      <c r="F100" s="17">
+        <f t="shared" si="4"/>
+        <v>0.30780507061003631</v>
+      </c>
+      <c r="G100" s="18">
+        <f>IF(I100=oui,L100,IF(M100=oui,P100,T100))</f>
+        <v>483.24187540217946</v>
+      </c>
+      <c r="I100" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E100,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J100" s="17">
+        <f>(Na-E100)/(2*Nf)</f>
+        <v>1.1658826079107596</v>
+      </c>
+      <c r="K100" s="17">
+        <f>J100*tf</f>
+        <v>14.806709120466646</v>
+      </c>
+      <c r="L100" s="17">
+        <f>(E100*(td-tc/2*F100)+Na*Ht/2-(Na-F100*Nc)*K100/2)/1000</f>
+        <v>547.04730855255366</v>
+      </c>
+      <c r="M100" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E100,E100&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N100" s="17">
+        <f>(E100-Nw)/(2*Nr)</f>
+        <v>-0.26523716705820544</v>
+      </c>
+      <c r="O100" s="18">
+        <f>dw/2+N100*rr</f>
+        <v>144.5257309929523</v>
+      </c>
+      <c r="P100" s="13">
+        <f>MplaRd+E100*(td-F100*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E100)*O100/1000</f>
+        <v>543.70045503003587</v>
+      </c>
+      <c r="Q100" s="67" t="str">
+        <f>IF(Nw&gt;E100,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R100" s="17">
+        <f>E100/2/Nw</f>
+        <v>0.46857059596413414</v>
+      </c>
+      <c r="S100" s="13">
+        <f>R100*dw</f>
+        <v>139.91517995489048</v>
+      </c>
+      <c r="T100" s="13">
+        <f>MplaRd+E100*(Ht/2+td/2-F100*tc-S100/2)/1000</f>
+        <v>483.24187540217946</v>
+      </c>
+    </row>
+    <row r="101" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B101" s="3">
+        <f>Feuil1!C92</f>
+        <v>18</v>
+      </c>
+      <c r="C101" s="18">
+        <f>Feuil1!D92</f>
+        <v>8.5</v>
+      </c>
+      <c r="D101" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E101" s="13">
+        <f>IF(D101=1,IF(C101&lt;=$D$43,0,C101*$G$36),IF(C101-$D$36&lt;$D$44,0,MIN((C101-$D$36-$D$44)*$G$37,(LL-C101)*$G$37)))</f>
+        <v>596.03866660783342</v>
+      </c>
+      <c r="F101" s="17">
+        <f t="shared" si="4"/>
+        <v>0.23085380295752722</v>
+      </c>
+      <c r="G101" s="18">
+        <f>IF(I101=oui,L101,IF(M101=oui,P101,T101))</f>
+        <v>466.59436074345575</v>
+      </c>
+      <c r="I101" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E101,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J101" s="17">
+        <f>(Na-E101)/(2*Nf)</f>
+        <v>1.2954937055994029</v>
+      </c>
+      <c r="K101" s="17">
+        <f>J101*tf</f>
+        <v>16.452770061112417</v>
+      </c>
+      <c r="L101" s="17">
+        <f>(E101*(td-tc/2*F101)+Na*Ht/2-(Na-F101*Nc)*K101/2)/1000</f>
+        <v>521.79453904127763</v>
+      </c>
+      <c r="M101" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E101,E101&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N101" s="17">
+        <f>(E101-Nw)/(2*Nr)</f>
+        <v>-1.2538204798254184</v>
+      </c>
+      <c r="O101" s="18">
+        <f>dw/2+N101*rr</f>
+        <v>126.73123136314248</v>
+      </c>
+      <c r="P101" s="13">
+        <f>MplaRd+E101*(td-F101*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E101)*O101/1000</f>
+        <v>510.19288609040814</v>
+      </c>
+      <c r="Q101" s="67" t="str">
+        <f>IF(Nw&gt;E101,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R101" s="17">
+        <f>E101/2/Nw</f>
+        <v>0.35142794697310059</v>
+      </c>
+      <c r="S101" s="13">
+        <f>R101*dw</f>
+        <v>104.93638496616785</v>
+      </c>
+      <c r="T101" s="13">
+        <f>MplaRd+E101*(Ht/2+td/2-F101*tc-S101/2)/1000</f>
+        <v>466.59436074345575</v>
+      </c>
+    </row>
+    <row r="102" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B102" s="3">
+        <f>Feuil1!C93</f>
+        <v>19</v>
+      </c>
+      <c r="C102" s="18">
+        <f>Feuil1!D93</f>
+        <v>9</v>
+      </c>
+      <c r="D102" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E102" s="13">
+        <f>IF(D102=1,IF(C102&lt;=$D$43,0,C102*$G$36),IF(C102-$D$36&lt;$D$44,0,MIN((C102-$D$36-$D$44)*$G$37,(LL-C102)*$G$37)))</f>
+        <v>397.35911107188895</v>
+      </c>
+      <c r="F102" s="17">
+        <f t="shared" si="4"/>
+        <v>0.15390253530501816</v>
+      </c>
+      <c r="G102" s="18">
+        <f>IF(I102=oui,L102,IF(M102=oui,P102,T102))</f>
+        <v>440.79570995685128</v>
+      </c>
+      <c r="I102" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E102,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J102" s="17">
+        <f>(Na-E102)/(2*Nf)</f>
+        <v>1.4251048032880462</v>
+      </c>
+      <c r="K102" s="17">
+        <f>J102*tf</f>
+        <v>18.098831001758185</v>
+      </c>
+      <c r="L102" s="17">
+        <f>(E102*(td-tc/2*F102)+Na*Ht/2-(Na-F102*Nc)*K102/2)/1000</f>
+        <v>495.05661776536198</v>
+      </c>
+      <c r="M102" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E102,E102&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N102" s="17">
+        <f>(E102-Nw)/(2*Nr)</f>
+        <v>-2.2424037925926315</v>
+      </c>
+      <c r="O102" s="18">
+        <f>dw/2+N102*rr</f>
+        <v>108.93673173333264</v>
+      </c>
+      <c r="P102" s="13">
+        <f>MplaRd+E102*(td-F102*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E102)*O102/1000</f>
+        <v>468.51372825274098</v>
+      </c>
+      <c r="Q102" s="67" t="str">
+        <f>IF(Nw&gt;E102,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R102" s="17">
+        <f>E102/2/Nw</f>
+        <v>0.23428529798206707</v>
+      </c>
+      <c r="S102" s="13">
+        <f>R102*dw</f>
+        <v>69.957589977445238</v>
+      </c>
+      <c r="T102" s="13">
+        <f>MplaRd+E102*(Ht/2+td/2-F102*tc-S102/2)/1000</f>
+        <v>440.79570995685128</v>
+      </c>
+    </row>
+    <row r="103" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B103" s="3">
+        <f>Feuil1!C94</f>
+        <v>20</v>
+      </c>
+      <c r="C103" s="18">
+        <f>Feuil1!D94</f>
+        <v>9.5</v>
+      </c>
+      <c r="D103" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E103" s="13">
+        <f>IF(D103=1,IF(C103&lt;=$D$43,0,C103*$G$36),IF(C103-$D$36&lt;$D$44,0,MIN((C103-$D$36-$D$44)*$G$37,(LL-C103)*$G$37)))</f>
+        <v>198.67955553594447</v>
+      </c>
+      <c r="F103" s="17">
+        <f t="shared" si="4"/>
+        <v>7.6951267652509078E-2</v>
+      </c>
+      <c r="G103" s="18">
+        <f>IF(I103=oui,L103,IF(M103=oui,P103,T103))</f>
+        <v>405.84592304236605</v>
+      </c>
+      <c r="I103" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E103,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J103" s="17">
+        <f>(Na-E103)/(2*Nf)</f>
+        <v>1.5547159009766895</v>
+      </c>
+      <c r="K103" s="17">
+        <f>J103*tf</f>
+        <v>19.744891942403957</v>
+      </c>
+      <c r="L103" s="17">
+        <f>(E103*(td-tc/2*F103)+Na*Ht/2-(Na-F103*Nc)*K103/2)/1000</f>
+        <v>466.83354472480664</v>
+      </c>
+      <c r="M103" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E103,E103&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N103" s="17">
+        <f>(E103-Nw)/(2*Nr)</f>
+        <v>-3.2309871053598442</v>
+      </c>
+      <c r="O103" s="18">
+        <f>dw/2+N103*rr</f>
+        <v>91.142232103522815</v>
+      </c>
+      <c r="P103" s="13">
+        <f>MplaRd+E103*(td-F103*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E103)*O103/1000</f>
+        <v>418.66298151703421</v>
+      </c>
+      <c r="Q103" s="67" t="str">
+        <f>IF(Nw&gt;E103,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R103" s="17">
+        <f>E103/2/Nw</f>
+        <v>0.11714264899103354</v>
+      </c>
+      <c r="S103" s="13">
+        <f>R103*dw</f>
+        <v>34.978794988722619</v>
+      </c>
+      <c r="T103" s="13">
+        <f>MplaRd+E103*(Ht/2+td/2-F103*tc-S103/2)/1000</f>
+        <v>405.84592304236605</v>
+      </c>
+    </row>
+    <row r="104" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B104" s="3">
+        <f>Feuil1!C95</f>
+        <v>21</v>
+      </c>
+      <c r="C104" s="18">
+        <f>Feuil1!D95</f>
+        <v>10</v>
+      </c>
+      <c r="D104" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="E104" s="13">
+        <f>IF(D104=1,IF(C104&lt;=$D$43,0,C104*$G$36),IF(C104-$D$36&lt;$D$44,0,MIN((C104-$D$36-$D$44)*$G$37,(LL-C104)*$G$37)))</f>
+        <v>0</v>
+      </c>
+      <c r="F104" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G104" s="18">
+        <f>IF(I104=oui,L104,IF(M104=oui,P104,T104))</f>
+        <v>361.745</v>
+      </c>
+      <c r="I104" s="3" t="str">
+        <f>IF(Na-2*Nf&lt;=E104,oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="J104" s="17">
+        <f>(Na-E104)/(2*Nf)</f>
+        <v>1.6843269986653329</v>
+      </c>
+      <c r="K104" s="17">
+        <f>J104*tf</f>
+        <v>21.390952883049724</v>
+      </c>
+      <c r="L104" s="17">
+        <f>(E104*(td-tc/2*F104)+Na*Ht/2-(Na-F104*Nc)*K104/2)/1000</f>
+        <v>437.12531991961151</v>
+      </c>
+      <c r="M104" s="3" t="str">
+        <f>IF(AND(Na-2*Nf&gt;E104,E104&gt;=Nw),oui,non)</f>
+        <v>non</v>
+      </c>
+      <c r="N104" s="17">
+        <f>(E104-Nw)/(2*Nr)</f>
+        <v>-4.2195704181270575</v>
+      </c>
+      <c r="O104" s="18">
+        <f>dw/2+N104*rr</f>
+        <v>73.347732473712981</v>
+      </c>
+      <c r="P104" s="13">
+        <f>MplaRd+E104*(td-F104*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E104)*O104/1000</f>
+        <v>360.64064588328802</v>
+      </c>
+      <c r="Q104" s="67" t="str">
+        <f>IF(Nw&gt;E104,oui,non)</f>
+        <v>oui</v>
+      </c>
+      <c r="R104" s="17">
+        <f>E104/2/Nw</f>
+        <v>0</v>
+      </c>
+      <c r="S104" s="13">
+        <f>R104*dw</f>
+        <v>0</v>
+      </c>
+      <c r="T104" s="13">
+        <f>MplaRd+E104*(Ht/2+td/2-F104*tc-S104/2)/1000</f>
+        <v>361.745</v>
+      </c>
+    </row>
+    <row r="109" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="G109" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="110" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="G110" t="s">
+        <v>202</v>
+      </c>
+      <c r="I110" t="s">
+        <v>203</v>
+      </c>
+      <c r="K110" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="111" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="E111" s="3">
+        <f>B84</f>
+        <v>1</v>
+      </c>
+      <c r="F111" s="13">
+        <f>C84</f>
+        <v>0</v>
+      </c>
+      <c r="G111" s="18">
+        <f>Feuil1!Q75</f>
+        <v>-340.37214428976085</v>
+      </c>
+      <c r="H111" s="17">
+        <f>IF(G111&gt;0,G111/$G84,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I111" s="18">
+        <f>Feuil1!S75</f>
+        <v>-70.37214428976084</v>
+      </c>
+      <c r="J111" s="17">
+        <f>IF(I111&gt;0,I111/$G84,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K111" s="18">
+        <f>Feuil1!U75</f>
+        <v>-340.37214428976085</v>
+      </c>
+      <c r="L111" s="17">
+        <f>IF(K111&gt;0,K111/$G84,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="E112" s="3">
+        <f t="shared" ref="E112:F112" si="5">B85</f>
+        <v>2</v>
+      </c>
+      <c r="F112" s="13">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="G112" s="18">
+        <f>Feuil1!Q76</f>
+        <v>-286.21268314456569</v>
+      </c>
+      <c r="H112" s="17">
+        <f t="shared" ref="H112:H129" si="6">IF(G112&gt;0,G112/$G85,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I112" s="18">
+        <f>Feuil1!S76</f>
+        <v>112.78731685543431</v>
+      </c>
+      <c r="J112" s="17">
+        <f t="shared" ref="J112:J129" si="7">IF(I112&gt;0,I112/$G85,0)</f>
+        <v>0.31178680245873286</v>
+      </c>
+      <c r="K112" s="18">
+        <f>Feuil1!U76</f>
+        <v>-143.71268314456569</v>
+      </c>
+      <c r="L112" s="17">
+        <f t="shared" ref="L112:L129" si="8">IF(K112&gt;0,K112/$G85,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E113" s="3">
+        <f t="shared" ref="E113:F113" si="9">B86</f>
+        <v>3</v>
+      </c>
+      <c r="F113" s="13">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="G113" s="18">
+        <f>Feuil1!Q77</f>
+        <v>-235.96278557102391</v>
+      </c>
+      <c r="H113" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I113" s="18">
+        <f>Feuil1!S77</f>
+        <v>277.03721442897609</v>
+      </c>
+      <c r="J113" s="17">
+        <f t="shared" si="7"/>
+        <v>0.76583564231427137</v>
+      </c>
+      <c r="K113" s="18">
+        <f>Feuil1!U77</f>
+        <v>34.037214428976078</v>
+      </c>
+      <c r="L113" s="17">
+        <f t="shared" si="8"/>
+        <v>9.4091734312778549E-2</v>
+      </c>
+    </row>
+    <row r="114" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E114" s="3">
+        <f t="shared" ref="E114:F114" si="10">B87</f>
+        <v>4</v>
+      </c>
+      <c r="F114" s="13">
+        <f t="shared" si="10"/>
+        <v>1.5</v>
+      </c>
+      <c r="G114" s="18">
+        <f>Feuil1!Q78</f>
+        <v>-189.62245156913554</v>
+      </c>
+      <c r="H114" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I114" s="18">
+        <f>Feuil1!S78</f>
+        <v>422.37754843086446</v>
+      </c>
+      <c r="J114" s="17">
+        <f t="shared" si="7"/>
+        <v>1.1676112964404883</v>
+      </c>
+      <c r="K114" s="18">
+        <f>Feuil1!U78</f>
+        <v>192.87754843086446</v>
+      </c>
+      <c r="L114" s="17">
+        <f t="shared" si="8"/>
+        <v>0.53318649443907851</v>
+      </c>
+    </row>
+    <row r="115" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E115" s="3">
+        <f t="shared" ref="E115:F115" si="11">B88</f>
+        <v>5</v>
+      </c>
+      <c r="F115" s="13">
+        <f t="shared" si="11"/>
+        <v>2</v>
+      </c>
+      <c r="G115" s="18">
+        <f>Feuil1!Q79</f>
+        <v>-147.19168113890052</v>
+      </c>
+      <c r="H115" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I115" s="18">
+        <f>Feuil1!S79</f>
+        <v>548.80831886109945</v>
+      </c>
+      <c r="J115" s="17">
+        <f t="shared" si="7"/>
+        <v>1.4539371349002377</v>
+      </c>
+      <c r="K115" s="18">
+        <f>Feuil1!U79</f>
+        <v>332.80831886109945</v>
+      </c>
+      <c r="L115" s="17">
+        <f t="shared" si="8"/>
+        <v>0.8816964994263139</v>
+      </c>
+    </row>
+    <row r="116" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E116" s="3">
+        <f t="shared" ref="E116:F116" si="12">B89</f>
+        <v>6</v>
+      </c>
+      <c r="F116" s="13">
+        <f t="shared" si="12"/>
+        <v>2.5</v>
+      </c>
+      <c r="G116" s="18">
+        <f>Feuil1!Q80</f>
+        <v>-108.67047428031889</v>
+      </c>
+      <c r="H116" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I116" s="18">
+        <f>Feuil1!S80</f>
+        <v>656.3295257196811</v>
+      </c>
+      <c r="J116" s="17">
+        <f t="shared" si="7"/>
+        <v>1.5682385622298081</v>
+      </c>
+      <c r="K116" s="18">
+        <f>Feuil1!U80</f>
+        <v>453.8295257196811</v>
+      </c>
+      <c r="L116" s="17">
+        <f t="shared" si="8"/>
+        <v>1.0843835832795394</v>
+      </c>
+    </row>
+    <row r="117" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E117" s="3">
+        <f t="shared" ref="E117:F117" si="13">B90</f>
+        <v>7</v>
+      </c>
+      <c r="F117" s="13">
+        <f t="shared" si="13"/>
+        <v>3</v>
+      </c>
+      <c r="G117" s="18">
+        <f>Feuil1!Q81</f>
+        <v>-74.058830993390643</v>
+      </c>
+      <c r="H117" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I117" s="18">
+        <f>Feuil1!S81</f>
+        <v>744.94116900660936</v>
+      </c>
+      <c r="J117" s="17">
+        <f t="shared" si="7"/>
+        <v>1.6539071204016087</v>
+      </c>
+      <c r="K117" s="18">
+        <f>Feuil1!U81</f>
+        <v>555.94116900660936</v>
+      </c>
+      <c r="L117" s="17">
+        <f t="shared" si="8"/>
+        <v>1.2342921779589113</v>
+      </c>
+    </row>
+    <row r="118" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E118" s="3">
+        <f t="shared" ref="E118:F118" si="14">B91</f>
+        <v>8</v>
+      </c>
+      <c r="F118" s="13">
+        <f t="shared" si="14"/>
+        <v>3.5</v>
+      </c>
+      <c r="G118" s="18">
+        <f>Feuil1!Q82</f>
+        <v>-43.356751278115752</v>
+      </c>
+      <c r="H118" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I118" s="18">
+        <f>Feuil1!S82</f>
+        <v>814.64324872188422</v>
+      </c>
+      <c r="J118" s="17">
+        <f t="shared" si="7"/>
+        <v>1.7217044403359252</v>
+      </c>
+      <c r="K118" s="18">
+        <f>Feuil1!U82</f>
+        <v>639.14324872188422</v>
+      </c>
+      <c r="L118" s="17">
+        <f t="shared" si="8"/>
+        <v>1.3507946835153533</v>
+      </c>
+    </row>
+    <row r="119" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E119" s="3">
+        <f t="shared" ref="E119:F119" si="15">B92</f>
+        <v>9</v>
+      </c>
+      <c r="F119" s="13">
+        <f t="shared" si="15"/>
+        <v>4</v>
+      </c>
+      <c r="G119" s="18">
+        <f>Feuil1!Q83</f>
+        <v>-16.564235134494282</v>
+      </c>
+      <c r="H119" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I119" s="18">
+        <f>Feuil1!S83</f>
+        <v>865.43576486550569</v>
+      </c>
+      <c r="J119" s="17">
+        <f t="shared" si="7"/>
+        <v>1.5648287898116933</v>
+      </c>
+      <c r="K119" s="18">
+        <f>Feuil1!U83</f>
+        <v>703.43576486550569</v>
+      </c>
+      <c r="L119" s="17">
+        <f t="shared" si="8"/>
+        <v>1.2719101536274235</v>
+      </c>
+    </row>
+    <row r="120" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E120" s="3">
+        <f t="shared" ref="E120:F120" si="16">B93</f>
+        <v>10</v>
+      </c>
+      <c r="F120" s="13">
+        <f t="shared" si="16"/>
+        <v>4.5</v>
+      </c>
+      <c r="G120" s="18">
+        <f>Feuil1!Q84</f>
+        <v>6.318717437473822</v>
+      </c>
+      <c r="H120" s="17">
+        <f t="shared" si="6"/>
+        <v>1.0924322715763612E-2</v>
+      </c>
+      <c r="I120" s="18">
+        <f>Feuil1!S84</f>
+        <v>897.31871743747388</v>
+      </c>
+      <c r="J120" s="17">
+        <f t="shared" si="7"/>
+        <v>1.5513590131514212</v>
+      </c>
+      <c r="K120" s="18">
+        <f>Feuil1!U84</f>
+        <v>748.81871743747388</v>
+      </c>
+      <c r="L120" s="17">
+        <f t="shared" si="8"/>
+        <v>1.2946198980788115</v>
+      </c>
+    </row>
+    <row r="121" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E121" s="3">
+        <f t="shared" ref="E121:F121" si="17">B94</f>
+        <v>11</v>
+      </c>
+      <c r="F121" s="13">
+        <f t="shared" si="17"/>
+        <v>5</v>
+      </c>
+      <c r="G121" s="18">
+        <f>Feuil1!Q85</f>
+        <v>25.292106437788561</v>
+      </c>
+      <c r="H121" s="17">
+        <f t="shared" si="6"/>
+        <v>4.2139778043996684E-2</v>
+      </c>
+      <c r="I121" s="18">
+        <f>Feuil1!S85</f>
+        <v>910.29210643778856</v>
+      </c>
+      <c r="J121" s="17">
+        <f t="shared" si="7"/>
+        <v>1.5166592555208547</v>
+      </c>
+      <c r="K121" s="18">
+        <f>Feuil1!U85</f>
+        <v>775.29210643778856</v>
+      </c>
+      <c r="L121" s="17">
+        <f t="shared" si="8"/>
+        <v>1.2917325555667576</v>
+      </c>
+    </row>
+    <row r="122" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E122" s="3">
+        <f t="shared" ref="E122:F122" si="18">B95</f>
+        <v>12</v>
+      </c>
+      <c r="F122" s="13">
+        <f t="shared" si="18"/>
+        <v>5.5</v>
+      </c>
+      <c r="G122" s="18">
+        <f>Feuil1!Q86</f>
+        <v>40.355931866449907</v>
+      </c>
+      <c r="H122" s="17">
+        <f t="shared" si="6"/>
+        <v>6.5037999143746292E-2</v>
+      </c>
+      <c r="I122" s="18">
+        <f>Feuil1!S86</f>
+        <v>904.35593186644996</v>
+      </c>
+      <c r="J122" s="17">
+        <f t="shared" si="7"/>
+        <v>1.4574685207869096</v>
+      </c>
+      <c r="K122" s="18">
+        <f>Feuil1!U86</f>
+        <v>782.85593186644996</v>
+      </c>
+      <c r="L122" s="17">
+        <f t="shared" si="8"/>
+        <v>1.2616579786808397</v>
+      </c>
+    </row>
+    <row r="123" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E123" s="3">
+        <f t="shared" ref="E123:F123" si="19">B96</f>
+        <v>13</v>
+      </c>
+      <c r="F123" s="13">
+        <f t="shared" si="19"/>
+        <v>6</v>
+      </c>
+      <c r="G123" s="18">
+        <f>Feuil1!Q87</f>
+        <v>51.510193723457888</v>
+      </c>
+      <c r="H123" s="17">
+        <f t="shared" si="6"/>
+        <v>8.1348128469880418E-2</v>
+      </c>
+      <c r="I123" s="18">
+        <f>Feuil1!S87</f>
+        <v>879.51019372345786</v>
+      </c>
+      <c r="J123" s="17">
+        <f t="shared" si="7"/>
+        <v>1.3889776577757806</v>
+      </c>
+      <c r="K123" s="18">
+        <f>Feuil1!U87</f>
+        <v>771.51019372345786</v>
+      </c>
+      <c r="L123" s="17">
+        <f t="shared" si="8"/>
+        <v>1.2184172843880545</v>
+      </c>
+    </row>
+    <row r="124" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E124" s="3">
+        <f t="shared" ref="E124:F124" si="20">B97</f>
+        <v>14</v>
+      </c>
+      <c r="F124" s="13">
+        <f t="shared" si="20"/>
+        <v>6.5</v>
+      </c>
+      <c r="G124" s="18">
+        <f>Feuil1!Q88</f>
+        <v>58.754892008812476</v>
+      </c>
+      <c r="H124" s="17">
+        <f t="shared" si="6"/>
+        <v>9.5708419354080018E-2</v>
+      </c>
+      <c r="I124" s="18">
+        <f>Feuil1!S88</f>
+        <v>835.75489200881248</v>
+      </c>
+      <c r="J124" s="17">
+        <f t="shared" si="7"/>
+        <v>1.3613977823260401</v>
+      </c>
+      <c r="K124" s="18">
+        <f>Feuil1!U88</f>
+        <v>741.25489200881248</v>
+      </c>
+      <c r="L124" s="17">
+        <f t="shared" si="8"/>
+        <v>1.2074625895321531</v>
+      </c>
+    </row>
+    <row r="125" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E125" s="3">
+        <f>B98</f>
+        <v>15</v>
+      </c>
+      <c r="F125" s="13">
+        <f>C98</f>
+        <v>7</v>
+      </c>
+      <c r="G125" s="18">
+        <f>Feuil1!Q89</f>
+        <v>62.090026722513699</v>
+      </c>
+      <c r="H125" s="17">
+        <f>IF(G125&gt;0,G125/$G98,0)</f>
+        <v>0.10468774189632066</v>
+      </c>
+      <c r="I125" s="18">
+        <f>Feuil1!S89</f>
+        <v>773.0900267225137</v>
+      </c>
+      <c r="J125" s="17">
+        <f>IF(I125&gt;0,I125/$G98,0)</f>
+        <v>1.3034790521486443</v>
+      </c>
+      <c r="K125" s="18">
+        <f>Feuil1!U89</f>
+        <v>692.0900267225137</v>
+      </c>
+      <c r="L125" s="17">
+        <f>IF(K125&gt;0,K125/$G98,0)</f>
+        <v>1.1669078902211643</v>
+      </c>
+    </row>
+    <row r="126" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E126" s="3">
+        <f t="shared" ref="E126:E129" si="21">B99</f>
+        <v>16</v>
+      </c>
+      <c r="F126" s="13">
+        <f t="shared" ref="F126:F129" si="22">C99</f>
+        <v>7.5</v>
+      </c>
+      <c r="G126" s="18">
+        <f>Feuil1!Q90</f>
+        <v>61.515597864561528</v>
+      </c>
+      <c r="H126" s="17">
+        <f t="shared" si="6"/>
+        <v>0.10810484895720011</v>
+      </c>
+      <c r="I126" s="18">
+        <f>Feuil1!S90</f>
+        <v>691.51559786456153</v>
+      </c>
+      <c r="J126" s="17">
+        <f t="shared" si="7"/>
+        <v>1.2152395791273385</v>
+      </c>
+      <c r="K126" s="18">
+        <f>Feuil1!U90</f>
+        <v>624.01559786456153</v>
+      </c>
+      <c r="L126" s="17">
+        <f t="shared" si="8"/>
+        <v>1.0966180008948236</v>
+      </c>
+    </row>
+    <row r="127" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E127" s="3">
+        <f t="shared" si="21"/>
+        <v>17</v>
+      </c>
+      <c r="F127" s="13">
+        <f t="shared" si="22"/>
+        <v>8</v>
+      </c>
+      <c r="G127" s="18">
+        <f>Feuil1!Q91</f>
+        <v>57.031605434955978</v>
+      </c>
+      <c r="H127" s="17">
+        <f t="shared" si="6"/>
+        <v>0.11801875693717821</v>
+      </c>
+      <c r="I127" s="18">
+        <f>Feuil1!S91</f>
+        <v>591.03160543495596</v>
+      </c>
+      <c r="J127" s="17">
+        <f t="shared" si="7"/>
+        <v>1.2230554418386614</v>
+      </c>
+      <c r="K127" s="18">
+        <f>Feuil1!U91</f>
+        <v>537.03160543495596</v>
+      </c>
+      <c r="L127" s="17">
+        <f t="shared" si="8"/>
+        <v>1.1113101590958148</v>
+      </c>
+    </row>
+    <row r="128" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E128" s="3">
+        <f t="shared" si="21"/>
+        <v>18</v>
+      </c>
+      <c r="F128" s="13">
+        <f t="shared" si="22"/>
+        <v>8.5</v>
+      </c>
+      <c r="G128" s="18">
+        <f>Feuil1!Q92</f>
+        <v>48.638049433697063</v>
+      </c>
+      <c r="H128" s="17">
+        <f t="shared" si="6"/>
+        <v>0.10424054280510127</v>
+      </c>
+      <c r="I128" s="18">
+        <f>Feuil1!S92</f>
+        <v>471.63804943369706</v>
+      </c>
+      <c r="J128" s="17">
+        <f t="shared" si="7"/>
+        <v>1.010809579186094</v>
+      </c>
+      <c r="K128" s="18">
+        <f>Feuil1!U92</f>
+        <v>431.13804943369706</v>
+      </c>
+      <c r="L128" s="17">
+        <f t="shared" si="8"/>
+        <v>0.92401041612833945</v>
+      </c>
+    </row>
+    <row r="129" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E129" s="3">
+        <f t="shared" si="21"/>
+        <v>19</v>
+      </c>
+      <c r="F129" s="13">
+        <f t="shared" si="22"/>
+        <v>9</v>
+      </c>
+      <c r="G129" s="18">
+        <f>Feuil1!Q93</f>
+        <v>36.334929860784747</v>
+      </c>
+      <c r="H129" s="17">
+        <f t="shared" si="6"/>
+        <v>8.2430316448273755E-2</v>
+      </c>
+      <c r="I129" s="18">
+        <f>Feuil1!S93</f>
+        <v>333.33492986078477</v>
+      </c>
+      <c r="J129" s="17">
+        <f t="shared" si="7"/>
+        <v>0.75621182858928992</v>
+      </c>
+      <c r="K129" s="18">
+        <f>Feuil1!U93</f>
+        <v>306.33492986078477</v>
+      </c>
+      <c r="L129" s="17">
+        <f t="shared" si="8"/>
+        <v>0.69495896384919753</v>
+      </c>
+    </row>
+    <row r="130" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E130" s="3">
+        <f>B103</f>
+        <v>20</v>
+      </c>
+      <c r="F130" s="13">
+        <f>C103</f>
+        <v>9.5</v>
+      </c>
+      <c r="G130" s="18">
+        <f>Feuil1!Q94</f>
+        <v>20.122246716219067</v>
+      </c>
+      <c r="H130" s="17">
+        <f>IF(G130&gt;0,G130/$G103,0)</f>
+        <v>4.9581000014427924E-2</v>
+      </c>
+      <c r="I130" s="18">
+        <f>Feuil1!S94</f>
+        <v>176.12224671621908</v>
+      </c>
+      <c r="J130" s="17">
+        <f>IF(I130&gt;0,I130/$G103,0)</f>
+        <v>0.43396332626910178</v>
+      </c>
+      <c r="K130" s="18">
+        <f>Feuil1!U94</f>
+        <v>162.62224671621908</v>
+      </c>
+      <c r="L130" s="17">
+        <f>IF(K130&gt;0,K130/$G103,0)</f>
+        <v>0.40069947111244736</v>
+      </c>
+    </row>
+    <row r="131" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E131" s="3">
+        <f>B104</f>
+        <v>21</v>
+      </c>
+      <c r="F131" s="13">
+        <f>C104</f>
+        <v>10</v>
+      </c>
+      <c r="G131" s="18">
+        <f>Feuil1!Q95</f>
+        <v>0</v>
+      </c>
+      <c r="H131" s="17">
+        <f>IF(G131&gt;0,G131/$G104,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I131" s="18">
+        <f>Feuil1!S95</f>
+        <v>0</v>
+      </c>
+      <c r="J131" s="17">
+        <f>IF(I131&gt;0,I131/$G104,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K131" s="18">
+        <f>Feuil1!U95</f>
+        <v>0</v>
+      </c>
+      <c r="L131" s="17">
+        <f>IF(K131&gt;0,K131/$G104,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="H134" s="88">
+        <f>MAX(H111:H131)</f>
+        <v>0.11801875693717821</v>
+      </c>
+      <c r="J134" s="88">
+        <f>MAX(J111:J131)</f>
+        <v>1.7217044403359252</v>
+      </c>
+      <c r="L134" s="88">
+        <f>MAX(L111:L131)</f>
+        <v>1.3507946835153533</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Prepa MV et V1.00 B2
</commit_message>
<xml_diff>
--- a/Manuel Validation/CAS C05/TEST C05.xlsx
+++ b/Manuel Validation/CAS C05/TEST C05.xlsx
@@ -9,14 +9,15 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Général" sheetId="1" r:id="rId1"/>
     <sheet name="MNégatif" sheetId="5" r:id="rId2"/>
     <sheet name="Connexion" sheetId="2" r:id="rId3"/>
-    <sheet name="Feuil2" sheetId="3" r:id="rId4"/>
-    <sheet name="Feuil3" sheetId="4" r:id="rId5"/>
+    <sheet name="Arma Trans" sheetId="6" r:id="rId4"/>
+    <sheet name="Feuil2" sheetId="3" r:id="rId5"/>
+    <sheet name="Feuil3" sheetId="4" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="AireA">Général!$E$16</definedName>
@@ -24,29 +25,31 @@
     <definedName name="Av">Général!$E$20</definedName>
     <definedName name="Avmin">Général!$J$36</definedName>
     <definedName name="b">Général!$E$12</definedName>
-    <definedName name="bb">Général!$E$27</definedName>
+    <definedName name="bb">Général!$E$28</definedName>
     <definedName name="beff_1">Général!$O$4</definedName>
     <definedName name="beff_a">Général!$O$5</definedName>
     <definedName name="beff_B">Connexion!$M$61</definedName>
     <definedName name="beff_m">Connexion!$M$60</definedName>
-    <definedName name="bm">Général!$E$32</definedName>
-    <definedName name="bt">Général!$E$28</definedName>
-    <definedName name="c_z">Général!$E$41</definedName>
+    <definedName name="bm">Général!$E$33</definedName>
+    <definedName name="bt">Général!$E$29</definedName>
+    <definedName name="c_z">Général!$E$42</definedName>
     <definedName name="d">Général!$E$6</definedName>
     <definedName name="dsc">Connexion!$D$4</definedName>
     <definedName name="dw">Général!$E$19</definedName>
-    <definedName name="e_s">Général!$E$40</definedName>
-    <definedName name="ebac">Général!$E$26</definedName>
+    <definedName name="e_s">Général!$E$41</definedName>
+    <definedName name="ebac">Général!$E$27</definedName>
     <definedName name="Ecm">Général!$J$9</definedName>
     <definedName name="Eta">Général!$J$35</definedName>
     <definedName name="EtaV">MNégatif!$D$9</definedName>
     <definedName name="Ey">Général!$J$6</definedName>
+    <definedName name="Fcd">'Arma Trans'!$E$12</definedName>
     <definedName name="Fck">Général!$J$7</definedName>
     <definedName name="Fcm">Général!$J$10</definedName>
+    <definedName name="Fsd">'Arma Trans'!$E$18</definedName>
     <definedName name="Fsk">Général!$J$8</definedName>
     <definedName name="Fusc">Connexion!$D$6</definedName>
     <definedName name="Fy">Général!$J$4</definedName>
-    <definedName name="fybac">Général!$E$30</definedName>
+    <definedName name="fybac">Général!$E$31</definedName>
     <definedName name="g">Général!$J$28</definedName>
     <definedName name="GammaC">Général!$J$16</definedName>
     <definedName name="GammaG">Général!$J$20</definedName>
@@ -55,7 +58,7 @@
     <definedName name="GammaQ">Général!$J$21</definedName>
     <definedName name="GammaS">Général!$J$17</definedName>
     <definedName name="GammaV">Général!$J$18</definedName>
-    <definedName name="hbac">Général!$E$25</definedName>
+    <definedName name="hbac">Général!$E$26</definedName>
     <definedName name="hsc">Connexion!$D$5</definedName>
     <definedName name="Ht">Général!$E$11</definedName>
     <definedName name="hw">Général!$E$18</definedName>
@@ -69,7 +72,7 @@
     <definedName name="MplRd_1">Général!$O$19</definedName>
     <definedName name="MplRd_app">Général!$O$37</definedName>
     <definedName name="MplRdMoins">Général!$W$48</definedName>
-    <definedName name="mubac">Général!$E$31</definedName>
+    <definedName name="mubac">Général!$E$32</definedName>
     <definedName name="Na">Général!$O$15</definedName>
     <definedName name="Nc">Général!$O$14</definedName>
     <definedName name="Nf">Général!$O$29</definedName>
@@ -78,12 +81,13 @@
     <definedName name="NrV">MNégatif!$D$5</definedName>
     <definedName name="Ns">Général!$O$25</definedName>
     <definedName name="Nu">Général!$J$5</definedName>
+    <definedName name="Nuc">'Arma Trans'!$E$14</definedName>
     <definedName name="Nw">Général!$O$31</definedName>
     <definedName name="NwV">MNégatif!$D$6</definedName>
     <definedName name="oui">Général!$T$2</definedName>
     <definedName name="p_1">Général!$O$40</definedName>
     <definedName name="p_w">Général!$R$40</definedName>
-    <definedName name="PhiS">Général!$E$39</definedName>
+    <definedName name="PhiS">Général!$E$40</definedName>
     <definedName name="PRd_dp">Connexion!$D$12</definedName>
     <definedName name="PRda">Connexion!$D$10</definedName>
     <definedName name="PRdc">Connexion!$D$11</definedName>
@@ -94,12 +98,14 @@
     <definedName name="RhoA">Général!$J$26</definedName>
     <definedName name="RhoC">Général!$J$27</definedName>
     <definedName name="rr">Général!$E$15</definedName>
-    <definedName name="tbac">Général!$E$29</definedName>
-    <definedName name="tc">Général!$E$37</definedName>
-    <definedName name="td">Général!$E$36</definedName>
+    <definedName name="tbac">Général!$E$30</definedName>
+    <definedName name="tc">Général!$E$38</definedName>
+    <definedName name="td">Général!$E$37</definedName>
     <definedName name="tf">Général!$E$13</definedName>
+    <definedName name="ThetaRad">'Arma Trans'!$G$13</definedName>
     <definedName name="tw">Général!$E$14</definedName>
     <definedName name="VplRd">Général!$J$37</definedName>
+    <definedName name="Wel">Général!$E$22</definedName>
     <definedName name="Wpl">Général!$E$21</definedName>
     <definedName name="zANPmoins">MNégatif!$D$15</definedName>
     <definedName name="zn">Général!$O$17</definedName>
@@ -115,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="261">
   <si>
     <t>Portee principale</t>
   </si>
@@ -838,6 +844,66 @@
   </si>
   <si>
     <t>Flexion négative MV</t>
+  </si>
+  <si>
+    <t>Wel</t>
+  </si>
+  <si>
+    <t>MelaRd</t>
+  </si>
+  <si>
+    <t>hw/tw</t>
+  </si>
+  <si>
+    <t>72 E / Eta</t>
+  </si>
+  <si>
+    <t>à Mi travée</t>
+  </si>
+  <si>
+    <t>Flux de cisaillement</t>
+  </si>
+  <si>
+    <t>Flux par surface a-a</t>
+  </si>
+  <si>
+    <t>Contrainte de cisaillement</t>
+  </si>
+  <si>
+    <t>ksf</t>
+  </si>
+  <si>
+    <t>b0min</t>
+  </si>
+  <si>
+    <t>fcd</t>
+  </si>
+  <si>
+    <t>Theta</t>
+  </si>
+  <si>
+    <t>°</t>
+  </si>
+  <si>
+    <t>Tlim</t>
+  </si>
+  <si>
+    <t>rad</t>
+  </si>
+  <si>
+    <t>Asf/sf</t>
+  </si>
+  <si>
+    <t>Fsd</t>
+  </si>
+  <si>
+    <t>mm2/mm</t>
+  </si>
+  <si>
+    <t>cm2/m</t>
+  </si>
+  <si>
+    <t>à l'appui intermédiaire</t>
   </si>
 </sst>
 </file>
@@ -850,7 +916,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -901,8 +967,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -990,6 +1080,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1157,7 +1253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1398,6 +1494,38 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="15" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="15" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="15" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1430,7 +1558,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2110,7 +2237,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3291,6 +3417,15 @@
       <c r="N21" s="2"/>
     </row>
     <row r="22" spans="3:28" x14ac:dyDescent="0.25">
+      <c r="D22" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="E22" s="4">
+        <v>903.6</v>
+      </c>
+      <c r="F22" t="s">
+        <v>198</v>
+      </c>
       <c r="I22" s="2"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9" t="s">
@@ -3309,12 +3444,6 @@
       </c>
     </row>
     <row r="23" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C23" s="5"/>
-      <c r="D23" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
       <c r="I23" s="2"/>
       <c r="V23" s="2" t="s">
         <v>124</v>
@@ -3326,6 +3455,12 @@
       </c>
     </row>
     <row r="24" spans="3:28" x14ac:dyDescent="0.25">
+      <c r="C24" s="5"/>
+      <c r="D24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
       <c r="H24" s="5"/>
       <c r="I24" s="5" t="s">
         <v>100</v>
@@ -3355,15 +3490,6 @@
       </c>
     </row>
     <row r="25" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="D25" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E25" s="4">
-        <v>58</v>
-      </c>
-      <c r="F25" t="s">
-        <v>2</v>
-      </c>
       <c r="I25" s="2"/>
       <c r="N25" s="2" t="s">
         <v>55</v>
@@ -3378,10 +3504,10 @@
     </row>
     <row r="26" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D26" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E26" s="4">
-        <v>207</v>
+        <v>58</v>
       </c>
       <c r="F26" t="s">
         <v>2</v>
@@ -3411,10 +3537,10 @@
     </row>
     <row r="27" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D27" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E27" s="4">
-        <v>62</v>
+        <v>207</v>
       </c>
       <c r="F27" t="s">
         <v>2</v>
@@ -3440,23 +3566,23 @@
       </c>
       <c r="W27" s="64">
         <f>Connexion!D74</f>
-        <v>612.80229895647165</v>
+        <v>607.72195372052818</v>
       </c>
       <c r="X27" s="64">
         <f>Connexion!E74</f>
-        <v>622.75352907963065</v>
+        <v>627.62441396684608</v>
       </c>
       <c r="Y27" s="64">
         <f>Connexion!F74</f>
-        <v>637.15672339254934</v>
+        <v>641.81814793103706</v>
       </c>
     </row>
     <row r="28" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D28" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E28" s="4">
-        <v>101</v>
+        <v>62</v>
       </c>
       <c r="F28" t="s">
         <v>2</v>
@@ -3488,10 +3614,10 @@
     </row>
     <row r="29" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D29" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E29" s="4">
-        <v>0.75</v>
+        <v>101</v>
       </c>
       <c r="F29" t="s">
         <v>2</v>
@@ -3509,26 +3635,26 @@
       </c>
       <c r="W29" s="66">
         <f>W28/W27</f>
-        <v>0.10132146506017604</v>
+        <v>0.10216847744662341</v>
       </c>
       <c r="X29" s="66">
         <f t="shared" ref="X29:Y29" si="0">X28/X27</f>
-        <v>1.4617213133791662</v>
+        <v>1.4503771462368165</v>
       </c>
       <c r="Y29" s="66">
         <f t="shared" si="0"/>
-        <v>1.2286709111348983</v>
+        <v>1.2197472670258107</v>
       </c>
     </row>
     <row r="30" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D30" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E30" s="4">
-        <v>355</v>
+        <v>0.75</v>
       </c>
       <c r="F30" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="I30" s="2"/>
       <c r="N30" s="15" t="s">
@@ -3544,13 +3670,13 @@
     </row>
     <row r="31" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D31" s="2" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="E31" s="4">
-        <v>8.5299999999999994</v>
+        <v>355</v>
       </c>
       <c r="F31" t="s">
-        <v>97</v>
+        <v>17</v>
       </c>
       <c r="I31" s="2"/>
       <c r="N31" s="15" t="s">
@@ -3566,14 +3692,13 @@
     </row>
     <row r="32" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D32" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="E32" s="4">
-        <f>(bb+bt)/2</f>
-        <v>81.5</v>
+        <v>8.5299999999999994</v>
       </c>
       <c r="F32" t="s">
-        <v>2</v>
+        <v>97</v>
       </c>
       <c r="I32" s="2"/>
       <c r="U32" s="52" t="s">
@@ -3582,6 +3707,16 @@
       <c r="V32" s="51"/>
     </row>
     <row r="33" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="D33" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E33" s="4">
+        <f>(bb+bt)/2</f>
+        <v>81.5</v>
+      </c>
+      <c r="F33" t="s">
+        <v>2</v>
+      </c>
       <c r="H33" s="9"/>
       <c r="I33" s="9" t="s">
         <v>131</v>
@@ -3606,12 +3741,6 @@
       </c>
     </row>
     <row r="34" spans="3:25" x14ac:dyDescent="0.25">
-      <c r="C34" s="5"/>
-      <c r="D34" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
       <c r="N34" s="2" t="s">
         <v>68</v>
       </c>
@@ -3640,6 +3769,12 @@
       </c>
     </row>
     <row r="35" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="C35" s="5"/>
+      <c r="D35" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
       <c r="I35" s="2" t="s">
         <v>133</v>
       </c>
@@ -3670,15 +3805,6 @@
       </c>
     </row>
     <row r="36" spans="3:25" x14ac:dyDescent="0.25">
-      <c r="D36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E36" s="4">
-        <v>130</v>
-      </c>
-      <c r="F36" t="s">
-        <v>2</v>
-      </c>
       <c r="I36" s="2" t="s">
         <v>134</v>
       </c>
@@ -3703,11 +3829,10 @@
     </row>
     <row r="37" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D37" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E37" s="7">
-        <f>td-hbac</f>
-        <v>72</v>
+        <v>35</v>
+      </c>
+      <c r="E37" s="4">
+        <v>130</v>
       </c>
       <c r="F37" t="s">
         <v>2</v>
@@ -3747,7 +3872,14 @@
     </row>
     <row r="38" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D38" s="2" t="s">
-        <v>58</v>
+        <v>36</v>
+      </c>
+      <c r="E38" s="7">
+        <f>td-hbac</f>
+        <v>72</v>
+      </c>
+      <c r="F38" t="s">
+        <v>2</v>
       </c>
       <c r="V38" t="s">
         <v>108</v>
@@ -3767,13 +3899,14 @@
     </row>
     <row r="39" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D39" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E39" s="4">
-        <v>16</v>
-      </c>
-      <c r="F39" t="s">
-        <v>2</v>
+        <v>58</v>
+      </c>
+      <c r="I39" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="J39" s="98">
+        <f>hw/tw</f>
+        <v>41.825000000000003</v>
       </c>
       <c r="N39" s="15" t="s">
         <v>75</v>
@@ -3798,14 +3931,21 @@
       </c>
     </row>
     <row r="40" spans="3:25" x14ac:dyDescent="0.25">
-      <c r="D40" s="15" t="s">
-        <v>25</v>
+      <c r="D40" s="2" t="s">
+        <v>56</v>
       </c>
       <c r="E40" s="4">
-        <v>180</v>
+        <v>16</v>
       </c>
       <c r="F40" t="s">
         <v>2</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="J40" s="98">
+        <f>72*SQRT(235/Fy)/Eta</f>
+        <v>48.816990808009628</v>
       </c>
       <c r="N40" s="15" t="s">
         <v>74</v>
@@ -3824,10 +3964,10 @@
     </row>
     <row r="41" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D41" s="15" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="E41" s="4">
-        <v>20</v>
+        <v>180</v>
       </c>
       <c r="F41" t="s">
         <v>2</v>
@@ -3837,6 +3977,15 @@
       </c>
     </row>
     <row r="42" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="D42" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E42" s="4">
+        <v>20</v>
+      </c>
+      <c r="F42" t="s">
+        <v>2</v>
+      </c>
       <c r="N42" s="2" t="s">
         <v>51</v>
       </c>
@@ -5148,67 +5297,67 @@
       <c r="D75" s="18">
         <v>0</v>
       </c>
-      <c r="F75" s="18">
+      <c r="F75" s="99">
         <f t="shared" ref="F75:F95" si="18">-qG_1*La^2/2*(LL-D75)/LL+qG_1*(D75*(LL-D75))/2</f>
         <v>-29.62751428871173</v>
       </c>
-      <c r="G75" s="18">
+      <c r="G75" s="100">
         <f t="shared" ref="G75:G95" si="19">+qG_1*La^2/2/LL+qG_1/2*(LL-2*D75)</f>
         <v>35.882211749661977</v>
       </c>
-      <c r="H75" s="17">
+      <c r="H75" s="101">
         <f t="shared" ref="H75:H95" si="20">-qG_2*La^2/2*(LL-D75)/LL+qG_2*(D75*(LL-D75))/2</f>
         <v>-22.5</v>
       </c>
-      <c r="I75" s="17">
+      <c r="I75" s="101">
         <f t="shared" ref="I75:I95" si="21">+qG_2*La^2/2/LL+qG_2/2*(LL-2*D75)</f>
         <v>27.25</v>
       </c>
-      <c r="J75" s="17">
+      <c r="J75" s="101">
         <f t="shared" ref="J75:J95" si="22">-qQ*La^2/2*(LL-D75)/LL</f>
         <v>-180</v>
       </c>
-      <c r="K75" s="17">
+      <c r="K75" s="101">
         <f t="shared" ref="K75:K95" si="23">+qQ*La^2/2/LL</f>
         <v>18</v>
       </c>
-      <c r="L75" s="17">
+      <c r="L75" s="101">
         <f t="shared" ref="L75:L95" si="24">qQ*(D75*(LL-D75))/2</f>
         <v>0</v>
       </c>
-      <c r="M75" s="17">
+      <c r="M75" s="101">
         <f t="shared" ref="M75:M95" si="25">qQ/2*(LL-2*D75)</f>
         <v>200</v>
       </c>
-      <c r="N75" s="17">
+      <c r="N75" s="101">
         <f t="shared" ref="N75:N95" si="26">J75+L75</f>
         <v>-180</v>
       </c>
-      <c r="O75" s="17">
+      <c r="O75" s="102">
         <f t="shared" ref="O75:O95" si="27">K75+M75</f>
         <v>218</v>
       </c>
-      <c r="Q75" s="18">
+      <c r="Q75" s="99">
         <f t="shared" si="9"/>
         <v>-340.37214428976085</v>
       </c>
-      <c r="R75" s="18">
+      <c r="R75" s="100">
         <f t="shared" si="10"/>
         <v>112.22848586204367</v>
       </c>
-      <c r="S75" s="18">
+      <c r="S75" s="100">
         <f t="shared" si="11"/>
         <v>-70.37214428976084</v>
       </c>
-      <c r="T75" s="18">
+      <c r="T75" s="100">
         <f t="shared" si="12"/>
         <v>385.22848586204367</v>
       </c>
-      <c r="U75" s="18">
+      <c r="U75" s="100">
         <f t="shared" si="13"/>
         <v>-340.37214428976085</v>
       </c>
-      <c r="V75" s="18">
+      <c r="V75" s="103">
         <f t="shared" si="14"/>
         <v>412.22848586204367</v>
       </c>
@@ -6710,67 +6859,67 @@
         <f t="shared" si="29"/>
         <v>10</v>
       </c>
-      <c r="F95" s="18">
+      <c r="F95" s="99">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="G95" s="18">
+      <c r="G95" s="100">
         <f t="shared" si="19"/>
         <v>-29.956708891919632</v>
       </c>
-      <c r="H95" s="17">
+      <c r="H95" s="101">
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="I95" s="17">
+      <c r="I95" s="101">
         <f t="shared" si="21"/>
         <v>-22.75</v>
       </c>
-      <c r="J95" s="17">
+      <c r="J95" s="101">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="K95" s="17">
+      <c r="K95" s="101">
         <f t="shared" si="23"/>
         <v>18</v>
       </c>
-      <c r="L95" s="17">
+      <c r="L95" s="101">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="M95" s="17">
+      <c r="M95" s="101">
         <f t="shared" si="25"/>
         <v>-200</v>
       </c>
-      <c r="N95" s="17">
+      <c r="N95" s="101">
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-      <c r="O95" s="17">
+      <c r="O95" s="102">
         <f t="shared" si="27"/>
         <v>-182</v>
       </c>
-      <c r="Q95" s="18">
+      <c r="Q95" s="99">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="R95" s="18">
+      <c r="R95" s="100">
         <f t="shared" si="10"/>
         <v>-44.154057004091513</v>
       </c>
-      <c r="S95" s="18">
+      <c r="S95" s="100">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="T95" s="18">
+      <c r="T95" s="100">
         <f t="shared" si="12"/>
         <v>-371.1540570040915</v>
       </c>
-      <c r="U95" s="18">
+      <c r="U95" s="100">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="V95" s="18">
+      <c r="V95" s="103">
         <f t="shared" si="14"/>
         <v>-344.1540570040915</v>
       </c>
@@ -7138,11 +7287,11 @@
         <v>-6.35</v>
       </c>
       <c r="I15" s="24">
-        <f>ABS(H15+zANPmoins)</f>
+        <f t="shared" ref="I15:I20" si="0">ABS(H15+zANPmoins)</f>
         <v>42.679755048875002</v>
       </c>
       <c r="J15" s="25">
-        <f t="shared" ref="J15:J20" si="0">G15*I15/1000</f>
+        <f t="shared" ref="J15:J20" si="1">G15*I15/1000</f>
         <v>32.711684858435007</v>
       </c>
       <c r="K15" s="3"/>
@@ -7162,11 +7311,11 @@
         <v>-21.7</v>
       </c>
       <c r="I16" s="24">
-        <f>ABS(H16+zANPmoins)</f>
+        <f t="shared" si="0"/>
         <v>27.329755048875004</v>
       </c>
       <c r="J16" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.6893383016010728</v>
       </c>
       <c r="K16" s="3"/>
@@ -7186,11 +7335,11 @@
         <v>-39.864877524437503</v>
       </c>
       <c r="I17" s="24">
-        <f>ABS(H17+zANPmoins)</f>
+        <f t="shared" si="0"/>
         <v>9.1648775244375003</v>
       </c>
       <c r="J17" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.46719851754903841</v>
       </c>
       <c r="K17" s="3"/>
@@ -7210,11 +7359,11 @@
         <v>-189.16487752443751</v>
       </c>
       <c r="I18" s="24">
-        <f>ABS(H18+zANPmoins)</f>
+        <f t="shared" si="0"/>
         <v>140.13512247556253</v>
       </c>
       <c r="J18" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>109.23004679139397</v>
       </c>
       <c r="K18" s="3"/>
@@ -7234,11 +7383,11 @@
         <v>-338.3</v>
       </c>
       <c r="I19" s="24">
-        <f>ABS(H19+zANPmoins)</f>
+        <f t="shared" si="0"/>
         <v>289.27024495112499</v>
       </c>
       <c r="J19" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>28.465148987590656</v>
       </c>
       <c r="K19" s="3"/>
@@ -7258,11 +7407,11 @@
         <v>-353.65</v>
       </c>
       <c r="I20" s="24">
-        <f>ABS(H20+zANPmoins)</f>
+        <f t="shared" si="0"/>
         <v>304.62024495112496</v>
       </c>
       <c r="J20" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>233.47466364156497</v>
       </c>
       <c r="K20" s="3"/>
@@ -7669,13 +7818,13 @@
         <v>169</v>
       </c>
       <c r="D52" s="3">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="E52" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="F52" s="3">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="H52" s="63">
         <v>7</v>
@@ -7689,15 +7838,15 @@
       </c>
       <c r="D53" s="18">
         <f>($D$36-$D$43)*$G$36+(D52-$D$36-$D$44)*$G$37</f>
-        <v>2066.2673775738222</v>
+        <v>2106.0032886810118</v>
       </c>
       <c r="E53" s="18">
         <f t="shared" ref="E53:F53" si="0">($D$36-$D$43)*$G$36+(E52-$D$36-$D$44)*$G$37</f>
-        <v>1231.8132443228558</v>
+        <v>1271.5491554300445</v>
       </c>
       <c r="F53" s="18">
         <f t="shared" si="0"/>
-        <v>1351.0209776444224</v>
+        <v>1390.7568887516115</v>
       </c>
     </row>
     <row r="54" spans="3:15" x14ac:dyDescent="0.25">
@@ -7706,15 +7855,15 @@
       </c>
       <c r="D54" s="18">
         <f>(LL-D52)*$G$37</f>
-        <v>1152.3414221084781</v>
+        <v>1112.605511001289</v>
       </c>
       <c r="E54" s="18">
         <f>(LL-E52)*$G$37</f>
-        <v>1986.7955553594447</v>
+        <v>1947.059644252256</v>
       </c>
       <c r="F54" s="18">
         <f>(LL-F52)*$G$37</f>
-        <v>1867.5878220378781</v>
+        <v>1827.851910930689</v>
       </c>
     </row>
     <row r="55" spans="3:15" x14ac:dyDescent="0.25">
@@ -7723,15 +7872,15 @@
       </c>
       <c r="D55" s="18">
         <f>MIN(D53:D54)</f>
-        <v>1152.3414221084781</v>
+        <v>1112.605511001289</v>
       </c>
       <c r="E55" s="18">
         <f t="shared" ref="E55:F55" si="1">MIN(E53:E54)</f>
-        <v>1231.8132443228558</v>
+        <v>1271.5491554300445</v>
       </c>
       <c r="F55" s="18">
         <f t="shared" si="1"/>
-        <v>1351.0209776444224</v>
+        <v>1390.7568887516115</v>
       </c>
     </row>
     <row r="56" spans="3:15" x14ac:dyDescent="0.25">
@@ -7778,15 +7927,15 @@
       </c>
       <c r="D59" s="62">
         <f>D55/MIN($D$57:$D$58)</f>
-        <v>0.44631735238455267</v>
+        <v>0.43092709885405078</v>
       </c>
       <c r="E59" s="62">
         <f t="shared" ref="E59:F59" si="2">E55/MIN($D$57:$D$58)</f>
-        <v>0.47709785944555627</v>
+        <v>0.49248811297605799</v>
       </c>
       <c r="F59" s="62">
         <f t="shared" si="2"/>
-        <v>0.52326862003706165</v>
+        <v>0.53865887356756359</v>
       </c>
       <c r="L59" s="2" t="s">
         <v>210</v>
@@ -7897,15 +8046,15 @@
       </c>
       <c r="D67" s="14">
         <f>Nc*D59</f>
-        <v>1354.3500058109248</v>
+        <v>1307.6482814726169</v>
       </c>
       <c r="E67" s="14">
         <f>Nc*E59</f>
-        <v>1447.7534544875402</v>
+        <v>1494.4551788258477</v>
       </c>
       <c r="F67" s="14">
         <f>Nc*F59</f>
-        <v>1587.8586275024634</v>
+        <v>1634.5603518407715</v>
       </c>
     </row>
     <row r="69" spans="3:17" x14ac:dyDescent="0.25">
@@ -7931,15 +8080,15 @@
       </c>
       <c r="D71" s="24">
         <f>(Na-D67)/2/Nf</f>
-        <v>0.80079980114240246</v>
+        <v>0.8312662562294002</v>
       </c>
       <c r="E71" s="24">
         <f>(Na-E67)/2/Nf</f>
-        <v>0.7398668909684073</v>
+        <v>0.70940043588140989</v>
       </c>
       <c r="F71" s="24">
         <f>(Na-F67)/2/Nf</f>
-        <v>0.64846752570741462</v>
+        <v>0.61800107062041676</v>
       </c>
     </row>
     <row r="72" spans="3:17" x14ac:dyDescent="0.25">
@@ -7948,15 +8097,15 @@
       </c>
       <c r="D72" s="14">
         <f>D71*tf</f>
-        <v>10.17015747450851</v>
+        <v>10.557081454113382</v>
       </c>
       <c r="E72" s="14">
         <f>E71*tf</f>
-        <v>9.396309515298773</v>
+        <v>9.0093855356939052</v>
       </c>
       <c r="F72" s="14">
         <f>F71*tf</f>
-        <v>8.2355375764841643</v>
+        <v>7.8486135968792921</v>
       </c>
     </row>
     <row r="73" spans="3:17" x14ac:dyDescent="0.25">
@@ -7971,15 +8120,15 @@
       </c>
       <c r="D74" s="65">
         <f>(D67*(td-tc/2*D59)+Na*Ht/2-(Na-D59*Nc)*D72/2)/1000</f>
-        <v>612.80229895647165</v>
+        <v>607.72195372052818</v>
       </c>
       <c r="E74" s="65">
         <f>(E67*(td-tc/2*E59)+Na*Ht/2-(Na-E59*Nc)*E72/2)/1000</f>
-        <v>622.75352907963065</v>
+        <v>627.62441396684608</v>
       </c>
       <c r="F74" s="65">
         <f>(F67*(td-tc/2*F59)+Na*Ht/2-(Na-F59*Nc)*F72/2)/1000</f>
-        <v>637.15672339254934</v>
+        <v>641.81814793103706</v>
       </c>
     </row>
     <row r="75" spans="3:17" x14ac:dyDescent="0.25">
@@ -7991,6 +8140,18 @@
     <row r="76" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C76" s="2"/>
     </row>
+    <row r="77" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="O77" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="P77" s="69">
+        <f>Wel*Fy/GammaM0/1000</f>
+        <v>320.77800000000002</v>
+      </c>
+      <c r="Q77" t="s">
+        <v>200</v>
+      </c>
+    </row>
     <row r="78" spans="3:17" x14ac:dyDescent="0.25">
       <c r="O78" s="1" t="s">
         <v>199</v>
@@ -8108,7 +8269,7 @@
         <v>2</v>
       </c>
       <c r="E84" s="13">
-        <f>IF(D84=1,IF(C84&lt;=$D$43,0,C84*$G$36),IF(C84-$D$36&lt;$D$44,0,MIN((C84-$D$36-$D$44)*$G$37,(LL-C84)*$G$37)))</f>
+        <f t="shared" ref="E84:E104" si="3">IF(D84=1,IF(C84&lt;=$D$43,0,C84*$G$36),IF(C84-$D$36&lt;$D$44,0,MIN((C84-$D$36-$D$44)*$G$37,(LL-C84)*$G$37)))</f>
         <v>0</v>
       </c>
       <c r="F84" s="17">
@@ -8116,7 +8277,7 @@
         <v>0</v>
       </c>
       <c r="G84" s="18">
-        <f>IF(L84=oui,O84,IF(P84=oui,S84,W84))</f>
+        <f t="shared" ref="G84:G104" si="4">IF(L84=oui,O84,IF(P84=oui,S84,W84))</f>
         <v>361.745</v>
       </c>
       <c r="H84" s="17">
@@ -8124,51 +8285,51 @@
         <v>1.5</v>
       </c>
       <c r="L84" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E84,oui,non)</f>
+        <f t="shared" ref="L84:L104" si="5">IF(Na-2*Nf&lt;=E84,oui,non)</f>
         <v>non</v>
       </c>
       <c r="M84" s="17">
-        <f>(Na-E84)/(2*Nf)</f>
+        <f t="shared" ref="M84:M104" si="6">(Na-E84)/(2*Nf)</f>
         <v>1.6843269986653329</v>
       </c>
       <c r="N84" s="17">
-        <f>M84*tf</f>
+        <f t="shared" ref="N84:N104" si="7">M84*tf</f>
         <v>21.390952883049724</v>
       </c>
       <c r="O84" s="17">
-        <f>(E84*(td-tc/2*F84)+Na*Ht/2-(Na-F84*Nc)*N84/2)/1000</f>
+        <f t="shared" ref="O84:O104" si="8">(E84*(td-tc/2*F84)+Na*Ht/2-(Na-F84*Nc)*N84/2)/1000</f>
         <v>437.12531991961151</v>
       </c>
       <c r="P84" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E84,E84&gt;=Nw),oui,non)</f>
+        <f t="shared" ref="P84:P104" si="9">IF(AND(Na-2*Nf&gt;E84,E84&gt;=Nw),oui,non)</f>
         <v>non</v>
       </c>
       <c r="Q84" s="17">
-        <f>(E84-Nw)/(2*Nr)</f>
+        <f t="shared" ref="Q84:Q104" si="10">(E84-Nw)/(2*Nr)</f>
         <v>-4.2195704181270575</v>
       </c>
       <c r="R84" s="18">
-        <f>dw/2+Q84*rr</f>
+        <f t="shared" ref="R84:R104" si="11">dw/2+Q84*rr</f>
         <v>73.347732473712981</v>
       </c>
       <c r="S84" s="13">
-        <f>MplaRd+E84*(td-F84*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E84)*R84/1000</f>
+        <f t="shared" ref="S84:S104" si="12">MplaRd+E84*(td-F84*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E84)*R84/1000</f>
         <v>360.64064588328802</v>
       </c>
       <c r="T84" s="68" t="str">
-        <f>IF(Nw&gt;E84,oui,non)</f>
+        <f t="shared" ref="T84:T104" si="13">IF(Nw&gt;E84,oui,non)</f>
         <v>oui</v>
       </c>
       <c r="U84" s="17">
-        <f>E84/2/Nw</f>
+        <f t="shared" ref="U84:U104" si="14">E84/2/Nw</f>
         <v>0</v>
       </c>
       <c r="V84" s="13">
-        <f>U84*dw</f>
+        <f t="shared" ref="V84:V104" si="15">U84*dw</f>
         <v>0</v>
       </c>
       <c r="W84" s="13">
-        <f>MplaRd+E84*(Ht/2+td-F84*tc/2-V84/2)/1000</f>
+        <f t="shared" ref="W84:W104" si="16">MplaRd+E84*(Ht/2+td-F84*tc/2-V84/2)/1000</f>
         <v>361.745</v>
       </c>
     </row>
@@ -8182,71 +8343,71 @@
         <v>0.5</v>
       </c>
       <c r="D85" s="3">
-        <f t="shared" ref="D85:D104" si="3">IF(C85&lt;$D$36,1,2)</f>
+        <f t="shared" ref="D85:D104" si="17">IF(C85&lt;$D$36,1,2)</f>
         <v>2</v>
       </c>
       <c r="E85" s="13">
-        <f>IF(D85=1,IF(C85&lt;=$D$43,0,C85*$G$36),IF(C85-$D$36&lt;$D$44,0,MIN((C85-$D$36-$D$44)*$G$37,(LL-C85)*$G$37)))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F85" s="17">
-        <f t="shared" ref="F85:F104" si="4">E85/MIN($D$57:$D$58)</f>
+        <f t="shared" ref="F85:F104" si="18">E85/MIN($D$57:$D$58)</f>
         <v>0</v>
       </c>
       <c r="G85" s="18">
-        <f>IF(L85=oui,O85,IF(P85=oui,S85,W85))</f>
+        <f t="shared" si="4"/>
         <v>361.745</v>
       </c>
       <c r="H85" s="17">
-        <f>IF(C85/LL&lt;0.25,beff_a+(beff_m-beff_a)*C85/LL/0.25,IF((LL-C85)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C85)/LL/0.25,beff_m))</f>
+        <f t="shared" ref="H85:H104" si="19">IF(C85/LL&lt;0.25,beff_a+(beff_m-beff_a)*C85/LL/0.25,IF((LL-C85)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C85)/LL/0.25,beff_m))</f>
         <v>1.625</v>
       </c>
       <c r="L85" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E85,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M85" s="17">
-        <f>(Na-E85)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.6843269986653329</v>
       </c>
       <c r="N85" s="17">
-        <f>M85*tf</f>
+        <f t="shared" si="7"/>
         <v>21.390952883049724</v>
       </c>
       <c r="O85" s="17">
-        <f>(E85*(td-tc/2*F85)+Na*Ht/2-(Na-F85*Nc)*N85/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>437.12531991961151</v>
       </c>
       <c r="P85" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E85,E85&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q85" s="17">
-        <f>(E85-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-4.2195704181270575</v>
       </c>
       <c r="R85" s="18">
-        <f>dw/2+Q85*rr</f>
+        <f t="shared" si="11"/>
         <v>73.347732473712981</v>
       </c>
       <c r="S85" s="13">
-        <f>MplaRd+E85*(td-F85*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E85)*R85/1000</f>
+        <f t="shared" si="12"/>
         <v>360.64064588328802</v>
       </c>
       <c r="T85" s="68" t="str">
-        <f>IF(Nw&gt;E85,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U85" s="17">
-        <f>E85/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="V85" s="13">
-        <f>U85*dw</f>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W85" s="13">
-        <f>MplaRd+E85*(Ht/2+td-F85*tc/2-V85/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>361.745</v>
       </c>
     </row>
@@ -8260,71 +8421,71 @@
         <v>1</v>
       </c>
       <c r="D86" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E86" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E86" s="13">
-        <f>IF(D86=1,IF(C86&lt;=$D$43,0,C86*$G$36),IF(C86-$D$36&lt;$D$44,0,MIN((C86-$D$36-$D$44)*$G$37,(LL-C86)*$G$37)))</f>
         <v>0</v>
       </c>
       <c r="F86" s="17">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="G86" s="18">
         <f t="shared" si="4"/>
+        <v>361.745</v>
+      </c>
+      <c r="H86" s="17">
+        <f t="shared" si="19"/>
+        <v>1.75</v>
+      </c>
+      <c r="L86" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>non</v>
+      </c>
+      <c r="M86" s="17">
+        <f t="shared" si="6"/>
+        <v>1.6843269986653329</v>
+      </c>
+      <c r="N86" s="17">
+        <f t="shared" si="7"/>
+        <v>21.390952883049724</v>
+      </c>
+      <c r="O86" s="17">
+        <f t="shared" si="8"/>
+        <v>437.12531991961151</v>
+      </c>
+      <c r="P86" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v>non</v>
+      </c>
+      <c r="Q86" s="17">
+        <f t="shared" si="10"/>
+        <v>-4.2195704181270575</v>
+      </c>
+      <c r="R86" s="18">
+        <f t="shared" si="11"/>
+        <v>73.347732473712981</v>
+      </c>
+      <c r="S86" s="13">
+        <f t="shared" si="12"/>
+        <v>360.64064588328802</v>
+      </c>
+      <c r="T86" s="68" t="str">
+        <f t="shared" si="13"/>
+        <v>oui</v>
+      </c>
+      <c r="U86" s="17">
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="G86" s="18">
-        <f>IF(L86=oui,O86,IF(P86=oui,S86,W86))</f>
-        <v>361.745</v>
-      </c>
-      <c r="H86" s="17">
-        <f>IF(C86/LL&lt;0.25,beff_a+(beff_m-beff_a)*C86/LL/0.25,IF((LL-C86)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C86)/LL/0.25,beff_m))</f>
-        <v>1.75</v>
-      </c>
-      <c r="L86" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E86,oui,non)</f>
-        <v>non</v>
-      </c>
-      <c r="M86" s="17">
-        <f>(Na-E86)/(2*Nf)</f>
-        <v>1.6843269986653329</v>
-      </c>
-      <c r="N86" s="17">
-        <f>M86*tf</f>
-        <v>21.390952883049724</v>
-      </c>
-      <c r="O86" s="17">
-        <f>(E86*(td-tc/2*F86)+Na*Ht/2-(Na-F86*Nc)*N86/2)/1000</f>
-        <v>437.12531991961151</v>
-      </c>
-      <c r="P86" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E86,E86&gt;=Nw),oui,non)</f>
-        <v>non</v>
-      </c>
-      <c r="Q86" s="17">
-        <f>(E86-Nw)/(2*Nr)</f>
-        <v>-4.2195704181270575</v>
-      </c>
-      <c r="R86" s="18">
-        <f>dw/2+Q86*rr</f>
-        <v>73.347732473712981</v>
-      </c>
-      <c r="S86" s="13">
-        <f>MplaRd+E86*(td-F86*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E86)*R86/1000</f>
-        <v>360.64064588328802</v>
-      </c>
-      <c r="T86" s="68" t="str">
-        <f>IF(Nw&gt;E86,oui,non)</f>
-        <v>oui</v>
-      </c>
-      <c r="U86" s="17">
-        <f>E86/2/Nw</f>
+      <c r="V86" s="13">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="V86" s="13">
-        <f>U86*dw</f>
-        <v>0</v>
-      </c>
       <c r="W86" s="13">
-        <f>MplaRd+E86*(Ht/2+td-F86*tc/2-V86/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>361.745</v>
       </c>
     </row>
@@ -8338,71 +8499,71 @@
         <v>1.5</v>
       </c>
       <c r="D87" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E87" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E87" s="13">
-        <f>IF(D87=1,IF(C87&lt;=$D$43,0,C87*$G$36),IF(C87-$D$36&lt;$D$44,0,MIN((C87-$D$36-$D$44)*$G$37,(LL-C87)*$G$37)))</f>
         <v>0</v>
       </c>
       <c r="F87" s="17">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="G87" s="18">
         <f t="shared" si="4"/>
+        <v>361.745</v>
+      </c>
+      <c r="H87" s="17">
+        <f t="shared" si="19"/>
+        <v>1.875</v>
+      </c>
+      <c r="L87" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>non</v>
+      </c>
+      <c r="M87" s="17">
+        <f t="shared" si="6"/>
+        <v>1.6843269986653329</v>
+      </c>
+      <c r="N87" s="17">
+        <f t="shared" si="7"/>
+        <v>21.390952883049724</v>
+      </c>
+      <c r="O87" s="17">
+        <f t="shared" si="8"/>
+        <v>437.12531991961151</v>
+      </c>
+      <c r="P87" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v>non</v>
+      </c>
+      <c r="Q87" s="17">
+        <f t="shared" si="10"/>
+        <v>-4.2195704181270575</v>
+      </c>
+      <c r="R87" s="18">
+        <f t="shared" si="11"/>
+        <v>73.347732473712981</v>
+      </c>
+      <c r="S87" s="13">
+        <f t="shared" si="12"/>
+        <v>360.64064588328802</v>
+      </c>
+      <c r="T87" s="68" t="str">
+        <f t="shared" si="13"/>
+        <v>oui</v>
+      </c>
+      <c r="U87" s="17">
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="G87" s="18">
-        <f>IF(L87=oui,O87,IF(P87=oui,S87,W87))</f>
-        <v>361.745</v>
-      </c>
-      <c r="H87" s="17">
-        <f>IF(C87/LL&lt;0.25,beff_a+(beff_m-beff_a)*C87/LL/0.25,IF((LL-C87)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C87)/LL/0.25,beff_m))</f>
-        <v>1.875</v>
-      </c>
-      <c r="L87" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E87,oui,non)</f>
-        <v>non</v>
-      </c>
-      <c r="M87" s="17">
-        <f>(Na-E87)/(2*Nf)</f>
-        <v>1.6843269986653329</v>
-      </c>
-      <c r="N87" s="17">
-        <f>M87*tf</f>
-        <v>21.390952883049724</v>
-      </c>
-      <c r="O87" s="17">
-        <f>(E87*(td-tc/2*F87)+Na*Ht/2-(Na-F87*Nc)*N87/2)/1000</f>
-        <v>437.12531991961151</v>
-      </c>
-      <c r="P87" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E87,E87&gt;=Nw),oui,non)</f>
-        <v>non</v>
-      </c>
-      <c r="Q87" s="17">
-        <f>(E87-Nw)/(2*Nr)</f>
-        <v>-4.2195704181270575</v>
-      </c>
-      <c r="R87" s="18">
-        <f>dw/2+Q87*rr</f>
-        <v>73.347732473712981</v>
-      </c>
-      <c r="S87" s="13">
-        <f>MplaRd+E87*(td-F87*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E87)*R87/1000</f>
-        <v>360.64064588328802</v>
-      </c>
-      <c r="T87" s="68" t="str">
-        <f>IF(Nw&gt;E87,oui,non)</f>
-        <v>oui</v>
-      </c>
-      <c r="U87" s="17">
-        <f>E87/2/Nw</f>
+      <c r="V87" s="13">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="V87" s="13">
-        <f>U87*dw</f>
-        <v>0</v>
-      </c>
       <c r="W87" s="13">
-        <f>MplaRd+E87*(Ht/2+td-F87*tc/2-V87/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>361.745</v>
       </c>
     </row>
@@ -8416,71 +8577,71 @@
         <v>2</v>
       </c>
       <c r="D88" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E88" s="13">
         <f t="shared" si="3"/>
+        <v>39.735911107188933</v>
+      </c>
+      <c r="F88" s="17">
+        <f t="shared" si="18"/>
+        <v>1.539025353050183E-2</v>
+      </c>
+      <c r="G88" s="18">
+        <f t="shared" si="4"/>
+        <v>373.90212536753432</v>
+      </c>
+      <c r="H88" s="17">
+        <f t="shared" si="19"/>
         <v>2</v>
       </c>
-      <c r="E88" s="13">
-        <f>IF(D88=1,IF(C88&lt;=$D$43,0,C88*$G$36),IF(C88-$D$36&lt;$D$44,0,MIN((C88-$D$36-$D$44)*$G$37,(LL-C88)*$G$37)))</f>
-        <v>39.735911107188933</v>
-      </c>
-      <c r="F88" s="17">
-        <f t="shared" si="4"/>
-        <v>1.539025353050183E-2</v>
-      </c>
-      <c r="G88" s="18">
-        <f>IF(L88=oui,O88,IF(P88=oui,S88,W88))</f>
-        <v>373.90212536753432</v>
-      </c>
-      <c r="H88" s="17">
-        <f>IF(C88/LL&lt;0.25,beff_a+(beff_m-beff_a)*C88/LL/0.25,IF((LL-C88)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C88)/LL/0.25,beff_m))</f>
-        <v>2</v>
-      </c>
       <c r="L88" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E88,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M88" s="17">
-        <f>(Na-E88)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.6584047791276044</v>
       </c>
       <c r="N88" s="17">
-        <f>M88*tf</f>
+        <f t="shared" si="7"/>
         <v>21.061740694920577</v>
       </c>
       <c r="O88" s="17">
-        <f>(E88*(td-tc/2*F88)+Na*Ht/2-(Na-F88*Nc)*N88/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>443.18577702182176</v>
       </c>
       <c r="P88" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E88,E88&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q88" s="17">
-        <f>(E88-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-4.0218537555736145</v>
       </c>
       <c r="R88" s="18">
-        <f>dw/2+Q88*rr</f>
+        <f t="shared" si="11"/>
         <v>76.906632399674947</v>
       </c>
       <c r="S88" s="13">
-        <f>MplaRd+E88*(td-F88*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E88)*R88/1000</f>
+        <f t="shared" si="12"/>
         <v>372.89884012188043</v>
       </c>
       <c r="T88" s="68" t="str">
-        <f>IF(Nw&gt;E88,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U88" s="17">
-        <f>E88/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>2.342852979820673E-2</v>
       </c>
       <c r="V88" s="13">
-        <f>U88*dw</f>
+        <f t="shared" si="15"/>
         <v>6.99575899774453</v>
       </c>
       <c r="W88" s="13">
-        <f>MplaRd+E88*(Ht/2+td-F88*tc/2-V88/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>373.90212536753432</v>
       </c>
     </row>
@@ -8494,71 +8655,71 @@
         <v>2.5</v>
       </c>
       <c r="D89" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E89" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E89" s="13">
-        <f>IF(D89=1,IF(C89&lt;=$D$43,0,C89*$G$36),IF(C89-$D$36&lt;$D$44,0,MIN((C89-$D$36-$D$44)*$G$37,(LL-C89)*$G$37)))</f>
         <v>238.41546664313341</v>
       </c>
       <c r="F89" s="17">
+        <f t="shared" si="18"/>
+        <v>9.2341521183010908E-2</v>
+      </c>
+      <c r="G89" s="18">
         <f t="shared" si="4"/>
-        <v>9.2341521183010908E-2</v>
-      </c>
-      <c r="G89" s="18">
-        <f>IF(L89=oui,O89,IF(P89=oui,S89,W89))</f>
         <v>429.85753993437902</v>
       </c>
       <c r="H89" s="17">
-        <f>IF(C89/LL&lt;0.25,beff_a+(beff_m-beff_a)*C89/LL/0.25,IF((LL-C89)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C89)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L89" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E89,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M89" s="17">
-        <f>(Na-E89)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.5287936814389607</v>
       </c>
       <c r="N89" s="17">
-        <f>M89*tf</f>
+        <f t="shared" si="7"/>
         <v>19.415679754274798</v>
       </c>
       <c r="O89" s="17">
-        <f>(E89*(td-tc/2*F89)+Na*Ht/2-(Na-F89*Nc)*N89/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>472.59697147408883</v>
       </c>
       <c r="P89" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E89,E89&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q89" s="17">
-        <f>(E89-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-3.0332704428064017</v>
       </c>
       <c r="R89" s="18">
-        <f>dw/2+Q89*rr</f>
+        <f t="shared" si="11"/>
         <v>94.701132029484782</v>
       </c>
       <c r="S89" s="13">
-        <f>MplaRd+E89*(td-F89*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E89)*R89/1000</f>
+        <f t="shared" si="12"/>
         <v>429.28685797601872</v>
       </c>
       <c r="T89" s="68" t="str">
-        <f>IF(Nw&gt;E89,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U89" s="17">
-        <f>E89/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.14057117878924028</v>
       </c>
       <c r="V89" s="13">
-        <f>U89*dw</f>
+        <f t="shared" si="15"/>
         <v>41.97455398646715</v>
       </c>
       <c r="W89" s="13">
-        <f>MplaRd+E89*(Ht/2+td-F89*tc/2-V89/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>429.85753993437902</v>
       </c>
     </row>
@@ -8572,71 +8733,71 @@
         <v>3</v>
       </c>
       <c r="D90" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E90" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E90" s="13">
-        <f>IF(D90=1,IF(C90&lt;=$D$43,0,C90*$G$36),IF(C90-$D$36&lt;$D$44,0,MIN((C90-$D$36-$D$44)*$G$37,(LL-C90)*$G$37)))</f>
         <v>437.09502217907789</v>
       </c>
       <c r="F90" s="17">
+        <f t="shared" si="18"/>
+        <v>0.16929278883551999</v>
+      </c>
+      <c r="G90" s="18">
         <f t="shared" si="4"/>
-        <v>0.16929278883551999</v>
-      </c>
-      <c r="G90" s="18">
-        <f>IF(L90=oui,O90,IF(P90=oui,S90,W90))</f>
         <v>477.76260071651222</v>
       </c>
       <c r="H90" s="17">
-        <f>IF(C90/LL&lt;0.25,beff_a+(beff_m-beff_a)*C90/LL/0.25,IF((LL-C90)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C90)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L90" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E90,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M90" s="17">
-        <f>(Na-E90)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.3991825837503176</v>
       </c>
       <c r="N90" s="17">
-        <f>M90*tf</f>
+        <f t="shared" si="7"/>
         <v>17.769618813629034</v>
       </c>
       <c r="O90" s="17">
-        <f>(E90*(td-tc/2*F90)+Na*Ht/2-(Na-F90*Nc)*N90/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>500.52301416171628</v>
       </c>
       <c r="P90" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E90,E90&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q90" s="17">
-        <f>(E90-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-2.0446871300391884</v>
       </c>
       <c r="R90" s="18">
-        <f>dw/2+Q90*rr</f>
+        <f t="shared" si="11"/>
         <v>112.49563165929462</v>
       </c>
       <c r="S90" s="13">
-        <f>MplaRd+E90*(td-F90*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E90)*R90/1000</f>
+        <f t="shared" si="12"/>
         <v>477.50328693211753</v>
       </c>
       <c r="T90" s="68" t="str">
-        <f>IF(Nw&gt;E90,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U90" s="17">
-        <f>E90/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.2577138277802738</v>
       </c>
       <c r="V90" s="13">
-        <f>U90*dw</f>
+        <f t="shared" si="15"/>
         <v>76.953348975189755</v>
       </c>
       <c r="W90" s="13">
-        <f>MplaRd+E90*(Ht/2+td-F90*tc/2-V90/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>477.76260071651222</v>
       </c>
     </row>
@@ -8650,71 +8811,71 @@
         <v>3.5</v>
       </c>
       <c r="D91" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E91" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E91" s="13">
-        <f>IF(D91=1,IF(C91&lt;=$D$43,0,C91*$G$36),IF(C91-$D$36&lt;$D$44,0,MIN((C91-$D$36-$D$44)*$G$37,(LL-C91)*$G$37)))</f>
         <v>635.77457771502236</v>
       </c>
       <c r="F91" s="17">
+        <f t="shared" si="18"/>
+        <v>0.24624405648802905</v>
+      </c>
+      <c r="G91" s="18">
         <f t="shared" si="4"/>
-        <v>0.24624405648802905</v>
-      </c>
-      <c r="G91" s="18">
-        <f>IF(L91=oui,O91,IF(P91=oui,S91,W91))</f>
         <v>517.61730771393377</v>
       </c>
       <c r="H91" s="17">
-        <f>IF(C91/LL&lt;0.25,beff_a+(beff_m-beff_a)*C91/LL/0.25,IF((LL-C91)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C91)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L91" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E91,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M91" s="17">
-        <f>(Na-E91)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.2695714860616742</v>
       </c>
       <c r="N91" s="17">
-        <f>M91*tf</f>
+        <f t="shared" si="7"/>
         <v>16.123557872983262</v>
       </c>
       <c r="O91" s="17">
-        <f>(E91*(td-tc/2*F91)+Na*Ht/2-(Na-F91*Nc)*N91/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>526.96390508470404</v>
       </c>
       <c r="P91" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E91,E91&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q91" s="17">
-        <f>(E91-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-1.0561038172719757</v>
       </c>
       <c r="R91" s="18">
-        <f>dw/2+Q91*rr</f>
+        <f t="shared" si="11"/>
         <v>130.29013128910447</v>
       </c>
       <c r="S91" s="13">
-        <f>MplaRd+E91*(td-F91*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E91)*R91/1000</f>
+        <f t="shared" si="12"/>
         <v>517.54812699017691</v>
       </c>
       <c r="T91" s="68" t="str">
-        <f>IF(Nw&gt;E91,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U91" s="17">
-        <f>E91/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.37485647677130735</v>
       </c>
       <c r="V91" s="13">
-        <f>U91*dw</f>
+        <f t="shared" si="15"/>
         <v>111.93214396391238</v>
       </c>
       <c r="W91" s="13">
-        <f>MplaRd+E91*(Ht/2+td-F91*tc/2-V91/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>517.61730771393377</v>
       </c>
       <c r="X91">
@@ -8732,71 +8893,71 @@
         <v>4</v>
       </c>
       <c r="D92" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E92" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E92" s="13">
-        <f>IF(D92=1,IF(C92&lt;=$D$43,0,C92*$G$36),IF(C92-$D$36&lt;$D$44,0,MIN((C92-$D$36-$D$44)*$G$37,(LL-C92)*$G$37)))</f>
         <v>834.45413325096683</v>
       </c>
       <c r="F92" s="17">
+        <f t="shared" si="18"/>
+        <v>0.32319532414053814</v>
+      </c>
+      <c r="G92" s="18">
         <f t="shared" si="4"/>
-        <v>0.32319532414053814</v>
-      </c>
-      <c r="G92" s="18">
-        <f>IF(L92=oui,O92,IF(P92=oui,S92,W92))</f>
         <v>549.42166092664388</v>
       </c>
       <c r="H92" s="17">
-        <f>IF(C92/LL&lt;0.25,beff_a+(beff_m-beff_a)*C92/LL/0.25,IF((LL-C92)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C92)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L92" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E92,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M92" s="17">
-        <f>(Na-E92)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.1399603883730309</v>
       </c>
       <c r="N92" s="17">
-        <f>M92*tf</f>
+        <f t="shared" si="7"/>
         <v>14.477496932337491</v>
       </c>
       <c r="O92" s="17">
-        <f>(E92*(td-tc/2*F92)+Na*Ht/2-(Na-F92*Nc)*N92/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>551.91964424305206</v>
       </c>
       <c r="P92" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E92,E92&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q92" s="17">
-        <f>(E92-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-6.7520504504762602E-2</v>
       </c>
       <c r="R92" s="18">
-        <f>dw/2+Q92*rr</f>
+        <f t="shared" si="11"/>
         <v>148.08463091891429</v>
       </c>
       <c r="S92" s="13">
-        <f>MplaRd+E92*(td-F92*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E92)*R92/1000</f>
+        <f t="shared" si="12"/>
         <v>549.42137815019669</v>
       </c>
       <c r="T92" s="68" t="str">
-        <f>IF(Nw&gt;E92,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U92" s="17">
-        <f>E92/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.49199912576234089</v>
       </c>
       <c r="V92" s="13">
-        <f>U92*dw</f>
+        <f t="shared" si="15"/>
         <v>146.91093895263501</v>
       </c>
       <c r="W92" s="13">
-        <f>MplaRd+E92*(Ht/2+td-F92*tc/2-V92/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>549.42166092664388</v>
       </c>
     </row>
@@ -8810,71 +8971,71 @@
         <v>4.5</v>
       </c>
       <c r="D93" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E93" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E93" s="13">
-        <f>IF(D93=1,IF(C93&lt;=$D$43,0,C93*$G$36),IF(C93-$D$36&lt;$D$44,0,MIN((C93-$D$36-$D$44)*$G$37,(LL-C93)*$G$37)))</f>
         <v>1033.1336887869113</v>
       </c>
       <c r="F93" s="17">
+        <f t="shared" si="18"/>
+        <v>0.40014659179304718</v>
+      </c>
+      <c r="G93" s="18">
         <f t="shared" si="4"/>
-        <v>0.40014659179304718</v>
-      </c>
-      <c r="G93" s="18">
-        <f>IF(L93=oui,O93,IF(P93=oui,S93,W93))</f>
         <v>573.12304041217703</v>
       </c>
       <c r="H93" s="17">
-        <f>IF(C93/LL&lt;0.25,beff_a+(beff_m-beff_a)*C93/LL/0.25,IF((LL-C93)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C93)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L93" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E93,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M93" s="17">
-        <f>(Na-E93)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.0103492906843876</v>
       </c>
       <c r="N93" s="17">
-        <f>M93*tf</f>
+        <f t="shared" si="7"/>
         <v>12.831435991691722</v>
       </c>
       <c r="O93" s="17">
-        <f>(E93*(td-tc/2*F93)+Na*Ht/2-(Na-F93*Nc)*N93/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>575.3902316367604</v>
       </c>
       <c r="P93" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E93,E93&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>oui</v>
       </c>
       <c r="Q93" s="17">
-        <f>(E93-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>0.92106280826245035</v>
       </c>
       <c r="R93" s="18">
-        <f>dw/2+Q93*rr</f>
+        <f t="shared" si="11"/>
         <v>165.87913054872411</v>
       </c>
       <c r="S93" s="13">
-        <f>MplaRd+E93*(td-F93*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E93)*R93/1000</f>
+        <f t="shared" si="12"/>
         <v>573.12304041217703</v>
       </c>
       <c r="T93" s="68" t="str">
-        <f>IF(Nw&gt;E93,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>non</v>
       </c>
       <c r="U93" s="17">
-        <f>E93/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.60914177475337439</v>
       </c>
       <c r="V93" s="13">
-        <f>U93*dw</f>
+        <f t="shared" si="15"/>
         <v>181.8897339413576</v>
       </c>
       <c r="W93" s="13">
-        <f>MplaRd+E93*(Ht/2+td-F93*tc/2-V93/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>573.17566035464233</v>
       </c>
     </row>
@@ -8888,71 +9049,71 @@
         <v>5</v>
       </c>
       <c r="D94" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E94" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E94" s="13">
-        <f>IF(D94=1,IF(C94&lt;=$D$43,0,C94*$G$36),IF(C94-$D$36&lt;$D$44,0,MIN((C94-$D$36-$D$44)*$G$37,(LL-C94)*$G$37)))</f>
         <v>1231.8132443228558</v>
       </c>
       <c r="F94" s="17">
+        <f t="shared" si="18"/>
+        <v>0.47709785944555627</v>
+      </c>
+      <c r="G94" s="18">
         <f t="shared" si="4"/>
-        <v>0.47709785944555627</v>
-      </c>
-      <c r="G94" s="18">
-        <f>IF(L94=oui,O94,IF(P94=oui,S94,W94))</f>
         <v>597.37566726582918</v>
       </c>
       <c r="H94" s="17">
-        <f>IF(C94/LL&lt;0.25,beff_a+(beff_m-beff_a)*C94/LL/0.25,IF((LL-C94)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C94)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L94" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E94,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>oui</v>
       </c>
       <c r="M94" s="17">
-        <f>(Na-E94)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>0.8807381929957443</v>
       </c>
       <c r="N94" s="17">
-        <f>M94*tf</f>
+        <f t="shared" si="7"/>
         <v>11.185375051045952</v>
       </c>
       <c r="O94" s="17">
-        <f>(E94*(td-tc/2*F94)+Na*Ht/2-(Na-F94*Nc)*N94/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>597.37566726582918</v>
       </c>
       <c r="P94" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E94,E94&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q94" s="17">
-        <f>(E94-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>1.9096461210296634</v>
       </c>
       <c r="R94" s="18">
-        <f>dw/2+Q94*rr</f>
+        <f t="shared" si="11"/>
         <v>183.67363017853395</v>
       </c>
       <c r="S94" s="13">
-        <f>MplaRd+E94*(td-F94*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E94)*R94/1000</f>
+        <f t="shared" si="12"/>
         <v>588.65311377611772</v>
       </c>
       <c r="T94" s="68" t="str">
-        <f>IF(Nw&gt;E94,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>non</v>
       </c>
       <c r="U94" s="17">
-        <f>E94/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.72628442374440794</v>
       </c>
       <c r="V94" s="13">
-        <f>U94*dw</f>
+        <f t="shared" si="15"/>
         <v>216.86852893008023</v>
       </c>
       <c r="W94" s="13">
-        <f>MplaRd+E94*(Ht/2+td-F94*tc/2-V94/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>588.87930599792935</v>
       </c>
     </row>
@@ -8966,71 +9127,71 @@
         <v>5.5</v>
       </c>
       <c r="D95" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E95" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E95" s="13">
-        <f>IF(D95=1,IF(C95&lt;=$D$43,0,C95*$G$36),IF(C95-$D$36&lt;$D$44,0,MIN((C95-$D$36-$D$44)*$G$37,(LL-C95)*$G$37)))</f>
         <v>1430.4927998588003</v>
       </c>
       <c r="F95" s="17">
+        <f t="shared" si="18"/>
+        <v>0.55404912709806531</v>
+      </c>
+      <c r="G95" s="18">
         <f t="shared" si="4"/>
-        <v>0.55404912709806531</v>
-      </c>
-      <c r="G95" s="18">
-        <f>IF(L95=oui,O95,IF(P95=oui,S95,W95))</f>
         <v>617.87595113025804</v>
       </c>
       <c r="H95" s="17">
-        <f>IF(C95/LL&lt;0.25,beff_a+(beff_m-beff_a)*C95/LL/0.25,IF((LL-C95)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C95)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L95" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E95,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>oui</v>
       </c>
       <c r="M95" s="17">
-        <f>(Na-E95)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>0.75112709530710087</v>
       </c>
       <c r="N95" s="17">
-        <f>M95*tf</f>
+        <f t="shared" si="7"/>
         <v>9.5393141104001806</v>
       </c>
       <c r="O95" s="17">
-        <f>(E95*(td-tc/2*F95)+Na*Ht/2-(Na-F95*Nc)*N95/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>617.87595113025804</v>
       </c>
       <c r="P95" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E95,E95&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q95" s="17">
-        <f>(E95-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>2.8982294337968764</v>
       </c>
       <c r="R95" s="18">
-        <f>dw/2+Q95*rr</f>
+        <f t="shared" si="11"/>
         <v>201.4681298083438</v>
       </c>
       <c r="S95" s="13">
-        <f>MplaRd+E95*(td-F95*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E95)*R95/1000</f>
+        <f t="shared" si="12"/>
         <v>596.01159824201909</v>
       </c>
       <c r="T95" s="68" t="str">
-        <f>IF(Nw&gt;E95,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>non</v>
       </c>
       <c r="U95" s="17">
-        <f>E95/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.84342707273544149</v>
       </c>
       <c r="V95" s="13">
-        <f>U95*dw</f>
+        <f t="shared" si="15"/>
         <v>251.84732391880286</v>
       </c>
       <c r="W95" s="13">
-        <f>MplaRd+E95*(Ht/2+td-F95*tc/2-V95/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>596.53259785650471</v>
       </c>
     </row>
@@ -9044,71 +9205,71 @@
         <v>6</v>
       </c>
       <c r="D96" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E96" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E96" s="13">
-        <f>IF(D96=1,IF(C96&lt;=$D$43,0,C96*$G$36),IF(C96-$D$36&lt;$D$44,0,MIN((C96-$D$36-$D$44)*$G$37,(LL-C96)*$G$37)))</f>
         <v>1589.4364442875558</v>
       </c>
       <c r="F96" s="17">
+        <f t="shared" si="18"/>
+        <v>0.61561014122007263</v>
+      </c>
+      <c r="G96" s="18">
         <f t="shared" si="4"/>
-        <v>0.61561014122007263</v>
-      </c>
-      <c r="G96" s="18">
-        <f>IF(L96=oui,O96,IF(P96=oui,S96,W96))</f>
         <v>633.20686895126073</v>
       </c>
       <c r="H96" s="17">
-        <f>IF(C96/LL&lt;0.25,beff_a+(beff_m-beff_a)*C96/LL/0.25,IF((LL-C96)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C96)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L96" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E96,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>oui</v>
       </c>
       <c r="M96" s="17">
-        <f>(Na-E96)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>0.64743821715618632</v>
       </c>
       <c r="N96" s="17">
-        <f>M96*tf</f>
+        <f t="shared" si="7"/>
         <v>8.222465357883566</v>
       </c>
       <c r="O96" s="17">
-        <f>(E96*(td-tc/2*F96)+Na*Ht/2-(Na-F96*Nc)*N96/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>633.20686895126073</v>
       </c>
       <c r="P96" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E96,E96&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q96" s="17">
-        <f>(E96-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>3.6890960840106466</v>
       </c>
       <c r="R96" s="18">
-        <f>dw/2+Q96*rr</f>
+        <f t="shared" si="11"/>
         <v>215.70372951219164</v>
       </c>
       <c r="S96" s="13">
-        <f>MplaRd+E96*(td-F96*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E96)*R96/1000</f>
+        <f t="shared" si="12"/>
         <v>596.01484180815157</v>
       </c>
       <c r="T96" s="68" t="str">
-        <f>IF(Nw&gt;E96,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>non</v>
       </c>
       <c r="U96" s="17">
-        <f>E96/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.93714119192826828</v>
       </c>
       <c r="V96" s="13">
-        <f>U96*dw</f>
+        <f t="shared" si="15"/>
         <v>279.83035990978095</v>
       </c>
       <c r="W96" s="13">
-        <f>MplaRd+E96*(Ht/2+td-F96*tc/2-V96/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>596.85897661837271</v>
       </c>
     </row>
@@ -9122,71 +9283,71 @@
         <v>6.5</v>
       </c>
       <c r="D97" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E97" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E97" s="13">
-        <f>IF(D97=1,IF(C97&lt;=$D$43,0,C97*$G$36),IF(C97-$D$36&lt;$D$44,0,MIN((C97-$D$36-$D$44)*$G$37,(LL-C97)*$G$37)))</f>
         <v>1390.7568887516113</v>
       </c>
       <c r="F97" s="17">
+        <f t="shared" si="18"/>
+        <v>0.53865887356756348</v>
+      </c>
+      <c r="G97" s="18">
         <f t="shared" si="4"/>
-        <v>0.53865887356756348</v>
-      </c>
-      <c r="G97" s="18">
-        <f>IF(L97=oui,O97,IF(P97=oui,S97,W97))</f>
         <v>613.89470649854354</v>
       </c>
       <c r="H97" s="17">
-        <f>IF(C97/LL&lt;0.25,beff_a+(beff_m-beff_a)*C97/LL/0.25,IF((LL-C97)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C97)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L97" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E97,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>oui</v>
       </c>
       <c r="M97" s="17">
-        <f>(Na-E97)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>0.77704931484482964</v>
       </c>
       <c r="N97" s="17">
-        <f>M97*tf</f>
+        <f t="shared" si="7"/>
         <v>9.8685262985293356</v>
       </c>
       <c r="O97" s="17">
-        <f>(E97*(td-tc/2*F97)+Na*Ht/2-(Na-F97*Nc)*N97/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>613.89470649854354</v>
       </c>
       <c r="P97" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E97,E97&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q97" s="17">
-        <f>(E97-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>2.7005127712434334</v>
       </c>
       <c r="R97" s="18">
-        <f>dw/2+Q97*rr</f>
+        <f t="shared" si="11"/>
         <v>197.90922988238179</v>
       </c>
       <c r="S97" s="13">
-        <f>MplaRd+E97*(td-F97*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E97)*R97/1000</f>
+        <f t="shared" si="12"/>
         <v>595.19362846068191</v>
       </c>
       <c r="T97" s="68" t="str">
-        <f>IF(Nw&gt;E97,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>non</v>
       </c>
       <c r="U97" s="17">
-        <f>E97/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.81999854293723473</v>
       </c>
       <c r="V97" s="13">
-        <f>U97*dw</f>
+        <f t="shared" si="15"/>
         <v>244.8515649210583</v>
       </c>
       <c r="W97" s="13">
-        <f>MplaRd+E97*(Ht/2+td-F97*tc/2-V97/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>595.64596778756663</v>
       </c>
     </row>
@@ -9200,71 +9361,71 @@
         <v>7</v>
       </c>
       <c r="D98" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E98" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E98" s="13">
-        <f>IF(D98=1,IF(C98&lt;=$D$43,0,C98*$G$36),IF(C98-$D$36&lt;$D$44,0,MIN((C98-$D$36-$D$44)*$G$37,(LL-C98)*$G$37)))</f>
         <v>1192.0773332156668</v>
       </c>
       <c r="F98" s="17">
+        <f t="shared" si="18"/>
+        <v>0.46170760591505444</v>
+      </c>
+      <c r="G98" s="18">
         <f t="shared" si="4"/>
-        <v>0.46170760591505444</v>
-      </c>
-      <c r="G98" s="18">
-        <f>IF(L98=oui,O98,IF(P98=oui,S98,W98))</f>
         <v>593.09739228118656</v>
       </c>
       <c r="H98" s="17">
-        <f>IF(C98/LL&lt;0.25,beff_a+(beff_m-beff_a)*C98/LL/0.25,IF((LL-C98)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C98)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L98" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E98,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>oui</v>
       </c>
       <c r="M98" s="17">
-        <f>(Na-E98)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>0.90666041253347296</v>
       </c>
       <c r="N98" s="17">
-        <f>M98*tf</f>
+        <f t="shared" si="7"/>
         <v>11.514587239175105</v>
       </c>
       <c r="O98" s="17">
-        <f>(E98*(td-tc/2*F98)+Na*Ht/2-(Na-F98*Nc)*N98/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>593.09739228118656</v>
       </c>
       <c r="P98" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E98,E98&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q98" s="17">
-        <f>(E98-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>1.7119294584762206</v>
       </c>
       <c r="R98" s="18">
-        <f>dw/2+Q98*rr</f>
+        <f t="shared" si="11"/>
         <v>180.11473025257197</v>
       </c>
       <c r="S98" s="13">
-        <f>MplaRd+E98*(td-F98*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E98)*R98/1000</f>
+        <f t="shared" si="12"/>
         <v>586.2008262151727</v>
       </c>
       <c r="T98" s="68" t="str">
-        <f>IF(Nw&gt;E98,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>non</v>
       </c>
       <c r="U98" s="17">
-        <f>E98/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.70285589394620118</v>
       </c>
       <c r="V98" s="13">
-        <f>U98*dw</f>
+        <f t="shared" si="15"/>
         <v>209.8727699323357</v>
       </c>
       <c r="W98" s="13">
-        <f>MplaRd+E98*(Ht/2+td-F98*tc/2-V98/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>586.38260517204878</v>
       </c>
     </row>
@@ -9278,71 +9439,71 @@
         <v>7.5</v>
       </c>
       <c r="D99" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E99" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E99" s="13">
-        <f>IF(D99=1,IF(C99&lt;=$D$43,0,C99*$G$36),IF(C99-$D$36&lt;$D$44,0,MIN((C99-$D$36-$D$44)*$G$37,(LL-C99)*$G$37)))</f>
         <v>993.39777767972237</v>
       </c>
       <c r="F99" s="17">
+        <f t="shared" si="18"/>
+        <v>0.38475633826254535</v>
+      </c>
+      <c r="G99" s="18">
         <f t="shared" si="4"/>
-        <v>0.38475633826254535</v>
-      </c>
-      <c r="G99" s="18">
-        <f>IF(L99=oui,O99,IF(P99=oui,S99,W99))</f>
         <v>569.03643507162406</v>
       </c>
       <c r="H99" s="17">
-        <f>IF(C99/LL&lt;0.25,beff_a+(beff_m-beff_a)*C99/LL/0.25,IF((LL-C99)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C99)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.125</v>
       </c>
       <c r="L99" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E99,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M99" s="17">
-        <f>(Na-E99)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.0362715102221163</v>
       </c>
       <c r="N99" s="17">
-        <f>M99*tf</f>
+        <f t="shared" si="7"/>
         <v>13.160648179820877</v>
       </c>
       <c r="O99" s="17">
-        <f>(E99*(td-tc/2*F99)+Na*Ht/2-(Na-F99*Nc)*N99/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>570.81492629918989</v>
       </c>
       <c r="P99" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E99,E99&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>oui</v>
       </c>
       <c r="Q99" s="17">
-        <f>(E99-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>0.72334614570900757</v>
       </c>
       <c r="R99" s="18">
-        <f>dw/2+Q99*rr</f>
+        <f t="shared" si="11"/>
         <v>162.32023062276215</v>
       </c>
       <c r="S99" s="13">
-        <f>MplaRd+E99*(td-F99*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E99)*R99/1000</f>
+        <f t="shared" si="12"/>
         <v>569.03643507162406</v>
       </c>
       <c r="T99" s="68" t="str">
-        <f>IF(Nw&gt;E99,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>non</v>
       </c>
       <c r="U99" s="17">
-        <f>E99/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.58571324495516763</v>
       </c>
       <c r="V99" s="13">
-        <f>U99*dw</f>
+        <f t="shared" si="15"/>
         <v>174.89397494361307</v>
       </c>
       <c r="W99" s="13">
-        <f>MplaRd+E99*(Ht/2+td-F99*tc/2-V99/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>569.06888877181962</v>
       </c>
     </row>
@@ -9356,71 +9517,71 @@
         <v>8</v>
       </c>
       <c r="D100" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E100" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E100" s="13">
-        <f>IF(D100=1,IF(C100&lt;=$D$43,0,C100*$G$36),IF(C100-$D$36&lt;$D$44,0,MIN((C100-$D$36-$D$44)*$G$37,(LL-C100)*$G$37)))</f>
         <v>794.71822214377789</v>
       </c>
       <c r="F100" s="17">
+        <f t="shared" si="18"/>
+        <v>0.30780507061003631</v>
+      </c>
+      <c r="G100" s="18">
         <f t="shared" si="4"/>
-        <v>0.30780507061003631</v>
-      </c>
-      <c r="G100" s="18">
-        <f>IF(L100=oui,O100,IF(P100=oui,S100,W100))</f>
         <v>543.70481858687879</v>
       </c>
       <c r="H100" s="17">
-        <f>IF(C100/LL&lt;0.25,beff_a+(beff_m-beff_a)*C100/LL/0.25,IF((LL-C100)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C100)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>2.0187499999999998</v>
       </c>
       <c r="L100" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E100,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M100" s="17">
-        <f>(Na-E100)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.1658826079107596</v>
       </c>
       <c r="N100" s="17">
-        <f>M100*tf</f>
+        <f t="shared" si="7"/>
         <v>14.806709120466646</v>
       </c>
       <c r="O100" s="17">
-        <f>(E100*(td-tc/2*F100)+Na*Ht/2-(Na-F100*Nc)*N100/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>547.04730855255366</v>
       </c>
       <c r="P100" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E100,E100&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q100" s="17">
-        <f>(E100-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-0.26523716705820544</v>
       </c>
       <c r="R100" s="18">
-        <f>dw/2+Q100*rr</f>
+        <f t="shared" si="11"/>
         <v>144.5257309929523</v>
       </c>
       <c r="S100" s="13">
-        <f>MplaRd+E100*(td-F100*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E100)*R100/1000</f>
+        <f t="shared" si="12"/>
         <v>543.70045503003587</v>
       </c>
       <c r="T100" s="68" t="str">
-        <f>IF(Nw&gt;E100,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U100" s="17">
-        <f>E100/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.46857059596413414</v>
       </c>
       <c r="V100" s="13">
-        <f>U100*dw</f>
+        <f t="shared" si="15"/>
         <v>139.91517995489048</v>
       </c>
       <c r="W100" s="13">
-        <f>MplaRd+E100*(Ht/2+td-F100*tc/2-V100/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>543.70481858687879</v>
       </c>
     </row>
@@ -9434,71 +9595,71 @@
         <v>8.5</v>
       </c>
       <c r="D101" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E101" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E101" s="13">
-        <f>IF(D101=1,IF(C101&lt;=$D$43,0,C101*$G$36),IF(C101-$D$36&lt;$D$44,0,MIN((C101-$D$36-$D$44)*$G$37,(LL-C101)*$G$37)))</f>
         <v>596.03866660783342</v>
       </c>
       <c r="F101" s="17">
+        <f t="shared" si="18"/>
+        <v>0.23085380295752722</v>
+      </c>
+      <c r="G101" s="18">
         <f t="shared" si="4"/>
-        <v>0.23085380295752722</v>
-      </c>
-      <c r="G101" s="18">
-        <f>IF(L101=oui,O101,IF(P101=oui,S101,W101))</f>
         <v>510.29039461722641</v>
       </c>
       <c r="H101" s="17">
-        <f>IF(C101/LL&lt;0.25,beff_a+(beff_m-beff_a)*C101/LL/0.25,IF((LL-C101)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C101)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>1.9125000000000001</v>
       </c>
       <c r="L101" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E101,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M101" s="17">
-        <f>(Na-E101)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.2954937055994029</v>
       </c>
       <c r="N101" s="17">
-        <f>M101*tf</f>
+        <f t="shared" si="7"/>
         <v>16.452770061112417</v>
       </c>
       <c r="O101" s="17">
-        <f>(E101*(td-tc/2*F101)+Na*Ht/2-(Na-F101*Nc)*N101/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>521.79453904127763</v>
       </c>
       <c r="P101" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E101,E101&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q101" s="17">
-        <f>(E101-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-1.2538204798254184</v>
       </c>
       <c r="R101" s="18">
-        <f>dw/2+Q101*rr</f>
+        <f t="shared" si="11"/>
         <v>126.73123136314248</v>
       </c>
       <c r="S101" s="13">
-        <f>MplaRd+E101*(td-F101*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E101)*R101/1000</f>
+        <f t="shared" si="12"/>
         <v>510.19288609040814</v>
       </c>
       <c r="T101" s="68" t="str">
-        <f>IF(Nw&gt;E101,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U101" s="17">
-        <f>E101/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.35142794697310059</v>
       </c>
       <c r="V101" s="13">
-        <f>U101*dw</f>
+        <f t="shared" si="15"/>
         <v>104.93638496616785</v>
       </c>
       <c r="W101" s="13">
-        <f>MplaRd+E101*(Ht/2+td-F101*tc/2-V101/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>510.29039461722641</v>
       </c>
     </row>
@@ -9512,71 +9673,71 @@
         <v>9</v>
       </c>
       <c r="D102" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E102" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E102" s="13">
-        <f>IF(D102=1,IF(C102&lt;=$D$43,0,C102*$G$36),IF(C102-$D$36&lt;$D$44,0,MIN((C102-$D$36-$D$44)*$G$37,(LL-C102)*$G$37)))</f>
         <v>397.35911107188895</v>
       </c>
       <c r="F102" s="17">
+        <f t="shared" si="18"/>
+        <v>0.15390253530501816</v>
+      </c>
+      <c r="G102" s="18">
         <f t="shared" si="4"/>
-        <v>0.15390253530501816</v>
-      </c>
-      <c r="G102" s="18">
-        <f>IF(L102=oui,O102,IF(P102=oui,S102,W102))</f>
         <v>468.82561686286249</v>
       </c>
       <c r="H102" s="17">
-        <f>IF(C102/LL&lt;0.25,beff_a+(beff_m-beff_a)*C102/LL/0.25,IF((LL-C102)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C102)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>1.8062499999999999</v>
       </c>
       <c r="L102" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E102,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M102" s="17">
-        <f>(Na-E102)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.4251048032880462</v>
       </c>
       <c r="N102" s="17">
-        <f>M102*tf</f>
+        <f t="shared" si="7"/>
         <v>18.098831001758185</v>
       </c>
       <c r="O102" s="17">
-        <f>(E102*(td-tc/2*F102)+Na*Ht/2-(Na-F102*Nc)*N102/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>495.05661776536198</v>
       </c>
       <c r="P102" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E102,E102&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q102" s="17">
-        <f>(E102-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-2.2424037925926315</v>
       </c>
       <c r="R102" s="18">
-        <f>dw/2+Q102*rr</f>
+        <f t="shared" si="11"/>
         <v>108.93673173333264</v>
       </c>
       <c r="S102" s="13">
-        <f>MplaRd+E102*(td-F102*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E102)*R102/1000</f>
+        <f t="shared" si="12"/>
         <v>468.51372825274098</v>
       </c>
       <c r="T102" s="68" t="str">
-        <f>IF(Nw&gt;E102,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U102" s="17">
-        <f>E102/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.23428529798206707</v>
       </c>
       <c r="V102" s="13">
-        <f>U102*dw</f>
+        <f t="shared" si="15"/>
         <v>69.957589977445238</v>
       </c>
       <c r="W102" s="13">
-        <f>MplaRd+E102*(Ht/2+td-F102*tc/2-V102/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>468.82561686286249</v>
       </c>
     </row>
@@ -9590,72 +9751,72 @@
         <v>9.5</v>
       </c>
       <c r="D103" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E103" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E103" s="13">
-        <f>IF(D103=1,IF(C103&lt;=$D$43,0,C103*$G$36),IF(C103-$D$36&lt;$D$44,0,MIN((C103-$D$36-$D$44)*$G$37,(LL-C103)*$G$37)))</f>
         <v>198.67955553594447</v>
       </c>
       <c r="F103" s="17">
+        <f t="shared" si="18"/>
+        <v>7.6951267652509078E-2</v>
+      </c>
+      <c r="G103" s="18">
         <f t="shared" si="4"/>
-        <v>7.6951267652509078E-2</v>
-      </c>
-      <c r="G103" s="18">
-        <f>IF(L103=oui,O103,IF(P103=oui,S103,W103))</f>
         <v>419.31048532378702</v>
       </c>
       <c r="H103" s="17">
-        <f>IF(C103/LL&lt;0.25,beff_a+(beff_m-beff_a)*C103/LL/0.25,IF((LL-C103)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C103)/LL/0.25,beff_m))</f>
+        <f t="shared" si="19"/>
         <v>1.7</v>
       </c>
       <c r="J103" s="67"/>
       <c r="L103" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E103,oui,non)</f>
+        <f t="shared" si="5"/>
         <v>non</v>
       </c>
       <c r="M103" s="17">
-        <f>(Na-E103)/(2*Nf)</f>
+        <f t="shared" si="6"/>
         <v>1.5547159009766895</v>
       </c>
       <c r="N103" s="17">
-        <f>M103*tf</f>
+        <f t="shared" si="7"/>
         <v>19.744891942403957</v>
       </c>
       <c r="O103" s="17">
-        <f>(E103*(td-tc/2*F103)+Na*Ht/2-(Na-F103*Nc)*N103/2)/1000</f>
+        <f t="shared" si="8"/>
         <v>466.83354472480664</v>
       </c>
       <c r="P103" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E103,E103&gt;=Nw),oui,non)</f>
+        <f t="shared" si="9"/>
         <v>non</v>
       </c>
       <c r="Q103" s="17">
-        <f>(E103-Nw)/(2*Nr)</f>
+        <f t="shared" si="10"/>
         <v>-3.2309871053598442</v>
       </c>
       <c r="R103" s="18">
-        <f>dw/2+Q103*rr</f>
+        <f t="shared" si="11"/>
         <v>91.142232103522815</v>
       </c>
       <c r="S103" s="13">
-        <f>MplaRd+E103*(td-F103*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E103)*R103/1000</f>
+        <f t="shared" si="12"/>
         <v>418.66298151703421</v>
       </c>
       <c r="T103" s="68" t="str">
-        <f>IF(Nw&gt;E103,oui,non)</f>
+        <f t="shared" si="13"/>
         <v>oui</v>
       </c>
       <c r="U103" s="17">
-        <f>E103/2/Nw</f>
+        <f t="shared" si="14"/>
         <v>0.11714264899103354</v>
       </c>
       <c r="V103" s="13">
-        <f>U103*dw</f>
+        <f t="shared" si="15"/>
         <v>34.978794988722619</v>
       </c>
       <c r="W103" s="13">
-        <f>MplaRd+E103*(Ht/2+td-F103*tc/2-V103/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>419.31048532378702</v>
       </c>
     </row>
@@ -9669,71 +9830,71 @@
         <v>10</v>
       </c>
       <c r="D104" s="3">
+        <f t="shared" si="17"/>
+        <v>2</v>
+      </c>
+      <c r="E104" s="13">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="E104" s="13">
-        <f>IF(D104=1,IF(C104&lt;=$D$43,0,C104*$G$36),IF(C104-$D$36&lt;$D$44,0,MIN((C104-$D$36-$D$44)*$G$37,(LL-C104)*$G$37)))</f>
         <v>0</v>
       </c>
       <c r="F104" s="17">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="G104" s="18">
         <f t="shared" si="4"/>
+        <v>361.745</v>
+      </c>
+      <c r="H104" s="17">
+        <f t="shared" si="19"/>
+        <v>1.59375</v>
+      </c>
+      <c r="L104" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>non</v>
+      </c>
+      <c r="M104" s="17">
+        <f t="shared" si="6"/>
+        <v>1.6843269986653329</v>
+      </c>
+      <c r="N104" s="17">
+        <f t="shared" si="7"/>
+        <v>21.390952883049724</v>
+      </c>
+      <c r="O104" s="17">
+        <f t="shared" si="8"/>
+        <v>437.12531991961151</v>
+      </c>
+      <c r="P104" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v>non</v>
+      </c>
+      <c r="Q104" s="17">
+        <f t="shared" si="10"/>
+        <v>-4.2195704181270575</v>
+      </c>
+      <c r="R104" s="18">
+        <f t="shared" si="11"/>
+        <v>73.347732473712981</v>
+      </c>
+      <c r="S104" s="13">
+        <f t="shared" si="12"/>
+        <v>360.64064588328802</v>
+      </c>
+      <c r="T104" s="68" t="str">
+        <f t="shared" si="13"/>
+        <v>oui</v>
+      </c>
+      <c r="U104" s="17">
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="G104" s="18">
-        <f>IF(L104=oui,O104,IF(P104=oui,S104,W104))</f>
-        <v>361.745</v>
-      </c>
-      <c r="H104" s="17">
-        <f>IF(C104/LL&lt;0.25,beff_a+(beff_m-beff_a)*C104/LL/0.25,IF((LL-C104)/LL&lt;0.25,beff_B+(beff_m-beff_B)*(LL-C104)/LL/0.25,beff_m))</f>
-        <v>1.59375</v>
-      </c>
-      <c r="L104" s="3" t="str">
-        <f>IF(Na-2*Nf&lt;=E104,oui,non)</f>
-        <v>non</v>
-      </c>
-      <c r="M104" s="17">
-        <f>(Na-E104)/(2*Nf)</f>
-        <v>1.6843269986653329</v>
-      </c>
-      <c r="N104" s="17">
-        <f>M104*tf</f>
-        <v>21.390952883049724</v>
-      </c>
-      <c r="O104" s="17">
-        <f>(E104*(td-tc/2*F104)+Na*Ht/2-(Na-F104*Nc)*N104/2)/1000</f>
-        <v>437.12531991961151</v>
-      </c>
-      <c r="P104" s="3" t="str">
-        <f>IF(AND(Na-2*Nf&gt;E104,E104&gt;=Nw),oui,non)</f>
-        <v>non</v>
-      </c>
-      <c r="Q104" s="17">
-        <f>(E104-Nw)/(2*Nr)</f>
-        <v>-4.2195704181270575</v>
-      </c>
-      <c r="R104" s="18">
-        <f>dw/2+Q104*rr</f>
-        <v>73.347732473712981</v>
-      </c>
-      <c r="S104" s="13">
-        <f>MplaRd+E104*(td-F104*tc/2+Ht/2)/1000-Nw*dw/4000+(Nw-E104)*R104/1000</f>
-        <v>360.64064588328802</v>
-      </c>
-      <c r="T104" s="68" t="str">
-        <f>IF(Nw&gt;E104,oui,non)</f>
-        <v>oui</v>
-      </c>
-      <c r="U104" s="17">
-        <f>E104/2/Nw</f>
+      <c r="V104" s="13">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="V104" s="13">
-        <f>U104*dw</f>
-        <v>0</v>
-      </c>
       <c r="W104" s="13">
-        <f>MplaRd+E104*(Ht/2+td-F104*tc/2-V104/2)/1000</f>
+        <f t="shared" si="16"/>
         <v>361.745</v>
       </c>
     </row>
@@ -9789,11 +9950,11 @@
     </row>
     <row r="112" spans="2:23" x14ac:dyDescent="0.25">
       <c r="E112" s="3">
-        <f t="shared" ref="E112:F112" si="5">B85</f>
+        <f t="shared" ref="E112:F112" si="20">B85</f>
         <v>2</v>
       </c>
       <c r="F112" s="13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="20"/>
         <v>0.5</v>
       </c>
       <c r="G112" s="18">
@@ -9801,7 +9962,7 @@
         <v>-286.21268314456569</v>
       </c>
       <c r="H112" s="17">
-        <f t="shared" ref="H112:H129" si="6">IF(G112&gt;0,G112/$G85,0)</f>
+        <f t="shared" ref="H112:H129" si="21">IF(G112&gt;0,G112/$G85,0)</f>
         <v>0</v>
       </c>
       <c r="I112" s="18">
@@ -9809,7 +9970,7 @@
         <v>112.78731685543431</v>
       </c>
       <c r="J112" s="17">
-        <f t="shared" ref="J112:J129" si="7">IF(I112&gt;0,I112/$G85,0)</f>
+        <f t="shared" ref="J112:J129" si="22">IF(I112&gt;0,I112/$G85,0)</f>
         <v>0.31178680245873286</v>
       </c>
       <c r="K112" s="18">
@@ -9817,17 +9978,17 @@
         <v>-143.71268314456569</v>
       </c>
       <c r="L112" s="17">
-        <f t="shared" ref="L112:L129" si="8">IF(K112&gt;0,K112/$G85,0)</f>
+        <f t="shared" ref="L112:L129" si="23">IF(K112&gt;0,K112/$G85,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="113" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E113" s="3">
-        <f t="shared" ref="E113:F113" si="9">B86</f>
+        <f t="shared" ref="E113:F113" si="24">B86</f>
         <v>3</v>
       </c>
       <c r="F113" s="13">
-        <f t="shared" si="9"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
       <c r="G113" s="18">
@@ -9835,7 +9996,7 @@
         <v>-235.96278557102391</v>
       </c>
       <c r="H113" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="I113" s="18">
@@ -9843,7 +10004,7 @@
         <v>277.03721442897609</v>
       </c>
       <c r="J113" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>0.76583564231427137</v>
       </c>
       <c r="K113" s="18">
@@ -9851,17 +10012,17 @@
         <v>34.037214428976078</v>
       </c>
       <c r="L113" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>9.4091734312778549E-2</v>
       </c>
     </row>
     <row r="114" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E114" s="3">
-        <f t="shared" ref="E114:F114" si="10">B87</f>
+        <f t="shared" ref="E114:F114" si="25">B87</f>
         <v>4</v>
       </c>
       <c r="F114" s="13">
-        <f t="shared" si="10"/>
+        <f t="shared" si="25"/>
         <v>1.5</v>
       </c>
       <c r="G114" s="18">
@@ -9869,7 +10030,7 @@
         <v>-189.62245156913554</v>
       </c>
       <c r="H114" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="I114" s="18">
@@ -9877,7 +10038,7 @@
         <v>422.37754843086446</v>
       </c>
       <c r="J114" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.1676112964404883</v>
       </c>
       <c r="K114" s="18">
@@ -9885,17 +10046,17 @@
         <v>192.87754843086446</v>
       </c>
       <c r="L114" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>0.53318649443907851</v>
       </c>
     </row>
     <row r="115" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E115" s="3">
-        <f t="shared" ref="E115:F115" si="11">B88</f>
+        <f t="shared" ref="E115:F115" si="26">B88</f>
         <v>5</v>
       </c>
       <c r="F115" s="13">
-        <f t="shared" si="11"/>
+        <f t="shared" si="26"/>
         <v>2</v>
       </c>
       <c r="G115" s="18">
@@ -9903,7 +10064,7 @@
         <v>-147.19168113890052</v>
       </c>
       <c r="H115" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="I115" s="18">
@@ -9911,7 +10072,7 @@
         <v>548.80831886109945</v>
       </c>
       <c r="J115" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.4677860371123532</v>
       </c>
       <c r="K115" s="18">
@@ -9919,17 +10080,17 @@
         <v>332.80831886109945</v>
       </c>
       <c r="L115" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>0.89009475015409201</v>
       </c>
     </row>
     <row r="116" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E116" s="3">
-        <f t="shared" ref="E116:F116" si="12">B89</f>
+        <f t="shared" ref="E116:F116" si="27">B89</f>
         <v>6</v>
       </c>
       <c r="F116" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="27"/>
         <v>2.5</v>
       </c>
       <c r="G116" s="18">
@@ -9937,7 +10098,7 @@
         <v>-108.67047428031889</v>
       </c>
       <c r="H116" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="I116" s="18">
@@ -9945,7 +10106,7 @@
         <v>656.3295257196811</v>
       </c>
       <c r="J116" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.5268535846082278</v>
       </c>
       <c r="K116" s="18">
@@ -9953,17 +10114,17 @@
         <v>453.8295257196811</v>
       </c>
       <c r="L116" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.0557672799899278</v>
       </c>
     </row>
     <row r="117" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E117" s="3">
-        <f t="shared" ref="E117:F117" si="13">B90</f>
+        <f t="shared" ref="E117:F117" si="28">B90</f>
         <v>7</v>
       </c>
       <c r="F117" s="13">
-        <f t="shared" si="13"/>
+        <f t="shared" si="28"/>
         <v>3</v>
       </c>
       <c r="G117" s="18">
@@ -9971,7 +10132,7 @@
         <v>-74.058830993390643</v>
       </c>
       <c r="H117" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="I117" s="18">
@@ -9979,7 +10140,7 @@
         <v>744.94116900660936</v>
       </c>
       <c r="J117" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.5592287213134786</v>
       </c>
       <c r="K117" s="18">
@@ -9987,17 +10148,17 @@
         <v>555.94116900660936</v>
       </c>
       <c r="L117" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.1636347595497236</v>
       </c>
     </row>
     <row r="118" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E118" s="3">
-        <f t="shared" ref="E118:F118" si="14">B91</f>
+        <f t="shared" ref="E118:F118" si="29">B91</f>
         <v>8</v>
       </c>
       <c r="F118" s="13">
-        <f t="shared" si="14"/>
+        <f t="shared" si="29"/>
         <v>3.5</v>
       </c>
       <c r="G118" s="18">
@@ -10005,7 +10166,7 @@
         <v>-43.356751278115752</v>
       </c>
       <c r="H118" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="I118" s="18">
@@ -10013,7 +10174,7 @@
         <v>814.64324872188422</v>
       </c>
       <c r="J118" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.5738330936416538</v>
       </c>
       <c r="K118" s="18">
@@ -10021,17 +10182,17 @@
         <v>639.14324872188422</v>
       </c>
       <c r="L118" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.2347795160572816</v>
       </c>
     </row>
     <row r="119" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E119" s="3">
-        <f t="shared" ref="E119:F119" si="15">B92</f>
+        <f t="shared" ref="E119:F119" si="30">B92</f>
         <v>9</v>
       </c>
       <c r="F119" s="13">
-        <f t="shared" si="15"/>
+        <f t="shared" si="30"/>
         <v>4</v>
       </c>
       <c r="G119" s="18">
@@ -10039,7 +10200,7 @@
         <v>-16.564235134494282</v>
       </c>
       <c r="H119" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="I119" s="18">
@@ -10047,7 +10208,7 @@
         <v>865.43576486550569</v>
       </c>
       <c r="J119" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.5751759102578493</v>
       </c>
       <c r="K119" s="18">
@@ -10055,17 +10216,17 @@
         <v>703.43576486550569</v>
       </c>
       <c r="L119" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.2803204076066179</v>
       </c>
     </row>
     <row r="120" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E120" s="3">
-        <f t="shared" ref="E120:F120" si="16">B93</f>
+        <f t="shared" ref="E120:F120" si="31">B93</f>
         <v>10</v>
       </c>
       <c r="F120" s="13">
-        <f t="shared" si="16"/>
+        <f t="shared" si="31"/>
         <v>4.5</v>
       </c>
       <c r="G120" s="18">
@@ -10073,7 +10234,7 @@
         <v>6.318717437473822</v>
       </c>
       <c r="H120" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>1.1025062668793675E-2</v>
       </c>
       <c r="I120" s="18">
@@ -10081,7 +10242,7 @@
         <v>897.31871743747388</v>
       </c>
       <c r="J120" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.5656650564809655</v>
       </c>
       <c r="K120" s="18">
@@ -10089,17 +10250,17 @@
         <v>748.81871743747388</v>
       </c>
       <c r="L120" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.3065583908456035</v>
       </c>
     </row>
     <row r="121" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E121" s="3">
-        <f t="shared" ref="E121:F121" si="17">B94</f>
+        <f t="shared" ref="E121:F121" si="32">B94</f>
         <v>11</v>
       </c>
       <c r="F121" s="13">
-        <f t="shared" si="17"/>
+        <f t="shared" si="32"/>
         <v>5</v>
       </c>
       <c r="G121" s="18">
@@ -10107,7 +10268,7 @@
         <v>25.292106437788561</v>
       </c>
       <c r="H121" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>4.2338695436909553E-2</v>
       </c>
       <c r="I121" s="18">
@@ -10115,7 +10276,7 @@
         <v>910.29210643778856</v>
       </c>
       <c r="J121" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.5238185221104983</v>
       </c>
       <c r="K121" s="18">
@@ -10123,17 +10284,17 @@
         <v>775.29210643778856</v>
       </c>
       <c r="L121" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.2978300739738491</v>
       </c>
     </row>
     <row r="122" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E122" s="3">
-        <f t="shared" ref="E122:F122" si="18">B95</f>
+        <f t="shared" ref="E122:F122" si="33">B95</f>
         <v>12</v>
       </c>
       <c r="F122" s="13">
-        <f t="shared" si="18"/>
+        <f t="shared" si="33"/>
         <v>5.5</v>
       </c>
       <c r="G122" s="18">
@@ -10141,7 +10302,7 @@
         <v>40.355931866449907</v>
       </c>
       <c r="H122" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>6.5313970858759382E-2</v>
       </c>
       <c r="I122" s="18">
@@ -10149,7 +10310,7 @@
         <v>904.35593186644996</v>
       </c>
       <c r="J122" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.4636529067236628</v>
       </c>
       <c r="K122" s="18">
@@ -10157,17 +10318,17 @@
         <v>782.85593186644996</v>
       </c>
       <c r="L122" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.2670114938676607</v>
       </c>
     </row>
     <row r="123" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E123" s="3">
-        <f t="shared" ref="E123:F123" si="19">B96</f>
+        <f t="shared" ref="E123:F123" si="34">B96</f>
         <v>13</v>
       </c>
       <c r="F123" s="13">
-        <f t="shared" si="19"/>
+        <f t="shared" si="34"/>
         <v>6</v>
       </c>
       <c r="G123" s="18">
@@ -10175,7 +10336,7 @@
         <v>51.510193723457888</v>
       </c>
       <c r="H123" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>8.1348128469880418E-2</v>
       </c>
       <c r="I123" s="18">
@@ -10183,7 +10344,7 @@
         <v>879.51019372345786</v>
       </c>
       <c r="J123" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.3889776577757806</v>
       </c>
       <c r="K123" s="18">
@@ -10191,17 +10352,17 @@
         <v>771.51019372345786</v>
       </c>
       <c r="L123" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.2184172843880545</v>
       </c>
     </row>
     <row r="124" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E124" s="3">
-        <f t="shared" ref="E124:F124" si="20">B97</f>
+        <f t="shared" ref="E124:F124" si="35">B97</f>
         <v>14</v>
       </c>
       <c r="F124" s="13">
-        <f t="shared" si="20"/>
+        <f t="shared" si="35"/>
         <v>6.5</v>
       </c>
       <c r="G124" s="18">
@@ -10209,7 +10370,7 @@
         <v>58.754892008812476</v>
       </c>
       <c r="H124" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>9.5708419354080018E-2</v>
       </c>
       <c r="I124" s="18">
@@ -10217,7 +10378,7 @@
         <v>835.75489200881248</v>
       </c>
       <c r="J124" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.3613977823260401</v>
       </c>
       <c r="K124" s="18">
@@ -10225,7 +10386,7 @@
         <v>741.25489200881248</v>
       </c>
       <c r="L124" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.2074625895321531</v>
       </c>
     </row>
@@ -10265,11 +10426,11 @@
     </row>
     <row r="126" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E126" s="3">
-        <f t="shared" ref="E126:E129" si="21">B99</f>
+        <f t="shared" ref="E126:E129" si="36">B99</f>
         <v>16</v>
       </c>
       <c r="F126" s="13">
-        <f t="shared" ref="F126:F129" si="22">C99</f>
+        <f t="shared" ref="F126:F129" si="37">C99</f>
         <v>7.5</v>
       </c>
       <c r="G126" s="18">
@@ -10277,7 +10438,7 @@
         <v>61.515597864561528</v>
       </c>
       <c r="H126" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>0.10810484895720011</v>
       </c>
       <c r="I126" s="18">
@@ -10285,7 +10446,7 @@
         <v>691.51559786456153</v>
       </c>
       <c r="J126" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.2152395791273385</v>
       </c>
       <c r="K126" s="18">
@@ -10293,17 +10454,17 @@
         <v>624.01559786456153</v>
       </c>
       <c r="L126" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>1.0966180008948236</v>
       </c>
     </row>
     <row r="127" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E127" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="36"/>
         <v>17</v>
       </c>
       <c r="F127" s="13">
-        <f t="shared" si="22"/>
+        <f t="shared" si="37"/>
         <v>8</v>
       </c>
       <c r="G127" s="18">
@@ -10311,7 +10472,7 @@
         <v>57.031605434955978</v>
       </c>
       <c r="H127" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>0.10489442705912469</v>
       </c>
       <c r="I127" s="18">
@@ -10319,7 +10480,7 @@
         <v>591.03160543495596</v>
       </c>
       <c r="J127" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>1.0870450016813946</v>
       </c>
       <c r="K127" s="18">
@@ -10327,17 +10488,17 @@
         <v>537.03160543495596</v>
       </c>
       <c r="L127" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>0.98772640424768188</v>
       </c>
     </row>
     <row r="128" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E128" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="36"/>
         <v>18</v>
       </c>
       <c r="F128" s="13">
-        <f t="shared" si="22"/>
+        <f t="shared" si="37"/>
         <v>8.5</v>
       </c>
       <c r="G128" s="18">
@@ -10345,7 +10506,7 @@
         <v>48.638049433697063</v>
       </c>
       <c r="H128" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>9.5314452215352632E-2</v>
       </c>
       <c r="I128" s="18">
@@ -10353,7 +10514,7 @@
         <v>471.63804943369706</v>
       </c>
       <c r="J128" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>0.92425421761559345</v>
       </c>
       <c r="K128" s="18">
@@ -10361,17 +10522,17 @@
         <v>431.13804943369706</v>
       </c>
       <c r="L128" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>0.84488764433259167</v>
       </c>
     </row>
     <row r="129" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E129" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="36"/>
         <v>19</v>
       </c>
       <c r="F129" s="13">
-        <f t="shared" si="22"/>
+        <f t="shared" si="37"/>
         <v>9</v>
       </c>
       <c r="G129" s="18">
@@ -10379,7 +10540,7 @@
         <v>36.334929860784747</v>
       </c>
       <c r="H129" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="21"/>
         <v>7.7502014723340465E-2</v>
       </c>
       <c r="I129" s="18">
@@ -10387,7 +10548,7 @@
         <v>333.33492986078477</v>
       </c>
       <c r="J129" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="22"/>
         <v>0.71099982140756079</v>
       </c>
       <c r="K129" s="18">
@@ -10395,7 +10556,7 @@
         <v>306.33492986078477</v>
       </c>
       <c r="L129" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="23"/>
         <v>0.65340911170899529</v>
       </c>
     </row>
@@ -10490,6 +10651,342 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="C4:H37"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="4" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C4" s="105" t="s">
+        <v>245</v>
+      </c>
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="104"/>
+    </row>
+    <row r="6" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D6" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="E6" s="18">
+        <f>Connexion!E37*Connexion!D23/(ebac/1000)</f>
+        <v>397.35911107188895</v>
+      </c>
+      <c r="F6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D7" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E7" s="18">
+        <f>4*dsc</f>
+        <v>76</v>
+      </c>
+      <c r="F7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D8" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E8" s="18">
+        <f>(beff_m-E7/1000)/beff_m/2</f>
+        <v>0.48211764705882354</v>
+      </c>
+    </row>
+    <row r="9" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D9" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E9" s="18">
+        <f>E8*E6</f>
+        <v>191.57383966736481</v>
+      </c>
+      <c r="F9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D10" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E10" s="23">
+        <f>E9/(tc/1000)/1000</f>
+        <v>2.6607477731578446</v>
+      </c>
+      <c r="F10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D11" s="2"/>
+      <c r="E11" s="3"/>
+    </row>
+    <row r="12" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D12" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E12" s="18">
+        <f>Fck/GammaC</f>
+        <v>23.333333333333332</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D13" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E13" s="106">
+        <v>36</v>
+      </c>
+      <c r="F13" t="s">
+        <v>253</v>
+      </c>
+      <c r="G13" s="23">
+        <f>E13*PI()/180</f>
+        <v>0.62831853071795862</v>
+      </c>
+      <c r="H13" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="14" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="3">
+        <f>0.6*(1-Fck/250)</f>
+        <v>0.51600000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D15" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E15" s="22">
+        <f>Nuc*Fcd*SIN(ThetaRad)*COS(ThetaRad)</f>
+        <v>5.7253602280968243</v>
+      </c>
+      <c r="F15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D16" s="2"/>
+      <c r="E16" s="109">
+        <f>E10/E15</f>
+        <v>0.46473019463481124</v>
+      </c>
+    </row>
+    <row r="18" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D18" s="15" t="s">
+        <v>257</v>
+      </c>
+      <c r="E18" s="25">
+        <f>Fsk/GammaS</f>
+        <v>434.78260869565219</v>
+      </c>
+      <c r="F18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D19" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="E19" s="107">
+        <f>E10*tc*TAN(ThetaRad)/Fsd</f>
+        <v>0.32012904607472809</v>
+      </c>
+      <c r="F19" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="20" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D20" s="2"/>
+      <c r="E20" s="108">
+        <f>E19*1000/100</f>
+        <v>3.201290460747281</v>
+      </c>
+      <c r="F20" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="21" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D21" s="2"/>
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C22" s="105" t="s">
+        <v>260</v>
+      </c>
+      <c r="D22" s="104"/>
+      <c r="E22" s="104"/>
+      <c r="F22" s="104"/>
+      <c r="G22" s="104"/>
+    </row>
+    <row r="24" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D24" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="E24" s="18">
+        <f>E6</f>
+        <v>397.35911107188895</v>
+      </c>
+      <c r="F24" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="25" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D25" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E25" s="18">
+        <f>4*dsc</f>
+        <v>76</v>
+      </c>
+      <c r="F25" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D26" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E26" s="18">
+        <f>(beff_a-E25/1000)/beff_a/2</f>
+        <v>0.47466666666666663</v>
+      </c>
+    </row>
+    <row r="27" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D27" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E27" s="18">
+        <f>E26*E24</f>
+        <v>188.61312472212327</v>
+      </c>
+      <c r="F27" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="28" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D28" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E28" s="23">
+        <f>E27/(tc/1000)/1000</f>
+        <v>2.6196267322517124</v>
+      </c>
+      <c r="F28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D29" s="2"/>
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D30" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E30" s="18">
+        <f>Fck/GammaC</f>
+        <v>23.333333333333332</v>
+      </c>
+      <c r="F30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D31" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E31" s="106">
+        <v>36</v>
+      </c>
+      <c r="F31" t="s">
+        <v>253</v>
+      </c>
+      <c r="G31" s="23">
+        <f>E31*PI()/180</f>
+        <v>0.62831853071795862</v>
+      </c>
+      <c r="H31" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="32" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D32" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E32" s="3">
+        <f>0.6*(1-Fck/250)</f>
+        <v>0.51600000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D33" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E33" s="22">
+        <f>Nuc*Fcd*SIN(G31)*COS(G31)</f>
+        <v>5.7253602280968243</v>
+      </c>
+      <c r="F33" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D34" s="2"/>
+      <c r="E34" s="3"/>
+    </row>
+    <row r="35" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D35" s="15" t="s">
+        <v>257</v>
+      </c>
+      <c r="E35" s="25">
+        <f>Fsk/GammaS</f>
+        <v>434.78260869565219</v>
+      </c>
+      <c r="F35" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D36" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="E36" s="107">
+        <f>E28*tc*TAN(ThetaRad)/Fsd</f>
+        <v>0.3151815498363843</v>
+      </c>
+      <c r="F36" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="37" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D37" s="2"/>
+      <c r="E37" s="108">
+        <f>E36*1000/10</f>
+        <v>31.518154983638432</v>
+      </c>
+      <c r="F37" t="s">
+        <v>259</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="C4:I15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -10660,7 +11157,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B3:N22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>